<commit_message>
📈 Daily Screener Report — 15-Sep-2026 19:34 IST
</commit_message>
<xml_diff>
--- a/output/swing_screener_report.xlsx
+++ b/output/swing_screener_report.xlsx
@@ -820,13 +820,13 @@
         <v>9.32</v>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>3908</v>
+        <v>3659</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>20.465115</v>
+        <v>19.165115</v>
       </c>
       <c r="AC2" s="2" t="n">
-        <v>6.62152</v>
+        <v>6.2009034</v>
       </c>
       <c r="AD2" s="2" t="inlineStr"/>
       <c r="AE2" s="2" t="n">
@@ -839,7 +839,7 @@
         <v>17</v>
       </c>
       <c r="AH2" s="2" t="n">
-        <v>4.0618505</v>
+        <v>3.803831</v>
       </c>
       <c r="AI2" s="2" t="n">
         <v>62</v>
@@ -950,13 +950,13 @@
         <v>1.16</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>247470</v>
+        <v>244178</v>
       </c>
       <c r="AB3" s="4" t="n">
-        <v>84.74545000000001</v>
+        <v>83.61818</v>
       </c>
       <c r="AC3" s="4" t="n">
-        <v>61.95091</v>
+        <v>61.126846</v>
       </c>
       <c r="AD3" s="4" t="inlineStr"/>
       <c r="AE3" s="4" t="n">
@@ -969,7 +969,7 @@
         <v>65.7</v>
       </c>
       <c r="AH3" s="4" t="n">
-        <v>14.764624</v>
+        <v>14.568227</v>
       </c>
       <c r="AI3" s="4" t="n">
         <v>32</v>
@@ -1080,13 +1080,13 @@
         <v>0.95</v>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>63950</v>
+        <v>62596</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>34.010715</v>
+        <v>33.272877</v>
       </c>
       <c r="AC4" s="2" t="n">
-        <v>20.596039</v>
+        <v>20.149221</v>
       </c>
       <c r="AD4" s="2" t="inlineStr"/>
       <c r="AE4" s="2" t="inlineStr"/>
@@ -1097,7 +1097,7 @@
         <v>367.9</v>
       </c>
       <c r="AH4" s="2" t="n">
-        <v>1.5225495</v>
+        <v>1.4895188</v>
       </c>
       <c r="AI4" s="2" t="n">
         <v>33</v>
@@ -1208,13 +1208,13 @@
         <v>1.24</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>416807</v>
+        <v>407655</v>
       </c>
       <c r="AB5" s="4" t="n">
-        <v>20.529152</v>
+        <v>20.078392</v>
       </c>
       <c r="AC5" s="4" t="n">
-        <v>16.399218</v>
+        <v>16.039139</v>
       </c>
       <c r="AD5" s="4" t="inlineStr"/>
       <c r="AE5" s="4" t="inlineStr"/>
@@ -1225,7 +1225,7 @@
         <v>22.5</v>
       </c>
       <c r="AH5" s="4" t="n">
-        <v>2.299658</v>
+        <v>2.2491643</v>
       </c>
       <c r="AI5" s="4" t="n">
         <v>16</v>
@@ -1335,14 +1335,12 @@
       <c r="Z6" s="2" t="n">
         <v>0.73</v>
       </c>
-      <c r="AA6" s="2" t="n">
-        <v>83379</v>
-      </c>
+      <c r="AA6" s="2" t="inlineStr"/>
       <c r="AB6" s="2" t="n">
-        <v>54.050488</v>
+        <v>52.359344</v>
       </c>
       <c r="AC6" s="2" t="n">
-        <v>40.93824</v>
+        <v>39.65736</v>
       </c>
       <c r="AD6" s="2" t="inlineStr"/>
       <c r="AE6" s="2" t="n">
@@ -1355,7 +1353,7 @@
         <v>103.4</v>
       </c>
       <c r="AH6" s="2" t="n">
-        <v>19.813597</v>
+        <v>19.193666</v>
       </c>
       <c r="AI6" s="2" t="n">
         <v>24</v>
@@ -1466,13 +1464,13 @@
         <v>1.17</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>30741</v>
+        <v>29235</v>
       </c>
       <c r="AB7" s="4" t="n">
-        <v>9.787946</v>
+        <v>9.308593999999999</v>
       </c>
       <c r="AC7" s="4" t="n">
-        <v>3.425781</v>
+        <v>3.2580078</v>
       </c>
       <c r="AD7" s="4" t="inlineStr"/>
       <c r="AE7" s="4" t="n">
@@ -1483,10 +1481,10 @@
       </c>
       <c r="AG7" s="4" t="inlineStr"/>
       <c r="AH7" s="4" t="n">
-        <v>2.1573088</v>
+        <v>2.0516572</v>
       </c>
       <c r="AI7" s="4" t="n">
-        <v>221</v>
+        <v>227</v>
       </c>
       <c r="AJ7" s="4" t="inlineStr"/>
       <c r="AK7" s="4" t="inlineStr">
@@ -1598,13 +1596,13 @@
         <v>1.35</v>
       </c>
       <c r="AA8" s="2" t="n">
-        <v>47490</v>
+        <v>46455</v>
       </c>
       <c r="AB8" s="2" t="n">
-        <v>38.00562</v>
+        <v>37.176968</v>
       </c>
       <c r="AC8" s="2" t="n">
-        <v>32.17346</v>
+        <v>31.471966</v>
       </c>
       <c r="AD8" s="2" t="inlineStr"/>
       <c r="AE8" s="2" t="n">
@@ -1617,7 +1615,7 @@
         <v>269</v>
       </c>
       <c r="AH8" s="2" t="n">
-        <v>7.843115</v>
+        <v>7.672108</v>
       </c>
       <c r="AI8" s="2" t="n">
         <v>99</v>
@@ -1728,13 +1726,13 @@
         <v>0.83</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>328034</v>
+        <v>313990</v>
       </c>
       <c r="AB9" s="4" t="n">
-        <v>35.211773</v>
+        <v>33.704235</v>
       </c>
       <c r="AC9" s="4" t="n">
-        <v>28.519903</v>
+        <v>27.298868</v>
       </c>
       <c r="AD9" s="4" t="inlineStr"/>
       <c r="AE9" s="4" t="n">
@@ -1747,10 +1745,10 @@
         <v>14.9</v>
       </c>
       <c r="AH9" s="4" t="n">
-        <v>7.992817</v>
+        <v>7.6506166</v>
       </c>
       <c r="AI9" s="4" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="AJ9" s="4" t="inlineStr"/>
       <c r="AK9" s="4" t="inlineStr">
@@ -1858,13 +1856,13 @@
         <v>0.96</v>
       </c>
       <c r="AA10" s="2" t="n">
-        <v>134180</v>
+        <v>131824</v>
       </c>
       <c r="AB10" s="2" t="n">
-        <v>6.074402</v>
+        <v>5.967742</v>
       </c>
       <c r="AC10" s="2" t="n">
-        <v>6.807199</v>
+        <v>6.6876717</v>
       </c>
       <c r="AD10" s="2" t="n">
         <v>14.97</v>
@@ -1877,7 +1875,7 @@
         <v>1.9</v>
       </c>
       <c r="AH10" s="2" t="n">
-        <v>0.85811514</v>
+        <v>0.84304756</v>
       </c>
       <c r="AI10" s="2" t="n">
         <v>257</v>
@@ -1988,13 +1986,13 @@
         <v>6.33</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>22644</v>
+        <v>21623</v>
       </c>
       <c r="AB11" s="4" t="n">
-        <v>33.945023</v>
+        <v>32.414562</v>
       </c>
       <c r="AC11" s="4" t="n">
-        <v>23.00935</v>
+        <v>21.97194</v>
       </c>
       <c r="AD11" s="4" t="inlineStr"/>
       <c r="AE11" s="4" t="n">
@@ -2007,7 +2005,7 @@
         <v>53.4</v>
       </c>
       <c r="AH11" s="4" t="n">
-        <v>4.453043</v>
+        <v>4.2522707</v>
       </c>
       <c r="AI11" s="4" t="n">
         <v>19</v>
@@ -2118,13 +2116,13 @@
         <v>1.17</v>
       </c>
       <c r="AA12" s="2" t="n">
-        <v>102436</v>
+        <v>102784</v>
       </c>
       <c r="AB12" s="2" t="n">
-        <v>30.02987</v>
+        <v>30.131987</v>
       </c>
       <c r="AC12" s="2" t="n">
-        <v>25.94684</v>
+        <v>26.035072</v>
       </c>
       <c r="AD12" s="2" t="n">
         <v>49.9</v>
@@ -2139,7 +2137,7 @@
         <v>120.2</v>
       </c>
       <c r="AH12" s="2" t="n">
-        <v>14.785403</v>
+        <v>14.835681</v>
       </c>
       <c r="AI12" s="2" t="n">
         <v>565</v>
@@ -2252,13 +2250,13 @@
         <v>0.33</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>19734</v>
+        <v>19116</v>
       </c>
       <c r="AB13" s="4" t="n">
-        <v>71.529205</v>
+        <v>69.28865999999999</v>
       </c>
       <c r="AC13" s="4" t="n">
-        <v>22.57592</v>
+        <v>21.868763</v>
       </c>
       <c r="AD13" s="4" t="inlineStr"/>
       <c r="AE13" s="4" t="n">
@@ -2271,7 +2269,7 @@
         <v>83.7</v>
       </c>
       <c r="AH13" s="4" t="n">
-        <v>4.059958</v>
+        <v>3.932786</v>
       </c>
       <c r="AI13" s="4" t="n">
         <v>5</v>
@@ -2382,13 +2380,13 @@
         <v>4.98</v>
       </c>
       <c r="AA14" s="2" t="n">
-        <v>6675</v>
+        <v>6628</v>
       </c>
       <c r="AB14" s="2" t="n">
-        <v>151.51057</v>
+        <v>150.44562</v>
       </c>
       <c r="AC14" s="2" t="n">
-        <v>44.18502</v>
+        <v>43.874447</v>
       </c>
       <c r="AD14" s="2" t="inlineStr"/>
       <c r="AE14" s="2" t="n">
@@ -2401,7 +2399,7 @@
         <v>-99.59999999999999</v>
       </c>
       <c r="AH14" s="2" t="n">
-        <v>2.3470993</v>
+        <v>2.3306017</v>
       </c>
       <c r="AI14" s="2" t="n">
         <v>0</v>
@@ -2512,13 +2510,13 @@
         <v>0.86</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>435430</v>
+        <v>416732</v>
       </c>
       <c r="AB15" s="4" t="n">
-        <v>53.18964</v>
+        <v>50.905617</v>
       </c>
       <c r="AC15" s="4" t="n">
-        <v>46.476307</v>
+        <v>44.480564</v>
       </c>
       <c r="AD15" s="4" t="inlineStr"/>
       <c r="AE15" s="4" t="n">
@@ -2529,7 +2527,7 @@
       </c>
       <c r="AG15" s="4" t="inlineStr"/>
       <c r="AH15" s="4" t="n">
-        <v>4.8879366</v>
+        <v>4.6780434</v>
       </c>
       <c r="AI15" s="4" t="n">
         <v>4</v>
@@ -2549,32 +2547,32 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>COALINDIA</t>
+          <t>SYRMA</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Coal India Limited</t>
+          <t>Syrma SGS Technology Limited</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Thermal Coal</t>
+          <t>Electronic Components</t>
         </is>
       </c>
       <c r="E16" s="5" t="n">
         <v>57.2</v>
       </c>
       <c r="F16" s="2" t="n">
-        <v>30.6</v>
+        <v>37</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>26.6</v>
+        <v>20.2</v>
       </c>
       <c r="H16" s="5" t="inlineStr">
         <is>
@@ -2583,27 +2581,27 @@
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>✅ Supertrend Buy | 📉 Tight Base</t>
+          <t>✅ Supertrend Buy | 📈 EMA Bull Stack | 🏆 Near 52W High | 📉 Tight Base</t>
         </is>
       </c>
       <c r="J16" s="2" t="n">
-        <v>426.4</v>
+        <v>1589.3</v>
       </c>
       <c r="K16" s="2" t="n">
-        <v>-1.3</v>
+        <v>-0.59</v>
       </c>
       <c r="L16" s="2" t="n">
-        <v>413.29</v>
+        <v>1502.6</v>
       </c>
       <c r="M16" s="2" t="n">
-        <v>414.3</v>
+        <v>1427.83</v>
       </c>
       <c r="N16" s="2" t="n">
-        <v>412.67</v>
+        <v>1139.63</v>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>✗</t>
+          <t>✓</t>
         </is>
       </c>
       <c r="P16" s="2" t="inlineStr">
@@ -2612,99 +2610,99 @@
         </is>
       </c>
       <c r="Q16" s="2" t="n">
-        <v>89.06999999999999</v>
+        <v>95.73999999999999</v>
       </c>
       <c r="R16" s="2" t="n">
-        <v>65.90000000000001</v>
+        <v>64.25</v>
       </c>
       <c r="S16" s="2" t="n">
-        <v>4.8555</v>
+        <v>43.2048</v>
       </c>
       <c r="T16" s="2" t="n">
-        <v>1.0669</v>
+        <v>30.3694</v>
       </c>
       <c r="U16" s="2" t="n">
-        <v>3.7886</v>
+        <v>12.8354</v>
       </c>
       <c r="V16" s="2" t="inlineStr"/>
       <c r="W16" s="2" t="n">
-        <v>30.37</v>
+        <v>21.86</v>
       </c>
       <c r="X16" s="2" t="n">
-        <v>3868222</v>
+        <v>638884</v>
       </c>
       <c r="Y16" s="2" t="n">
-        <v>11099503</v>
+        <v>986557</v>
       </c>
       <c r="Z16" s="2" t="n">
-        <v>0.35</v>
+        <v>0.65</v>
       </c>
       <c r="AA16" s="2" t="n">
-        <v>262779</v>
+        <v>29042</v>
       </c>
       <c r="AB16" s="2" t="n">
-        <v>8.431876000000001</v>
+        <v>77.75658</v>
       </c>
       <c r="AC16" s="2" t="n">
-        <v>7.5333066</v>
+        <v>48.67879</v>
       </c>
       <c r="AD16" s="2" t="inlineStr"/>
       <c r="AE16" s="2" t="n">
-        <v>11.629</v>
+        <v>13.045</v>
       </c>
       <c r="AF16" s="2" t="n">
-        <v>45.1</v>
+        <v>68.3</v>
       </c>
       <c r="AG16" s="2" t="n">
-        <v>1.2</v>
+        <v>86</v>
       </c>
       <c r="AH16" s="2" t="n">
-        <v>2.2061257</v>
+        <v>10.076659</v>
       </c>
       <c r="AI16" s="2" t="n">
-        <v>492</v>
+        <v>9</v>
       </c>
       <c r="AJ16" s="2" t="inlineStr"/>
       <c r="AK16" s="2" t="inlineStr">
         <is>
-          <t>https://www.screener.in/company/COALINDIA/</t>
+          <t>https://www.screener.in/company/SYRMA/</t>
         </is>
       </c>
       <c r="AL16" s="2" t="inlineStr">
         <is>
-          <t>https://www.tradingview.com/chart/?symbol=NSE:COALINDIA</t>
+          <t>https://www.tradingview.com/chart/?symbol=NSE:SYRMA</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>BEML</t>
+          <t>COALINDIA</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>BEML Limited</t>
+          <t>Coal India Limited</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>Conglomerates</t>
+          <t>Thermal Coal</t>
         </is>
       </c>
       <c r="E17" s="5" t="n">
-        <v>56.8</v>
+        <v>57.2</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>40.2</v>
+        <v>30.6</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>16.6</v>
+        <v>26.6</v>
       </c>
       <c r="H17" s="5" t="inlineStr">
         <is>
@@ -2713,27 +2711,27 @@
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>✅ Supertrend Buy | 📈 EMA Bull Stack | 📉 Tight Base</t>
+          <t>✅ Supertrend Buy | 📉 Tight Base</t>
         </is>
       </c>
       <c r="J17" s="4" t="n">
-        <v>2023.4</v>
+        <v>426.4</v>
       </c>
       <c r="K17" s="4" t="n">
-        <v>-0.28</v>
+        <v>-1.3</v>
       </c>
       <c r="L17" s="4" t="n">
-        <v>1992.51</v>
+        <v>413.29</v>
       </c>
       <c r="M17" s="4" t="n">
-        <v>1909.2</v>
+        <v>414.3</v>
       </c>
       <c r="N17" s="4" t="n">
-        <v>1838.32</v>
+        <v>412.67</v>
       </c>
       <c r="O17" s="4" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>✗</t>
         </is>
       </c>
       <c r="P17" s="4" t="inlineStr">
@@ -2742,97 +2740,99 @@
         </is>
       </c>
       <c r="Q17" s="4" t="n">
-        <v>89.16</v>
+        <v>89.06999999999999</v>
       </c>
       <c r="R17" s="4" t="n">
-        <v>57.23</v>
+        <v>65.90000000000001</v>
       </c>
       <c r="S17" s="4" t="n">
-        <v>57.6403</v>
+        <v>4.8555</v>
       </c>
       <c r="T17" s="4" t="n">
-        <v>57.154</v>
+        <v>1.0669</v>
       </c>
       <c r="U17" s="4" t="n">
-        <v>0.4863</v>
+        <v>3.7886</v>
       </c>
       <c r="V17" s="4" t="inlineStr"/>
       <c r="W17" s="4" t="n">
-        <v>37.77</v>
+        <v>30.37</v>
       </c>
       <c r="X17" s="4" t="n">
-        <v>230934</v>
+        <v>3868222</v>
       </c>
       <c r="Y17" s="4" t="n">
-        <v>472856</v>
+        <v>11099503</v>
       </c>
       <c r="Z17" s="4" t="n">
-        <v>0.49</v>
+        <v>0.35</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>16912</v>
+        <v>258372</v>
       </c>
       <c r="AB17" s="4" t="n">
-        <v>94.39796</v>
+        <v>8.290488</v>
       </c>
       <c r="AC17" s="4" t="n">
-        <v>28.064962</v>
+        <v>7.4069858</v>
       </c>
       <c r="AD17" s="4" t="inlineStr"/>
       <c r="AE17" s="4" t="n">
-        <v>10.529</v>
+        <v>11.629</v>
       </c>
       <c r="AF17" s="4" t="n">
-        <v>29.3</v>
-      </c>
-      <c r="AG17" s="4" t="inlineStr"/>
+        <v>45.1</v>
+      </c>
+      <c r="AG17" s="4" t="n">
+        <v>1.2</v>
+      </c>
       <c r="AH17" s="4" t="n">
-        <v>5.764437</v>
+        <v>2.169133</v>
       </c>
       <c r="AI17" s="4" t="n">
-        <v>87</v>
+        <v>492</v>
       </c>
       <c r="AJ17" s="4" t="inlineStr"/>
       <c r="AK17" s="4" t="inlineStr">
         <is>
-          <t>https://www.screener.in/company/BEML/</t>
+          <t>https://www.screener.in/company/COALINDIA/</t>
         </is>
       </c>
       <c r="AL17" s="4" t="inlineStr">
         <is>
-          <t>https://www.tradingview.com/chart/?symbol=NSE:BEML</t>
+          <t>https://www.tradingview.com/chart/?symbol=NSE:COALINDIA</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>AUROPHARMA</t>
+          <t>BEML</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Aurobindo Pharma Limited</t>
+          <t>BEML Limited</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Drug Manufacturers - Specialty &amp; Generic</t>
+          <t>Conglomerates</t>
         </is>
       </c>
       <c r="E18" s="5" t="n">
-        <v>56.2</v>
+        <v>56.8</v>
       </c>
       <c r="F18" s="2" t="n">
-        <v>37</v>
+        <v>40.2</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>19.2</v>
+        <v>16.6</v>
       </c>
       <c r="H18" s="5" t="inlineStr">
         <is>
@@ -2841,23 +2841,23 @@
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>✅ Supertrend Buy | 📈 EMA Bull Stack | 🏆 Near 52W High | 📉 Tight Base</t>
+          <t>✅ Supertrend Buy | 📈 EMA Bull Stack | 📉 Tight Base</t>
         </is>
       </c>
       <c r="J18" s="2" t="n">
-        <v>1679.8</v>
+        <v>2023.4</v>
       </c>
       <c r="K18" s="2" t="n">
-        <v>0.68</v>
+        <v>-0.28</v>
       </c>
       <c r="L18" s="2" t="n">
-        <v>1652.16</v>
+        <v>1992.51</v>
       </c>
       <c r="M18" s="2" t="n">
-        <v>1607.4</v>
+        <v>1909.2</v>
       </c>
       <c r="N18" s="2" t="n">
-        <v>1427.88</v>
+        <v>1838.32</v>
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
@@ -2870,79 +2870,77 @@
         </is>
       </c>
       <c r="Q18" s="2" t="n">
-        <v>97.83</v>
+        <v>89.16</v>
       </c>
       <c r="R18" s="2" t="n">
-        <v>56.97</v>
+        <v>57.23</v>
       </c>
       <c r="S18" s="2" t="n">
-        <v>21.638</v>
+        <v>57.6403</v>
       </c>
       <c r="T18" s="2" t="n">
-        <v>21.0404</v>
+        <v>57.154</v>
       </c>
       <c r="U18" s="2" t="n">
-        <v>0.5976</v>
+        <v>0.4863</v>
       </c>
       <c r="V18" s="2" t="inlineStr"/>
       <c r="W18" s="2" t="n">
-        <v>26.1</v>
+        <v>37.77</v>
       </c>
       <c r="X18" s="2" t="n">
-        <v>494251</v>
+        <v>230934</v>
       </c>
       <c r="Y18" s="2" t="n">
-        <v>821577</v>
+        <v>472856</v>
       </c>
       <c r="Z18" s="2" t="n">
-        <v>0.6</v>
+        <v>0.49</v>
       </c>
       <c r="AA18" s="2" t="n">
-        <v>96652</v>
+        <v>16152</v>
       </c>
       <c r="AB18" s="2" t="n">
-        <v>26.246876</v>
+        <v>90.41025500000001</v>
       </c>
       <c r="AC18" s="2" t="n">
-        <v>18.06618</v>
+        <v>26.804424</v>
       </c>
       <c r="AD18" s="2" t="inlineStr"/>
       <c r="AE18" s="2" t="n">
-        <v>21.31</v>
+        <v>10.529</v>
       </c>
       <c r="AF18" s="2" t="n">
-        <v>16.3</v>
-      </c>
-      <c r="AG18" s="2" t="n">
-        <v>25.8</v>
-      </c>
+        <v>29.3</v>
+      </c>
+      <c r="AG18" s="2" t="inlineStr"/>
       <c r="AH18" s="2" t="n">
-        <v>2.5748363</v>
+        <v>5.5055275</v>
       </c>
       <c r="AI18" s="2" t="n">
-        <v>24</v>
+        <v>87</v>
       </c>
       <c r="AJ18" s="2" t="inlineStr"/>
       <c r="AK18" s="2" t="inlineStr">
         <is>
-          <t>https://www.screener.in/company/AUROPHARMA/</t>
+          <t>https://www.screener.in/company/BEML/</t>
         </is>
       </c>
       <c r="AL18" s="2" t="inlineStr">
         <is>
-          <t>https://www.tradingview.com/chart/?symbol=NSE:AUROPHARMA</t>
+          <t>https://www.tradingview.com/chart/?symbol=NSE:BEML</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>LAURUSLABS</t>
+          <t>AUROPHARMA</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Laurus Labs Limited</t>
+          <t>Aurobindo Pharma Limited</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
@@ -2956,13 +2954,13 @@
         </is>
       </c>
       <c r="E19" s="5" t="n">
-        <v>56.1</v>
+        <v>56.2</v>
       </c>
       <c r="F19" s="4" t="n">
-        <v>41.6</v>
+        <v>37</v>
       </c>
       <c r="G19" s="4" t="n">
-        <v>14.5</v>
+        <v>19.2</v>
       </c>
       <c r="H19" s="5" t="inlineStr">
         <is>
@@ -2971,23 +2969,23 @@
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>📤 20D Breakout | ⚡ Fresh MACD Cross | ✅ Supertrend Buy | 📈 EMA Bull Stack | 🏆 At 52W High | 📉 Tight Base</t>
+          <t>✅ Supertrend Buy | 📈 EMA Bull Stack | 🏆 Near 52W High | 📉 Tight Base</t>
         </is>
       </c>
       <c r="J19" s="4" t="n">
-        <v>1969</v>
+        <v>1679.8</v>
       </c>
       <c r="K19" s="4" t="n">
-        <v>1.23</v>
+        <v>0.68</v>
       </c>
       <c r="L19" s="4" t="n">
-        <v>1876.92</v>
+        <v>1652.16</v>
       </c>
       <c r="M19" s="4" t="n">
-        <v>1757.38</v>
+        <v>1607.4</v>
       </c>
       <c r="N19" s="4" t="n">
-        <v>1383.32</v>
+        <v>1427.88</v>
       </c>
       <c r="O19" s="4" t="inlineStr">
         <is>
@@ -3000,103 +2998,99 @@
         </is>
       </c>
       <c r="Q19" s="4" t="n">
-        <v>99.34999999999999</v>
+        <v>97.83</v>
       </c>
       <c r="R19" s="4" t="n">
-        <v>67.81</v>
+        <v>56.97</v>
       </c>
       <c r="S19" s="4" t="n">
-        <v>51.4245</v>
+        <v>21.638</v>
       </c>
       <c r="T19" s="4" t="n">
-        <v>50.9688</v>
+        <v>21.0404</v>
       </c>
       <c r="U19" s="4" t="n">
-        <v>0.4558</v>
-      </c>
-      <c r="V19" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+        <v>0.5976</v>
+      </c>
+      <c r="V19" s="4" t="inlineStr"/>
       <c r="W19" s="4" t="n">
-        <v>31.73</v>
+        <v>26.1</v>
       </c>
       <c r="X19" s="4" t="n">
-        <v>2277375</v>
+        <v>494251</v>
       </c>
       <c r="Y19" s="4" t="n">
-        <v>3578275</v>
+        <v>821577</v>
       </c>
       <c r="Z19" s="4" t="n">
-        <v>0.64</v>
+        <v>0.6</v>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>106387</v>
+        <v>95513</v>
       </c>
       <c r="AB19" s="4" t="n">
-        <v>97.09072999999999</v>
+        <v>25.9375</v>
       </c>
       <c r="AC19" s="4" t="n">
-        <v>68.03257000000001</v>
+        <v>17.853231</v>
       </c>
       <c r="AD19" s="4" t="inlineStr"/>
       <c r="AE19" s="4" t="n">
-        <v>46.369</v>
+        <v>21.31</v>
       </c>
       <c r="AF19" s="4" t="n">
-        <v>29.1</v>
+        <v>16.3</v>
       </c>
       <c r="AG19" s="4" t="n">
-        <v>125.2</v>
+        <v>25.8</v>
       </c>
       <c r="AH19" s="4" t="n">
-        <v>20.056023</v>
+        <v>2.5444863</v>
       </c>
       <c r="AI19" s="4" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="AJ19" s="4" t="inlineStr"/>
       <c r="AK19" s="4" t="inlineStr">
         <is>
-          <t>https://www.screener.in/company/LAURUSLABS/</t>
+          <t>https://www.screener.in/company/AUROPHARMA/</t>
         </is>
       </c>
       <c r="AL19" s="4" t="inlineStr">
         <is>
-          <t>https://www.tradingview.com/chart/?symbol=NSE:LAURUSLABS</t>
+          <t>https://www.tradingview.com/chart/?symbol=NSE:AUROPHARMA</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>ARVIND</t>
+          <t>LAURUSLABS</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Arvind Limited</t>
+          <t>Laurus Labs Limited</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Consumer Cyclical</t>
+          <t>Healthcare</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Textile Manufacturing</t>
+          <t>Drug Manufacturers - Specialty &amp; Generic</t>
         </is>
       </c>
       <c r="E20" s="5" t="n">
         <v>56.1</v>
       </c>
       <c r="F20" s="2" t="n">
-        <v>37</v>
+        <v>41.6</v>
       </c>
       <c r="G20" s="2" t="n">
-        <v>19.1</v>
+        <v>14.5</v>
       </c>
       <c r="H20" s="5" t="inlineStr">
         <is>
@@ -3105,23 +3099,23 @@
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>✅ Supertrend Buy | 📈 EMA Bull Stack | 🏆 Near 52W High | 📉 Tight Base</t>
+          <t>📤 20D Breakout | ⚡ Fresh MACD Cross | ✅ Supertrend Buy | 📈 EMA Bull Stack | 🏆 At 52W High | 📉 Tight Base</t>
         </is>
       </c>
       <c r="J20" s="2" t="n">
-        <v>575.1</v>
+        <v>1969</v>
       </c>
       <c r="K20" s="2" t="n">
-        <v>0.93</v>
+        <v>1.23</v>
       </c>
       <c r="L20" s="2" t="n">
-        <v>555.64</v>
+        <v>1876.92</v>
       </c>
       <c r="M20" s="2" t="n">
-        <v>537.96</v>
+        <v>1757.38</v>
       </c>
       <c r="N20" s="2" t="n">
-        <v>452.21</v>
+        <v>1383.32</v>
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
@@ -3134,99 +3128,103 @@
         </is>
       </c>
       <c r="Q20" s="2" t="n">
-        <v>94.72</v>
+        <v>99.34999999999999</v>
       </c>
       <c r="R20" s="2" t="n">
-        <v>60.25</v>
+        <v>67.81</v>
       </c>
       <c r="S20" s="2" t="n">
-        <v>10.3313</v>
+        <v>51.4245</v>
       </c>
       <c r="T20" s="2" t="n">
-        <v>7.8876</v>
+        <v>50.9688</v>
       </c>
       <c r="U20" s="2" t="n">
-        <v>2.4436</v>
-      </c>
-      <c r="V20" s="2" t="inlineStr"/>
+        <v>0.4558</v>
+      </c>
+      <c r="V20" s="2" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="W20" s="2" t="n">
-        <v>21.09</v>
+        <v>31.73</v>
       </c>
       <c r="X20" s="2" t="n">
-        <v>470791</v>
+        <v>2277375</v>
       </c>
       <c r="Y20" s="2" t="n">
-        <v>779550</v>
+        <v>3578275</v>
       </c>
       <c r="Z20" s="2" t="n">
-        <v>0.6</v>
+        <v>0.64</v>
       </c>
       <c r="AA20" s="2" t="n">
-        <v>15691</v>
+        <v>104113</v>
       </c>
       <c r="AB20" s="2" t="n">
-        <v>36.46018</v>
+        <v>95.01479</v>
       </c>
       <c r="AC20" s="2" t="n">
-        <v>22.456064</v>
+        <v>66.577934</v>
       </c>
       <c r="AD20" s="2" t="inlineStr"/>
       <c r="AE20" s="2" t="n">
-        <v>40.071</v>
+        <v>46.369</v>
       </c>
       <c r="AF20" s="2" t="n">
-        <v>24.7</v>
+        <v>29.1</v>
       </c>
       <c r="AG20" s="2" t="n">
-        <v>0.5</v>
+        <v>125.2</v>
       </c>
       <c r="AH20" s="2" t="n">
-        <v>3.7383904</v>
+        <v>19.627195</v>
       </c>
       <c r="AI20" s="2" t="n">
-        <v>79</v>
+        <v>12</v>
       </c>
       <c r="AJ20" s="2" t="inlineStr"/>
       <c r="AK20" s="2" t="inlineStr">
         <is>
-          <t>https://www.screener.in/company/ARVIND/</t>
+          <t>https://www.screener.in/company/LAURUSLABS/</t>
         </is>
       </c>
       <c r="AL20" s="2" t="inlineStr">
         <is>
-          <t>https://www.tradingview.com/chart/?symbol=NSE:ARVIND</t>
+          <t>https://www.tradingview.com/chart/?symbol=NSE:LAURUSLABS</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>SYRMA</t>
+          <t>ARVIND</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Syrma SGS Technology Limited</t>
+          <t>Arvind Limited</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Consumer Cyclical</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>Electronic Components</t>
+          <t>Textile Manufacturing</t>
         </is>
       </c>
       <c r="E21" s="5" t="n">
-        <v>55.1</v>
+        <v>56.1</v>
       </c>
       <c r="F21" s="4" t="n">
         <v>37</v>
       </c>
       <c r="G21" s="4" t="n">
-        <v>18.1</v>
+        <v>19.1</v>
       </c>
       <c r="H21" s="5" t="inlineStr">
         <is>
@@ -3239,19 +3237,19 @@
         </is>
       </c>
       <c r="J21" s="4" t="n">
-        <v>1589.3</v>
+        <v>575.1</v>
       </c>
       <c r="K21" s="4" t="n">
-        <v>-0.59</v>
+        <v>0.93</v>
       </c>
       <c r="L21" s="4" t="n">
-        <v>1502.6</v>
+        <v>555.64</v>
       </c>
       <c r="M21" s="4" t="n">
-        <v>1427.83</v>
+        <v>537.96</v>
       </c>
       <c r="N21" s="4" t="n">
-        <v>1139.63</v>
+        <v>452.21</v>
       </c>
       <c r="O21" s="4" t="inlineStr">
         <is>
@@ -3264,67 +3262,67 @@
         </is>
       </c>
       <c r="Q21" s="4" t="n">
-        <v>95.73999999999999</v>
+        <v>94.72</v>
       </c>
       <c r="R21" s="4" t="n">
-        <v>64.25</v>
+        <v>60.25</v>
       </c>
       <c r="S21" s="4" t="n">
-        <v>43.2048</v>
+        <v>10.3313</v>
       </c>
       <c r="T21" s="4" t="n">
-        <v>30.3694</v>
+        <v>7.8876</v>
       </c>
       <c r="U21" s="4" t="n">
-        <v>12.8354</v>
+        <v>2.4436</v>
       </c>
       <c r="V21" s="4" t="inlineStr"/>
       <c r="W21" s="4" t="n">
-        <v>21.86</v>
+        <v>21.09</v>
       </c>
       <c r="X21" s="4" t="n">
-        <v>638884</v>
+        <v>470791</v>
       </c>
       <c r="Y21" s="4" t="n">
-        <v>986557</v>
+        <v>779550</v>
       </c>
       <c r="Z21" s="4" t="n">
-        <v>0.65</v>
+        <v>0.6</v>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>30720</v>
+        <v>14433</v>
       </c>
       <c r="AB21" s="4" t="n">
-        <v>82.24858999999999</v>
+        <v>34.804043</v>
       </c>
       <c r="AC21" s="4" t="n">
-        <v>51.490974</v>
+        <v>21.436043</v>
       </c>
       <c r="AD21" s="4" t="inlineStr"/>
       <c r="AE21" s="4" t="n">
-        <v>13.045</v>
+        <v>40.071</v>
       </c>
       <c r="AF21" s="4" t="n">
-        <v>68.3</v>
+        <v>24.7</v>
       </c>
       <c r="AG21" s="4" t="n">
-        <v>86</v>
+        <v>0.5</v>
       </c>
       <c r="AH21" s="4" t="n">
-        <v>10.65879</v>
+        <v>3.5685813</v>
       </c>
       <c r="AI21" s="4" t="n">
-        <v>9</v>
+        <v>78</v>
       </c>
       <c r="AJ21" s="4" t="inlineStr"/>
       <c r="AK21" s="4" t="inlineStr">
         <is>
-          <t>https://www.screener.in/company/SYRMA/</t>
+          <t>https://www.screener.in/company/ARVIND/</t>
         </is>
       </c>
       <c r="AL21" s="4" t="inlineStr">
         <is>
-          <t>https://www.tradingview.com/chart/?symbol=NSE:SYRMA</t>
+          <t>https://www.tradingview.com/chart/?symbol=NSE:ARVIND</t>
         </is>
       </c>
     </row>
@@ -3422,13 +3420,13 @@
         <v>1.05</v>
       </c>
       <c r="AA22" s="2" t="n">
-        <v>8992</v>
+        <v>8718</v>
       </c>
       <c r="AB22" s="2" t="n">
-        <v>38.647785</v>
+        <v>37.473732</v>
       </c>
       <c r="AC22" s="2" t="n">
-        <v>26.15682</v>
+        <v>25.362223</v>
       </c>
       <c r="AD22" s="2" t="inlineStr"/>
       <c r="AE22" s="2" t="n">
@@ -3441,7 +3439,7 @@
         <v>4.7</v>
       </c>
       <c r="AH22" s="2" t="n">
-        <v>5.680102</v>
+        <v>5.5075502</v>
       </c>
       <c r="AI22" s="2" t="n">
         <v>71</v>
@@ -3552,13 +3550,13 @@
         <v>0.96</v>
       </c>
       <c r="AA23" s="4" t="n">
-        <v>150077</v>
+        <v>143757</v>
       </c>
       <c r="AB23" s="4" t="n">
-        <v>61.747852</v>
+        <v>59.147564</v>
       </c>
       <c r="AC23" s="4" t="n">
-        <v>31.269657</v>
+        <v>29.524443</v>
       </c>
       <c r="AD23" s="4" t="inlineStr"/>
       <c r="AE23" s="4" t="n">
@@ -3569,7 +3567,7 @@
       </c>
       <c r="AG23" s="4" t="inlineStr"/>
       <c r="AH23" s="4" t="n">
-        <v>5.739856</v>
+        <v>5.4981427</v>
       </c>
       <c r="AI23" s="4" t="n">
         <v>32</v>
@@ -3680,13 +3678,13 @@
         <v>15.55</v>
       </c>
       <c r="AA24" s="2" t="n">
-        <v>8836</v>
+        <v>8632</v>
       </c>
       <c r="AB24" s="2" t="n">
-        <v>277.7073</v>
+        <v>271.26828</v>
       </c>
       <c r="AC24" s="2" t="n">
-        <v>110.41397</v>
+        <v>107.853874</v>
       </c>
       <c r="AD24" s="2" t="inlineStr"/>
       <c r="AE24" s="2" t="n">
@@ -3699,7 +3697,7 @@
         <v>-50</v>
       </c>
       <c r="AH24" s="2" t="n">
-        <v>14.559729</v>
+        <v>14.222141</v>
       </c>
       <c r="AI24" s="2" t="n">
         <v>14</v>
@@ -3810,13 +3808,13 @@
         <v>0.95</v>
       </c>
       <c r="AA25" s="4" t="n">
-        <v>98709</v>
+        <v>96330</v>
       </c>
       <c r="AB25" s="4" t="n">
-        <v>382.7778</v>
+        <v>373.55557</v>
       </c>
       <c r="AC25" s="4" t="n">
-        <v>117.3637</v>
+        <v>114.53607</v>
       </c>
       <c r="AD25" s="4" t="inlineStr"/>
       <c r="AE25" s="4" t="n">
@@ -3829,7 +3827,7 @@
         <v>250</v>
       </c>
       <c r="AH25" s="4" t="n">
-        <v>68.59817</v>
+        <v>66.94544</v>
       </c>
       <c r="AI25" s="4" t="n">
         <v>0</v>
@@ -3940,13 +3938,13 @@
         <v>0.67</v>
       </c>
       <c r="AA26" s="2" t="n">
-        <v>15156</v>
+        <v>14451</v>
       </c>
       <c r="AB26" s="2" t="n">
-        <v>113.697945</v>
+        <v>108.414444</v>
       </c>
       <c r="AC26" s="2" t="n">
-        <v>61.957245</v>
+        <v>59.078117</v>
       </c>
       <c r="AD26" s="2" t="inlineStr"/>
       <c r="AE26" s="2" t="n">
@@ -3959,7 +3957,7 @@
         <v>145.3</v>
       </c>
       <c r="AH26" s="2" t="n">
-        <v>20.974878</v>
+        <v>20.000185</v>
       </c>
       <c r="AI26" s="2" t="n">
         <v>0</v>
@@ -4070,13 +4068,13 @@
         <v>0.68</v>
       </c>
       <c r="AA27" s="4" t="n">
-        <v>68276</v>
+        <v>66935</v>
       </c>
       <c r="AB27" s="4" t="n">
-        <v>38.02578</v>
+        <v>37.279156</v>
       </c>
       <c r="AC27" s="4" t="n">
-        <v>24.769888</v>
+        <v>24.283543</v>
       </c>
       <c r="AD27" s="4" t="inlineStr"/>
       <c r="AE27" s="4" t="n">
@@ -4089,7 +4087,7 @@
         <v>930.7</v>
       </c>
       <c r="AH27" s="4" t="n">
-        <v>6.494932</v>
+        <v>6.367407</v>
       </c>
       <c r="AI27" s="4" t="n">
         <v>31</v>
@@ -4200,13 +4198,13 @@
         <v>0.67</v>
       </c>
       <c r="AA28" s="2" t="n">
-        <v>406557</v>
+        <v>394853</v>
       </c>
       <c r="AB28" s="2" t="n">
-        <v>30.122908</v>
+        <v>29.255718</v>
       </c>
       <c r="AC28" s="2" t="n">
-        <v>22.573994</v>
+        <v>21.924126</v>
       </c>
       <c r="AD28" s="2" t="inlineStr"/>
       <c r="AE28" s="2" t="n">
@@ -4219,10 +4217,10 @@
         <v>2.4</v>
       </c>
       <c r="AH28" s="2" t="n">
-        <v>4.2367854</v>
+        <v>4.114815</v>
       </c>
       <c r="AI28" s="2" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="AJ28" s="2" t="inlineStr"/>
       <c r="AK28" s="2" t="inlineStr">
@@ -4330,13 +4328,13 @@
         <v>0.65</v>
       </c>
       <c r="AA29" s="4" t="n">
-        <v>26917</v>
+        <v>25999</v>
       </c>
       <c r="AB29" s="4" t="n">
-        <v>44.050896</v>
+        <v>42.548145</v>
       </c>
       <c r="AC29" s="4" t="n">
-        <v>30.756302</v>
+        <v>29.707083</v>
       </c>
       <c r="AD29" s="4" t="inlineStr"/>
       <c r="AE29" s="4" t="n">
@@ -4349,10 +4347,10 @@
         <v>13.5</v>
       </c>
       <c r="AH29" s="4" t="n">
-        <v>6.296418</v>
+        <v>6.0816226</v>
       </c>
       <c r="AI29" s="4" t="n">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="AJ29" s="4" t="inlineStr"/>
       <c r="AK29" s="4" t="inlineStr">
@@ -4460,13 +4458,13 @@
         <v>1.58</v>
       </c>
       <c r="AA30" s="2" t="n">
-        <v>114963</v>
+        <v>112707</v>
       </c>
       <c r="AB30" s="2" t="n">
-        <v>8.992729000000001</v>
+        <v>8.816247000000001</v>
       </c>
       <c r="AC30" s="2" t="n">
-        <v>7.7787905</v>
+        <v>7.626131</v>
       </c>
       <c r="AD30" s="2" t="n">
         <v>16.17</v>
@@ -4479,7 +4477,7 @@
         <v>47.5</v>
       </c>
       <c r="AH30" s="2" t="n">
-        <v>1.3701752</v>
+        <v>1.3432854</v>
       </c>
       <c r="AI30" s="2" t="n">
         <v>214</v>
@@ -4590,13 +4588,13 @@
         <v>1.2</v>
       </c>
       <c r="AA31" s="4" t="n">
-        <v>173186</v>
+        <v>166551</v>
       </c>
       <c r="AB31" s="4" t="n">
-        <v>39.53125</v>
+        <v>38.016827</v>
       </c>
       <c r="AC31" s="4" t="n">
-        <v>23.731358</v>
+        <v>22.82222</v>
       </c>
       <c r="AD31" s="4" t="inlineStr"/>
       <c r="AE31" s="4" t="n">
@@ -4609,7 +4607,7 @@
         <v>104.2</v>
       </c>
       <c r="AH31" s="4" t="n">
-        <v>4.226203</v>
+        <v>4.064299</v>
       </c>
       <c r="AI31" s="4" t="n">
         <v>30</v>
@@ -4720,13 +4718,13 @@
         <v>0.42</v>
       </c>
       <c r="AA32" s="2" t="n">
-        <v>14190</v>
+        <v>13768</v>
       </c>
       <c r="AB32" s="2" t="n">
-        <v>36.72956</v>
+        <v>35.638367</v>
       </c>
       <c r="AC32" s="2" t="n">
-        <v>32.014244</v>
+        <v>31.063137</v>
       </c>
       <c r="AD32" s="2" t="inlineStr"/>
       <c r="AE32" s="2" t="n">
@@ -4739,7 +4737,7 @@
         <v>14.9</v>
       </c>
       <c r="AH32" s="2" t="n">
-        <v>7.214954</v>
+        <v>7.0006056</v>
       </c>
       <c r="AI32" s="2" t="n">
         <v>133</v>
@@ -4850,13 +4848,13 @@
         <v>0.85</v>
       </c>
       <c r="AA33" s="4" t="n">
-        <v>135955</v>
+        <v>133588</v>
       </c>
       <c r="AB33" s="4" t="n">
-        <v>6.5865383</v>
+        <v>6.4718933</v>
       </c>
       <c r="AC33" s="4" t="n">
-        <v>6.6503115</v>
+        <v>6.5345564</v>
       </c>
       <c r="AD33" s="4" t="n">
         <v>15.8</v>
@@ -4865,7 +4863,7 @@
       <c r="AF33" s="4" t="inlineStr"/>
       <c r="AG33" s="4" t="inlineStr"/>
       <c r="AH33" s="4" t="n">
-        <v>0.9744488</v>
+        <v>0.9574875</v>
       </c>
       <c r="AI33" s="4" t="n">
         <v>281</v>
@@ -4976,13 +4974,13 @@
         <v>0.9</v>
       </c>
       <c r="AA34" s="2" t="n">
-        <v>27867</v>
+        <v>27193</v>
       </c>
       <c r="AB34" s="2" t="n">
-        <v>27.551943</v>
+        <v>26.874435</v>
       </c>
       <c r="AC34" s="2" t="n">
-        <v>17.266348</v>
+        <v>16.841764</v>
       </c>
       <c r="AD34" s="2" t="inlineStr"/>
       <c r="AE34" s="2" t="n">
@@ -4995,10 +4993,10 @@
         <v>100</v>
       </c>
       <c r="AH34" s="2" t="n">
-        <v>4.5410557</v>
+        <v>4.4293904</v>
       </c>
       <c r="AI34" s="2" t="n">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="AJ34" s="2" t="inlineStr"/>
       <c r="AK34" s="2" t="inlineStr">
@@ -5106,13 +5104,13 @@
         <v>0.63</v>
       </c>
       <c r="AA35" s="4" t="n">
-        <v>85094</v>
+        <v>84724</v>
       </c>
       <c r="AB35" s="4" t="n">
-        <v>18.412615</v>
+        <v>18.332443</v>
       </c>
       <c r="AC35" s="4" t="n">
-        <v>12.763987</v>
+        <v>12.70841</v>
       </c>
       <c r="AD35" s="4" t="inlineStr"/>
       <c r="AE35" s="4" t="inlineStr"/>
@@ -5123,7 +5121,7 @@
         <v>32.7</v>
       </c>
       <c r="AH35" s="4" t="n">
-        <v>2.1207178</v>
+        <v>2.1114838</v>
       </c>
       <c r="AI35" s="4" t="n">
         <v>35</v>
@@ -5234,13 +5232,13 @@
         <v>1.23</v>
       </c>
       <c r="AA36" s="2" t="n">
-        <v>66302</v>
+        <v>64383</v>
       </c>
       <c r="AB36" s="2" t="n">
-        <v>9.823130000000001</v>
+        <v>9.538774999999999</v>
       </c>
       <c r="AC36" s="2" t="n">
-        <v>9.309279</v>
+        <v>9.0398</v>
       </c>
       <c r="AD36" s="2" t="inlineStr"/>
       <c r="AE36" s="2" t="n">
@@ -5253,7 +5251,7 @@
         <v>91.09999999999999</v>
       </c>
       <c r="AH36" s="2" t="n">
-        <v>3.0684493</v>
+        <v>2.9796257</v>
       </c>
       <c r="AI36" s="2" t="n">
         <v>111</v>
@@ -5364,13 +5362,13 @@
         <v>0.64</v>
       </c>
       <c r="AA37" s="4" t="n">
-        <v>35969</v>
+        <v>33973</v>
       </c>
       <c r="AB37" s="4" t="n">
-        <v>61.370758</v>
+        <v>57.966057</v>
       </c>
       <c r="AC37" s="4" t="n">
-        <v>45.201927</v>
+        <v>42.694233</v>
       </c>
       <c r="AD37" s="4" t="inlineStr"/>
       <c r="AE37" s="4" t="n">
@@ -5381,7 +5379,7 @@
       </c>
       <c r="AG37" s="4" t="inlineStr"/>
       <c r="AH37" s="4" t="n">
-        <v>7.089856</v>
+        <v>6.696528</v>
       </c>
       <c r="AI37" s="4" t="n">
         <v>9</v>
@@ -5492,13 +5490,13 @@
         <v>0.95</v>
       </c>
       <c r="AA38" s="2" t="n">
-        <v>74332</v>
+        <v>73116</v>
       </c>
       <c r="AB38" s="2" t="n">
-        <v>33.285713</v>
+        <v>32.741314</v>
       </c>
       <c r="AC38" s="2" t="n">
-        <v>12.763607</v>
+        <v>12.554853</v>
       </c>
       <c r="AD38" s="2" t="inlineStr"/>
       <c r="AE38" s="2" t="inlineStr"/>
@@ -5509,7 +5507,7 @@
         <v>-23.2</v>
       </c>
       <c r="AH38" s="2" t="n">
-        <v>1.5643258</v>
+        <v>1.5387408</v>
       </c>
       <c r="AI38" s="2" t="n">
         <v>29</v>
@@ -5620,13 +5618,13 @@
         <v>0.93</v>
       </c>
       <c r="AA39" s="4" t="n">
-        <v>188872</v>
+        <v>184478</v>
       </c>
       <c r="AB39" s="4" t="n">
-        <v>79.359116</v>
+        <v>77.51318000000001</v>
       </c>
       <c r="AC39" s="4" t="n">
-        <v>53.305927</v>
+        <v>52.066006</v>
       </c>
       <c r="AD39" s="4" t="inlineStr"/>
       <c r="AE39" s="4" t="n">
@@ -5639,7 +5637,7 @@
         <v>-8.199999999999999</v>
       </c>
       <c r="AH39" s="4" t="n">
-        <v>20.034132</v>
+        <v>19.568129</v>
       </c>
       <c r="AI39" s="4" t="n">
         <v>77</v>
@@ -5750,13 +5748,13 @@
         <v>1.06</v>
       </c>
       <c r="AA40" s="2" t="n">
-        <v>81796</v>
+        <v>78651</v>
       </c>
       <c r="AB40" s="2" t="n">
-        <v>37.876923</v>
+        <v>36.420513</v>
       </c>
       <c r="AC40" s="2" t="n">
-        <v>25.843508</v>
+        <v>24.849796</v>
       </c>
       <c r="AD40" s="2" t="inlineStr"/>
       <c r="AE40" s="2" t="n">
@@ -5769,7 +5767,7 @@
         <v>30.9</v>
       </c>
       <c r="AH40" s="2" t="n">
-        <v>6.5026073</v>
+        <v>6.252575</v>
       </c>
       <c r="AI40" s="2" t="n">
         <v>87</v>
@@ -5880,13 +5878,13 @@
         <v>0.42</v>
       </c>
       <c r="AA41" s="4" t="n">
-        <v>12095</v>
+        <v>11877</v>
       </c>
       <c r="AB41" s="4" t="n">
-        <v>59.611454</v>
+        <v>58.537834</v>
       </c>
       <c r="AC41" s="4" t="n">
-        <v>37.462543</v>
+        <v>36.787834</v>
       </c>
       <c r="AD41" s="4" t="inlineStr"/>
       <c r="AE41" s="4" t="n">
@@ -5899,7 +5897,7 @@
         <v>12.7</v>
       </c>
       <c r="AH41" s="4" t="n">
-        <v>7.988052</v>
+        <v>7.844185</v>
       </c>
       <c r="AI41" s="4" t="n">
         <v>34</v>
@@ -6010,13 +6008,13 @@
         <v>0.63</v>
       </c>
       <c r="AA42" s="2" t="n">
-        <v>127048</v>
+        <v>125294</v>
       </c>
       <c r="AB42" s="2" t="n">
-        <v>60.975777</v>
+        <v>60.133873</v>
       </c>
       <c r="AC42" s="2" t="n">
-        <v>40.553112</v>
+        <v>39.99319</v>
       </c>
       <c r="AD42" s="2" t="inlineStr"/>
       <c r="AE42" s="2" t="n">
@@ -6029,7 +6027,7 @@
         <v>34.1</v>
       </c>
       <c r="AH42" s="2" t="n">
-        <v>13.401565</v>
+        <v>13.216527</v>
       </c>
       <c r="AI42" s="2" t="n">
         <v>23</v>
@@ -6140,13 +6138,13 @@
         <v>0.46</v>
       </c>
       <c r="AA43" s="4" t="n">
-        <v>222596</v>
+        <v>215074</v>
       </c>
       <c r="AB43" s="4" t="n">
-        <v>39.21496</v>
+        <v>37.88983</v>
       </c>
       <c r="AC43" s="4" t="n">
-        <v>21.73056</v>
+        <v>20.996256</v>
       </c>
       <c r="AD43" s="4" t="inlineStr"/>
       <c r="AE43" s="4" t="n">
@@ -6159,7 +6157,7 @@
         <v>51.3</v>
       </c>
       <c r="AH43" s="4" t="n">
-        <v>2.1513093</v>
+        <v>2.0786138</v>
       </c>
       <c r="AI43" s="4" t="n">
         <v>30</v>
@@ -6270,13 +6268,13 @@
         <v>1.06</v>
       </c>
       <c r="AA44" s="2" t="n">
-        <v>114157</v>
+        <v>112355</v>
       </c>
       <c r="AB44" s="2" t="n">
-        <v>11.543882</v>
+        <v>11.361703</v>
       </c>
       <c r="AC44" s="2" t="n">
-        <v>9.491602</v>
+        <v>9.341809</v>
       </c>
       <c r="AD44" s="2" t="inlineStr"/>
       <c r="AE44" s="2" t="n">
@@ -6289,10 +6287,10 @@
         <v>97.2</v>
       </c>
       <c r="AH44" s="2" t="n">
-        <v>1.2808652</v>
+        <v>1.2606512</v>
       </c>
       <c r="AI44" s="2" t="n">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="AJ44" s="2" t="inlineStr"/>
       <c r="AK44" s="2" t="inlineStr">
@@ -6400,13 +6398,13 @@
         <v>0.91</v>
       </c>
       <c r="AA45" s="4" t="n">
-        <v>137434</v>
+        <v>134429</v>
       </c>
       <c r="AB45" s="4" t="n">
-        <v>49.257645</v>
+        <v>48.180496</v>
       </c>
       <c r="AC45" s="4" t="n">
-        <v>37.798206</v>
+        <v>37.098824</v>
       </c>
       <c r="AD45" s="4" t="inlineStr"/>
       <c r="AE45" s="4" t="n">
@@ -6419,7 +6417,7 @@
         <v>62.1</v>
       </c>
       <c r="AH45" s="4" t="n">
-        <v>17.428116</v>
+        <v>17.047005</v>
       </c>
       <c r="AI45" s="4" t="n">
         <v>30</v>
@@ -6530,13 +6528,13 @@
         <v>1.06</v>
       </c>
       <c r="AA46" s="2" t="n">
-        <v>206715</v>
+        <v>204587</v>
       </c>
       <c r="AB46" s="2" t="n">
-        <v>35.84178</v>
+        <v>35.472893</v>
       </c>
       <c r="AC46" s="2" t="n">
-        <v>27.720856</v>
+        <v>27.435549</v>
       </c>
       <c r="AD46" s="2" t="inlineStr"/>
       <c r="AE46" s="2" t="n">
@@ -6549,10 +6547,10 @@
         <v>21.3</v>
       </c>
       <c r="AH46" s="2" t="n">
-        <v>8.229373000000001</v>
+        <v>8.144674999999999</v>
       </c>
       <c r="AI46" s="2" t="n">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="AJ46" s="2" t="inlineStr"/>
       <c r="AK46" s="2" t="inlineStr">
@@ -6569,32 +6567,32 @@
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
         <is>
-          <t>DEVYANI</t>
+          <t>SIEMENS</t>
         </is>
       </c>
       <c r="B47" s="4" t="inlineStr">
         <is>
-          <t>Devyani International Limited</t>
+          <t>Siemens Limited</t>
         </is>
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>Consumer Cyclical</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>Restaurants</t>
+          <t>Specialty Industrial Machinery</t>
         </is>
       </c>
       <c r="E47" s="6" t="n">
-        <v>43.8</v>
+        <v>44.2</v>
       </c>
       <c r="F47" s="4" t="n">
-        <v>25.6</v>
+        <v>24.8</v>
       </c>
       <c r="G47" s="4" t="n">
-        <v>18.2</v>
+        <v>19.4</v>
       </c>
       <c r="H47" s="6" t="inlineStr">
         <is>
@@ -6603,23 +6601,23 @@
       </c>
       <c r="I47" s="4" t="inlineStr">
         <is>
-          <t>✅ Supertrend Buy | 📈 EMA Bull Stack | 📉 Tight Base</t>
+          <t>✅ Supertrend Buy | 📈 EMA Bull Stack | 🏆 Near 52W High | 📉 Tight Base | 👤 High Promoter</t>
         </is>
       </c>
       <c r="J47" s="4" t="n">
-        <v>137.97</v>
+        <v>3957</v>
       </c>
       <c r="K47" s="4" t="n">
-        <v>1.51</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="L47" s="4" t="n">
-        <v>138.18</v>
+        <v>3967.66</v>
       </c>
       <c r="M47" s="4" t="n">
-        <v>131.31</v>
+        <v>3871.69</v>
       </c>
       <c r="N47" s="4" t="n">
-        <v>128.93</v>
+        <v>3554.51</v>
       </c>
       <c r="O47" s="4" t="inlineStr">
         <is>
@@ -6632,97 +6630,99 @@
         </is>
       </c>
       <c r="Q47" s="4" t="n">
-        <v>72.23999999999999</v>
+        <v>95.36</v>
       </c>
       <c r="R47" s="4" t="n">
-        <v>52.63</v>
+        <v>51.18</v>
       </c>
       <c r="S47" s="4" t="n">
-        <v>2.0762</v>
+        <v>26.3831</v>
       </c>
       <c r="T47" s="4" t="n">
-        <v>3.8089</v>
+        <v>47.9326</v>
       </c>
       <c r="U47" s="4" t="n">
-        <v>-1.7327</v>
+        <v>-21.5495</v>
       </c>
       <c r="V47" s="4" t="inlineStr"/>
       <c r="W47" s="4" t="n">
-        <v>38.43</v>
+        <v>23.5</v>
       </c>
       <c r="X47" s="4" t="n">
-        <v>2136370</v>
+        <v>172514</v>
       </c>
       <c r="Y47" s="4" t="n">
-        <v>3344274</v>
+        <v>338996</v>
       </c>
       <c r="Z47" s="4" t="n">
-        <v>0.64</v>
+        <v>0.51</v>
       </c>
       <c r="AA47" s="4" t="n">
-        <v>17015</v>
-      </c>
-      <c r="AB47" s="4" t="inlineStr"/>
+        <v>134257</v>
+      </c>
+      <c r="AB47" s="4" t="n">
+        <v>79.401855</v>
+      </c>
       <c r="AC47" s="4" t="n">
-        <v>133.11726</v>
+        <v>55.62931</v>
       </c>
       <c r="AD47" s="4" t="inlineStr"/>
       <c r="AE47" s="4" t="n">
-        <v>203.327</v>
+        <v>2.213</v>
       </c>
       <c r="AF47" s="4" t="n">
-        <v>16.5</v>
+        <v>14.8</v>
       </c>
       <c r="AG47" s="4" t="n">
-        <v>300</v>
+        <v>406.1</v>
       </c>
       <c r="AH47" s="4" t="n">
-        <v>11.035585</v>
+        <v>9.700544000000001</v>
       </c>
       <c r="AI47" s="4" t="n">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="AJ47" s="4" t="inlineStr"/>
       <c r="AK47" s="4" t="inlineStr">
         <is>
-          <t>https://www.screener.in/company/DEVYANI/</t>
+          <t>https://www.screener.in/company/SIEMENS/</t>
         </is>
       </c>
       <c r="AL47" s="4" t="inlineStr">
         <is>
-          <t>https://www.tradingview.com/chart/?symbol=NSE:DEVYANI</t>
+          <t>https://www.tradingview.com/chart/?symbol=NSE:SIEMENS</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>BAJAJCON</t>
+          <t>DEVYANI</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Bajaj Consumer Care Limited</t>
+          <t>Devyani International Limited</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>Consumer Defensive</t>
+          <t>Consumer Cyclical</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>Household &amp; Personal Products</t>
+          <t>Restaurants</t>
         </is>
       </c>
       <c r="E48" s="6" t="n">
         <v>43.8</v>
       </c>
       <c r="F48" s="2" t="n">
-        <v>22.6</v>
+        <v>25.6</v>
       </c>
       <c r="G48" s="2" t="n">
-        <v>21.2</v>
+        <v>18.2</v>
       </c>
       <c r="H48" s="6" t="inlineStr">
         <is>
@@ -6731,27 +6731,27 @@
       </c>
       <c r="I48" s="2" t="inlineStr">
         <is>
-          <t>✅ Supertrend Buy | 🎯 VCP Pattern</t>
+          <t>✅ Supertrend Buy | 📈 EMA Bull Stack | 📉 Tight Base</t>
         </is>
       </c>
       <c r="J48" s="2" t="n">
-        <v>520.5</v>
+        <v>137.97</v>
       </c>
       <c r="K48" s="2" t="n">
-        <v>-0.75</v>
+        <v>1.51</v>
       </c>
       <c r="L48" s="2" t="n">
-        <v>503.87</v>
+        <v>138.18</v>
       </c>
       <c r="M48" s="2" t="n">
-        <v>518.42</v>
+        <v>131.31</v>
       </c>
       <c r="N48" s="2" t="n">
-        <v>454.21</v>
+        <v>128.93</v>
       </c>
       <c r="O48" s="2" t="inlineStr">
         <is>
-          <t>✗</t>
+          <t>✓</t>
         </is>
       </c>
       <c r="P48" s="2" t="inlineStr">
@@ -6760,54 +6760,52 @@
         </is>
       </c>
       <c r="Q48" s="2" t="n">
-        <v>75.22</v>
+        <v>72.23999999999999</v>
       </c>
       <c r="R48" s="2" t="n">
-        <v>54.95</v>
+        <v>52.63</v>
       </c>
       <c r="S48" s="2" t="n">
-        <v>-2.2248</v>
+        <v>2.0762</v>
       </c>
       <c r="T48" s="2" t="n">
-        <v>-10.7361</v>
+        <v>3.8089</v>
       </c>
       <c r="U48" s="2" t="n">
-        <v>8.5113</v>
+        <v>-1.7327</v>
       </c>
       <c r="V48" s="2" t="inlineStr"/>
       <c r="W48" s="2" t="n">
-        <v>18.88</v>
+        <v>38.43</v>
       </c>
       <c r="X48" s="2" t="n">
-        <v>901856</v>
+        <v>2136370</v>
       </c>
       <c r="Y48" s="2" t="n">
-        <v>1026158</v>
+        <v>3344274</v>
       </c>
       <c r="Z48" s="2" t="n">
-        <v>0.88</v>
+        <v>0.64</v>
       </c>
       <c r="AA48" s="2" t="n">
-        <v>6825</v>
-      </c>
-      <c r="AB48" s="2" t="n">
-        <v>30.990509</v>
-      </c>
+        <v>16795</v>
+      </c>
+      <c r="AB48" s="2" t="inlineStr"/>
       <c r="AC48" s="2" t="n">
-        <v>23.078623</v>
+        <v>131.40024</v>
       </c>
       <c r="AD48" s="2" t="inlineStr"/>
       <c r="AE48" s="2" t="n">
-        <v>2.092</v>
+        <v>203.327</v>
       </c>
       <c r="AF48" s="2" t="n">
-        <v>28.1</v>
+        <v>16.5</v>
       </c>
       <c r="AG48" s="2" t="n">
-        <v>95.7</v>
+        <v>300</v>
       </c>
       <c r="AH48" s="2" t="n">
-        <v>9.265827</v>
+        <v>10.893243</v>
       </c>
       <c r="AI48" s="2" t="n">
         <v>0</v>
@@ -6815,44 +6813,44 @@
       <c r="AJ48" s="2" t="inlineStr"/>
       <c r="AK48" s="2" t="inlineStr">
         <is>
-          <t>https://www.screener.in/company/BAJAJCON/</t>
+          <t>https://www.screener.in/company/DEVYANI/</t>
         </is>
       </c>
       <c r="AL48" s="2" t="inlineStr">
         <is>
-          <t>https://www.tradingview.com/chart/?symbol=NSE:BAJAJCON</t>
+          <t>https://www.tradingview.com/chart/?symbol=NSE:DEVYANI</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
         <is>
-          <t>TITAN</t>
+          <t>BAJAJCON</t>
         </is>
       </c>
       <c r="B49" s="4" t="inlineStr">
         <is>
-          <t>Titan Company Limited</t>
+          <t>Bajaj Consumer Care Limited</t>
         </is>
       </c>
       <c r="C49" s="4" t="inlineStr">
         <is>
-          <t>Consumer Cyclical</t>
+          <t>Consumer Defensive</t>
         </is>
       </c>
       <c r="D49" s="4" t="inlineStr">
         <is>
-          <t>Luxury Goods</t>
+          <t>Household &amp; Personal Products</t>
         </is>
       </c>
       <c r="E49" s="6" t="n">
-        <v>43.5</v>
+        <v>43.8</v>
       </c>
       <c r="F49" s="4" t="n">
-        <v>24.8</v>
+        <v>22.6</v>
       </c>
       <c r="G49" s="4" t="n">
-        <v>18.7</v>
+        <v>21.2</v>
       </c>
       <c r="H49" s="6" t="inlineStr">
         <is>
@@ -6861,27 +6859,27 @@
       </c>
       <c r="I49" s="4" t="inlineStr">
         <is>
-          <t>✅ Supertrend Buy | 📈 EMA Bull Stack | 🏆 Near 52W High | 📉 Tight Base</t>
+          <t>✅ Supertrend Buy | 🎯 VCP Pattern</t>
         </is>
       </c>
       <c r="J49" s="4" t="n">
-        <v>5009.5</v>
+        <v>520.5</v>
       </c>
       <c r="K49" s="4" t="n">
-        <v>-0.23</v>
+        <v>-0.75</v>
       </c>
       <c r="L49" s="4" t="n">
-        <v>5025.17</v>
+        <v>503.87</v>
       </c>
       <c r="M49" s="4" t="n">
-        <v>4882.7</v>
+        <v>518.42</v>
       </c>
       <c r="N49" s="4" t="n">
-        <v>4389.01</v>
+        <v>454.21</v>
       </c>
       <c r="O49" s="4" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>✗</t>
         </is>
       </c>
       <c r="P49" s="4" t="inlineStr">
@@ -6890,99 +6888,99 @@
         </is>
       </c>
       <c r="Q49" s="4" t="n">
-        <v>96.58</v>
+        <v>75.22</v>
       </c>
       <c r="R49" s="4" t="n">
-        <v>51.21</v>
+        <v>54.95</v>
       </c>
       <c r="S49" s="4" t="n">
-        <v>27.0005</v>
+        <v>-2.2248</v>
       </c>
       <c r="T49" s="4" t="n">
-        <v>52.504</v>
+        <v>-10.7361</v>
       </c>
       <c r="U49" s="4" t="n">
-        <v>-25.5035</v>
+        <v>8.5113</v>
       </c>
       <c r="V49" s="4" t="inlineStr"/>
       <c r="W49" s="4" t="n">
-        <v>28</v>
+        <v>18.88</v>
       </c>
       <c r="X49" s="4" t="n">
-        <v>403235</v>
+        <v>901856</v>
       </c>
       <c r="Y49" s="4" t="n">
-        <v>493929</v>
+        <v>1026158</v>
       </c>
       <c r="Z49" s="4" t="n">
-        <v>0.82</v>
+        <v>0.88</v>
       </c>
       <c r="AA49" s="4" t="n">
-        <v>444499</v>
+        <v>6581</v>
       </c>
       <c r="AB49" s="4" t="n">
-        <v>76.92721</v>
+        <v>29.881374</v>
       </c>
       <c r="AC49" s="4" t="n">
-        <v>56.3325</v>
+        <v>22.25265</v>
       </c>
       <c r="AD49" s="4" t="inlineStr"/>
       <c r="AE49" s="4" t="n">
-        <v>195.001</v>
+        <v>2.092</v>
       </c>
       <c r="AF49" s="4" t="n">
-        <v>29.3</v>
+        <v>28.1</v>
       </c>
       <c r="AG49" s="4" t="n">
-        <v>62.8</v>
+        <v>95.7</v>
       </c>
       <c r="AH49" s="4" t="n">
-        <v>28.32178</v>
+        <v>8.934208</v>
       </c>
       <c r="AI49" s="4" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="AJ49" s="4" t="inlineStr"/>
       <c r="AK49" s="4" t="inlineStr">
         <is>
-          <t>https://www.screener.in/company/TITAN/</t>
+          <t>https://www.screener.in/company/BAJAJCON/</t>
         </is>
       </c>
       <c r="AL49" s="4" t="inlineStr">
         <is>
-          <t>https://www.tradingview.com/chart/?symbol=NSE:TITAN</t>
+          <t>https://www.tradingview.com/chart/?symbol=NSE:BAJAJCON</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>BAJFINANCE</t>
+          <t>TITAN</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>Bajaj Finance Limited</t>
+          <t>Titan Company Limited</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>Financial Services</t>
+          <t>Consumer Cyclical</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>Credit Services</t>
+          <t>Luxury Goods</t>
         </is>
       </c>
       <c r="E50" s="6" t="n">
-        <v>42.8</v>
+        <v>43.5</v>
       </c>
       <c r="F50" s="2" t="n">
-        <v>21.6</v>
+        <v>24.8</v>
       </c>
       <c r="G50" s="2" t="n">
-        <v>21.2</v>
+        <v>18.7</v>
       </c>
       <c r="H50" s="6" t="inlineStr">
         <is>
@@ -6991,23 +6989,23 @@
       </c>
       <c r="I50" s="2" t="inlineStr">
         <is>
-          <t>📈 EMA Bull Stack | 📉 Tight Base</t>
+          <t>✅ Supertrend Buy | 📈 EMA Bull Stack | 🏆 Near 52W High | 📉 Tight Base</t>
         </is>
       </c>
       <c r="J50" s="2" t="n">
-        <v>1034.5</v>
+        <v>5009.5</v>
       </c>
       <c r="K50" s="2" t="n">
-        <v>-0.86</v>
+        <v>-0.23</v>
       </c>
       <c r="L50" s="2" t="n">
-        <v>1062.18</v>
+        <v>5025.17</v>
       </c>
       <c r="M50" s="2" t="n">
-        <v>1051.74</v>
+        <v>4882.7</v>
       </c>
       <c r="N50" s="2" t="n">
-        <v>987.7</v>
+        <v>4389.01</v>
       </c>
       <c r="O50" s="2" t="inlineStr">
         <is>
@@ -7016,103 +7014,103 @@
       </c>
       <c r="P50" s="2" t="inlineStr">
         <is>
-          <t>Sell</t>
+          <t>Buy</t>
         </is>
       </c>
       <c r="Q50" s="2" t="n">
-        <v>87.94</v>
+        <v>96.58</v>
       </c>
       <c r="R50" s="2" t="n">
-        <v>38.18</v>
+        <v>51.21</v>
       </c>
       <c r="S50" s="2" t="n">
-        <v>-8.506399999999999</v>
+        <v>27.0005</v>
       </c>
       <c r="T50" s="2" t="n">
-        <v>-3.1581</v>
+        <v>52.504</v>
       </c>
       <c r="U50" s="2" t="n">
-        <v>-5.3483</v>
+        <v>-25.5035</v>
       </c>
       <c r="V50" s="2" t="inlineStr"/>
       <c r="W50" s="2" t="n">
-        <v>20.11</v>
+        <v>28</v>
       </c>
       <c r="X50" s="2" t="n">
-        <v>5411299</v>
+        <v>403235</v>
       </c>
       <c r="Y50" s="2" t="n">
-        <v>4741846</v>
+        <v>493929</v>
       </c>
       <c r="Z50" s="2" t="n">
-        <v>1.14</v>
+        <v>0.82</v>
       </c>
       <c r="AA50" s="2" t="n">
-        <v>643553</v>
+        <v>430879</v>
       </c>
       <c r="AB50" s="2" t="n">
-        <v>31.772112</v>
+        <v>74.57002</v>
       </c>
       <c r="AC50" s="2" t="n">
-        <v>20.47806</v>
+        <v>54.60637</v>
       </c>
       <c r="AD50" s="2" t="inlineStr"/>
       <c r="AE50" s="2" t="n">
-        <v>314.833</v>
+        <v>195.001</v>
       </c>
       <c r="AF50" s="2" t="n">
-        <v>26.1</v>
+        <v>29.3</v>
       </c>
       <c r="AG50" s="2" t="n">
-        <v>27.2</v>
+        <v>62.8</v>
       </c>
       <c r="AH50" s="2" t="n">
-        <v>5.6424913</v>
+        <v>27.45395</v>
       </c>
       <c r="AI50" s="2" t="n">
-        <v>52</v>
+        <v>30</v>
       </c>
       <c r="AJ50" s="2" t="inlineStr"/>
       <c r="AK50" s="2" t="inlineStr">
         <is>
-          <t>https://www.screener.in/company/BAJFINANCE/</t>
+          <t>https://www.screener.in/company/TITAN/</t>
         </is>
       </c>
       <c r="AL50" s="2" t="inlineStr">
         <is>
-          <t>https://www.tradingview.com/chart/?symbol=NSE:BAJFINANCE</t>
+          <t>https://www.tradingview.com/chart/?symbol=NSE:TITAN</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
         <is>
-          <t>OBEROIRLTY</t>
+          <t>BAJFINANCE</t>
         </is>
       </c>
       <c r="B51" s="4" t="inlineStr">
         <is>
-          <t>Oberoi Realty Limited</t>
+          <t>Bajaj Finance Limited</t>
         </is>
       </c>
       <c r="C51" s="4" t="inlineStr">
         <is>
-          <t>Real Estate</t>
+          <t>Financial Services</t>
         </is>
       </c>
       <c r="D51" s="4" t="inlineStr">
         <is>
-          <t>Real Estate - Development</t>
+          <t>Credit Services</t>
         </is>
       </c>
       <c r="E51" s="6" t="n">
-        <v>42.7</v>
+        <v>42.8</v>
       </c>
       <c r="F51" s="4" t="n">
-        <v>16.8</v>
+        <v>21.6</v>
       </c>
       <c r="G51" s="4" t="n">
-        <v>25.9</v>
+        <v>21.2</v>
       </c>
       <c r="H51" s="6" t="inlineStr">
         <is>
@@ -7125,19 +7123,19 @@
         </is>
       </c>
       <c r="J51" s="4" t="n">
-        <v>1741.1</v>
+        <v>1034.5</v>
       </c>
       <c r="K51" s="4" t="n">
-        <v>-2.84</v>
+        <v>-0.86</v>
       </c>
       <c r="L51" s="4" t="n">
-        <v>1839.03</v>
+        <v>1062.18</v>
       </c>
       <c r="M51" s="4" t="n">
-        <v>1825.71</v>
+        <v>1051.74</v>
       </c>
       <c r="N51" s="4" t="n">
-        <v>1718.2</v>
+        <v>987.7</v>
       </c>
       <c r="O51" s="4" t="inlineStr">
         <is>
@@ -7150,99 +7148,99 @@
         </is>
       </c>
       <c r="Q51" s="4" t="n">
-        <v>87.76000000000001</v>
+        <v>87.94</v>
       </c>
       <c r="R51" s="4" t="n">
-        <v>33.3</v>
+        <v>38.18</v>
       </c>
       <c r="S51" s="4" t="n">
-        <v>-11.61</v>
+        <v>-8.506399999999999</v>
       </c>
       <c r="T51" s="4" t="n">
-        <v>3.5206</v>
+        <v>-3.1581</v>
       </c>
       <c r="U51" s="4" t="n">
-        <v>-15.1306</v>
+        <v>-5.3483</v>
       </c>
       <c r="V51" s="4" t="inlineStr"/>
       <c r="W51" s="4" t="n">
-        <v>17.09</v>
+        <v>20.11</v>
       </c>
       <c r="X51" s="4" t="n">
-        <v>543198</v>
+        <v>5411299</v>
       </c>
       <c r="Y51" s="4" t="n">
-        <v>534782</v>
+        <v>4741846</v>
       </c>
       <c r="Z51" s="4" t="n">
-        <v>1.02</v>
+        <v>1.14</v>
       </c>
       <c r="AA51" s="4" t="n">
-        <v>63307</v>
+        <v>627815</v>
       </c>
       <c r="AB51" s="4" t="n">
-        <v>24.094934</v>
+        <v>30.966555</v>
       </c>
       <c r="AC51" s="4" t="n">
-        <v>16.313793</v>
+        <v>19.977243</v>
       </c>
       <c r="AD51" s="4" t="inlineStr"/>
       <c r="AE51" s="4" t="n">
-        <v>15.765</v>
+        <v>314.833</v>
       </c>
       <c r="AF51" s="4" t="n">
-        <v>31.7</v>
+        <v>26.1</v>
       </c>
       <c r="AG51" s="4" t="n">
-        <v>28.9</v>
+        <v>27.2</v>
       </c>
       <c r="AH51" s="4" t="n">
-        <v>3.532424</v>
+        <v>5.504497</v>
       </c>
       <c r="AI51" s="4" t="n">
-        <v>45</v>
+        <v>52</v>
       </c>
       <c r="AJ51" s="4" t="inlineStr"/>
       <c r="AK51" s="4" t="inlineStr">
         <is>
-          <t>https://www.screener.in/company/OBEROIRLTY/</t>
+          <t>https://www.screener.in/company/BAJFINANCE/</t>
         </is>
       </c>
       <c r="AL51" s="4" t="inlineStr">
         <is>
-          <t>https://www.tradingview.com/chart/?symbol=NSE:OBEROIRLTY</t>
+          <t>https://www.tradingview.com/chart/?symbol=NSE:BAJFINANCE</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>ICICIBANK</t>
+          <t>OBEROIRLTY</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>ICICI Bank Limited</t>
+          <t>Oberoi Realty Limited</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>Financial Services</t>
+          <t>Real Estate</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>Banks - Regional</t>
+          <t>Real Estate - Development</t>
         </is>
       </c>
       <c r="E52" s="6" t="n">
-        <v>42.4</v>
+        <v>42.7</v>
       </c>
       <c r="F52" s="2" t="n">
-        <v>14.4</v>
+        <v>16.8</v>
       </c>
       <c r="G52" s="2" t="n">
-        <v>28</v>
+        <v>25.9</v>
       </c>
       <c r="H52" s="6" t="inlineStr">
         <is>
@@ -7251,23 +7249,23 @@
       </c>
       <c r="I52" s="2" t="inlineStr">
         <is>
-          <t>📈 EMA Bull Stack | 🏆 Near 52W High | 📉 Tight Base</t>
+          <t>📈 EMA Bull Stack | 📉 Tight Base</t>
         </is>
       </c>
       <c r="J52" s="2" t="n">
-        <v>1379.3</v>
+        <v>1741.1</v>
       </c>
       <c r="K52" s="2" t="n">
-        <v>-0.38</v>
+        <v>-2.84</v>
       </c>
       <c r="L52" s="2" t="n">
-        <v>1413.67</v>
+        <v>1839.03</v>
       </c>
       <c r="M52" s="2" t="n">
-        <v>1404.33</v>
+        <v>1825.71</v>
       </c>
       <c r="N52" s="2" t="n">
-        <v>1368.17</v>
+        <v>1718.2</v>
       </c>
       <c r="O52" s="2" t="inlineStr">
         <is>
@@ -7280,79 +7278,79 @@
         </is>
       </c>
       <c r="Q52" s="2" t="n">
-        <v>93.98</v>
+        <v>87.76000000000001</v>
       </c>
       <c r="R52" s="2" t="n">
-        <v>37.69</v>
+        <v>33.3</v>
       </c>
       <c r="S52" s="2" t="n">
-        <v>-6.3513</v>
+        <v>-11.61</v>
       </c>
       <c r="T52" s="2" t="n">
-        <v>0.2673</v>
+        <v>3.5206</v>
       </c>
       <c r="U52" s="2" t="n">
-        <v>-6.6186</v>
+        <v>-15.1306</v>
       </c>
       <c r="V52" s="2" t="inlineStr"/>
       <c r="W52" s="2" t="n">
-        <v>16.47</v>
+        <v>17.09</v>
       </c>
       <c r="X52" s="2" t="n">
-        <v>7064417</v>
+        <v>543198</v>
       </c>
       <c r="Y52" s="2" t="n">
-        <v>8929162</v>
+        <v>534782</v>
       </c>
       <c r="Z52" s="2" t="n">
-        <v>0.79</v>
+        <v>1.02</v>
       </c>
       <c r="AA52" s="2" t="n">
-        <v>990020</v>
+        <v>60667</v>
       </c>
       <c r="AB52" s="2" t="n">
-        <v>17.82502</v>
+        <v>23.090229</v>
       </c>
       <c r="AC52" s="2" t="n">
-        <v>14.673405</v>
-      </c>
-      <c r="AD52" s="2" t="n">
-        <v>16.07</v>
-      </c>
-      <c r="AE52" s="2" t="inlineStr"/>
+        <v>15.633544</v>
+      </c>
+      <c r="AD52" s="2" t="inlineStr"/>
+      <c r="AE52" s="2" t="n">
+        <v>15.765</v>
+      </c>
       <c r="AF52" s="2" t="n">
-        <v>11.4</v>
+        <v>31.7</v>
       </c>
       <c r="AG52" s="2" t="n">
-        <v>13.8</v>
+        <v>28.9</v>
       </c>
       <c r="AH52" s="2" t="n">
-        <v>2.600603</v>
+        <v>3.38513</v>
       </c>
       <c r="AI52" s="2" t="n">
-        <v>87</v>
+        <v>46</v>
       </c>
       <c r="AJ52" s="2" t="inlineStr"/>
       <c r="AK52" s="2" t="inlineStr">
         <is>
-          <t>https://www.screener.in/company/ICICIBANK/</t>
+          <t>https://www.screener.in/company/OBEROIRLTY/</t>
         </is>
       </c>
       <c r="AL52" s="2" t="inlineStr">
         <is>
-          <t>https://www.tradingview.com/chart/?symbol=NSE:ICICIBANK</t>
+          <t>https://www.tradingview.com/chart/?symbol=NSE:OBEROIRLTY</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="4" t="inlineStr">
         <is>
-          <t>BAJAJFINSV</t>
+          <t>ICICIBANK</t>
         </is>
       </c>
       <c r="B53" s="4" t="inlineStr">
         <is>
-          <t>Bajaj Finserv Ltd.</t>
+          <t>ICICI Bank Limited</t>
         </is>
       </c>
       <c r="C53" s="4" t="inlineStr">
@@ -7362,17 +7360,17 @@
       </c>
       <c r="D53" s="4" t="inlineStr">
         <is>
-          <t>Financial Conglomerates</t>
+          <t>Banks - Regional</t>
         </is>
       </c>
       <c r="E53" s="6" t="n">
-        <v>42.3</v>
+        <v>42.4</v>
       </c>
       <c r="F53" s="4" t="n">
-        <v>21.6</v>
+        <v>14.4</v>
       </c>
       <c r="G53" s="4" t="n">
-        <v>20.7</v>
+        <v>28</v>
       </c>
       <c r="H53" s="6" t="inlineStr">
         <is>
@@ -7381,23 +7379,23 @@
       </c>
       <c r="I53" s="4" t="inlineStr">
         <is>
-          <t>📈 EMA Bull Stack | 📉 Tight Base</t>
+          <t>📈 EMA Bull Stack | 🏆 Near 52W High | 📉 Tight Base</t>
         </is>
       </c>
       <c r="J53" s="4" t="n">
-        <v>1913.5</v>
+        <v>1379.3</v>
       </c>
       <c r="K53" s="4" t="n">
-        <v>-1.39</v>
+        <v>-0.38</v>
       </c>
       <c r="L53" s="4" t="n">
-        <v>1969.95</v>
+        <v>1413.67</v>
       </c>
       <c r="M53" s="4" t="n">
-        <v>1947.5</v>
+        <v>1404.33</v>
       </c>
       <c r="N53" s="4" t="n">
-        <v>1909.48</v>
+        <v>1368.17</v>
       </c>
       <c r="O53" s="4" t="inlineStr">
         <is>
@@ -7410,99 +7408,99 @@
         </is>
       </c>
       <c r="Q53" s="4" t="n">
-        <v>87.25</v>
+        <v>93.98</v>
       </c>
       <c r="R53" s="4" t="n">
-        <v>37.4</v>
+        <v>37.69</v>
       </c>
       <c r="S53" s="4" t="n">
-        <v>-11.4508</v>
+        <v>-6.3513</v>
       </c>
       <c r="T53" s="4" t="n">
-        <v>1.7117</v>
+        <v>0.2673</v>
       </c>
       <c r="U53" s="4" t="n">
-        <v>-13.1625</v>
+        <v>-6.6186</v>
       </c>
       <c r="V53" s="4" t="inlineStr"/>
       <c r="W53" s="4" t="n">
-        <v>24.04</v>
+        <v>16.47</v>
       </c>
       <c r="X53" s="4" t="n">
-        <v>762375</v>
+        <v>7064417</v>
       </c>
       <c r="Y53" s="4" t="n">
-        <v>620459</v>
+        <v>8929162</v>
       </c>
       <c r="Z53" s="4" t="n">
-        <v>1.23</v>
+        <v>0.79</v>
       </c>
       <c r="AA53" s="4" t="n">
-        <v>306207</v>
+        <v>969277</v>
       </c>
       <c r="AB53" s="4" t="n">
-        <v>30.30087</v>
+        <v>17.451538</v>
       </c>
       <c r="AC53" s="4" t="n">
-        <v>20.15821</v>
-      </c>
-      <c r="AD53" s="4" t="inlineStr"/>
-      <c r="AE53" s="4" t="n">
-        <v>256.404</v>
-      </c>
+        <v>14.365957</v>
+      </c>
+      <c r="AD53" s="4" t="n">
+        <v>16.07</v>
+      </c>
+      <c r="AE53" s="4" t="inlineStr"/>
       <c r="AF53" s="4" t="n">
-        <v>19.3</v>
+        <v>11.4</v>
       </c>
       <c r="AG53" s="4" t="n">
-        <v>12.7</v>
+        <v>13.8</v>
       </c>
       <c r="AH53" s="4" t="n">
-        <v>3.9263203</v>
+        <v>2.5461135</v>
       </c>
       <c r="AI53" s="4" t="n">
-        <v>7</v>
+        <v>87</v>
       </c>
       <c r="AJ53" s="4" t="inlineStr"/>
       <c r="AK53" s="4" t="inlineStr">
         <is>
-          <t>https://www.screener.in/company/BAJAJFINSV/</t>
+          <t>https://www.screener.in/company/ICICIBANK/</t>
         </is>
       </c>
       <c r="AL53" s="4" t="inlineStr">
         <is>
-          <t>https://www.tradingview.com/chart/?symbol=NSE:BAJAJFINSV</t>
+          <t>https://www.tradingview.com/chart/?symbol=NSE:ICICIBANK</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>HEROMOTOCO</t>
+          <t>BAJAJFINSV</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>Hero MotoCorp Limited</t>
+          <t>Bajaj Finserv Ltd.</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>Consumer Cyclical</t>
+          <t>Financial Services</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>Auto Manufacturers</t>
+          <t>Financial Conglomerates</t>
         </is>
       </c>
       <c r="E54" s="6" t="n">
         <v>42.3</v>
       </c>
       <c r="F54" s="2" t="n">
-        <v>20</v>
+        <v>21.6</v>
       </c>
       <c r="G54" s="2" t="n">
-        <v>22.3</v>
+        <v>20.7</v>
       </c>
       <c r="H54" s="6" t="inlineStr">
         <is>
@@ -7515,19 +7513,19 @@
         </is>
       </c>
       <c r="J54" s="2" t="n">
-        <v>5221.5</v>
+        <v>1913.5</v>
       </c>
       <c r="K54" s="2" t="n">
-        <v>-1.11</v>
+        <v>-1.39</v>
       </c>
       <c r="L54" s="2" t="n">
-        <v>5410.18</v>
+        <v>1969.95</v>
       </c>
       <c r="M54" s="2" t="n">
-        <v>5350.88</v>
+        <v>1947.5</v>
       </c>
       <c r="N54" s="2" t="n">
-        <v>5177.17</v>
+        <v>1909.48</v>
       </c>
       <c r="O54" s="2" t="inlineStr">
         <is>
@@ -7540,99 +7538,99 @@
         </is>
       </c>
       <c r="Q54" s="2" t="n">
-        <v>84.55</v>
+        <v>87.25</v>
       </c>
       <c r="R54" s="2" t="n">
-        <v>39.04</v>
+        <v>37.4</v>
       </c>
       <c r="S54" s="2" t="n">
-        <v>-57.624</v>
+        <v>-11.4508</v>
       </c>
       <c r="T54" s="2" t="n">
-        <v>-5.0728</v>
+        <v>1.7117</v>
       </c>
       <c r="U54" s="2" t="n">
-        <v>-52.5512</v>
+        <v>-13.1625</v>
       </c>
       <c r="V54" s="2" t="inlineStr"/>
       <c r="W54" s="2" t="n">
-        <v>33.38</v>
+        <v>24.04</v>
       </c>
       <c r="X54" s="2" t="n">
-        <v>251663</v>
+        <v>762375</v>
       </c>
       <c r="Y54" s="2" t="n">
-        <v>535409</v>
+        <v>620459</v>
       </c>
       <c r="Z54" s="2" t="n">
-        <v>0.47</v>
+        <v>1.23</v>
       </c>
       <c r="AA54" s="2" t="n">
-        <v>104504</v>
+        <v>296925</v>
       </c>
       <c r="AB54" s="2" t="n">
-        <v>19.202337</v>
+        <v>29.382421</v>
       </c>
       <c r="AC54" s="2" t="n">
-        <v>16.035471</v>
+        <v>19.547195</v>
       </c>
       <c r="AD54" s="2" t="inlineStr"/>
       <c r="AE54" s="2" t="n">
-        <v>3.57</v>
+        <v>256.404</v>
       </c>
       <c r="AF54" s="2" t="n">
-        <v>34.9</v>
+        <v>19.3</v>
       </c>
       <c r="AG54" s="2" t="n">
-        <v>-17.2</v>
+        <v>12.7</v>
       </c>
       <c r="AH54" s="2" t="n">
-        <v>4.834387</v>
+        <v>3.8073099</v>
       </c>
       <c r="AI54" s="2" t="n">
-        <v>354</v>
+        <v>7</v>
       </c>
       <c r="AJ54" s="2" t="inlineStr"/>
       <c r="AK54" s="2" t="inlineStr">
         <is>
-          <t>https://www.screener.in/company/HEROMOTOCO/</t>
+          <t>https://www.screener.in/company/BAJAJFINSV/</t>
         </is>
       </c>
       <c r="AL54" s="2" t="inlineStr">
         <is>
-          <t>https://www.tradingview.com/chart/?symbol=NSE:HEROMOTOCO</t>
+          <t>https://www.tradingview.com/chart/?symbol=NSE:BAJAJFINSV</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
         <is>
-          <t>SIEMENS</t>
+          <t>HEROMOTOCO</t>
         </is>
       </c>
       <c r="B55" s="4" t="inlineStr">
         <is>
-          <t>Siemens Limited</t>
+          <t>Hero MotoCorp Limited</t>
         </is>
       </c>
       <c r="C55" s="4" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Consumer Cyclical</t>
         </is>
       </c>
       <c r="D55" s="4" t="inlineStr">
         <is>
-          <t>Specialty Industrial Machinery</t>
+          <t>Auto Manufacturers</t>
         </is>
       </c>
       <c r="E55" s="6" t="n">
-        <v>42.1</v>
+        <v>42.3</v>
       </c>
       <c r="F55" s="4" t="n">
-        <v>24.8</v>
+        <v>20</v>
       </c>
       <c r="G55" s="4" t="n">
-        <v>17.3</v>
+        <v>22.3</v>
       </c>
       <c r="H55" s="6" t="inlineStr">
         <is>
@@ -7641,23 +7639,23 @@
       </c>
       <c r="I55" s="4" t="inlineStr">
         <is>
-          <t>✅ Supertrend Buy | 📈 EMA Bull Stack | 🏆 Near 52W High | 📉 Tight Base | 👤 High Promoter</t>
+          <t>📈 EMA Bull Stack | 📉 Tight Base</t>
         </is>
       </c>
       <c r="J55" s="4" t="n">
-        <v>3957</v>
+        <v>5221.5</v>
       </c>
       <c r="K55" s="4" t="n">
-        <v>0.07000000000000001</v>
+        <v>-1.11</v>
       </c>
       <c r="L55" s="4" t="n">
-        <v>3967.66</v>
+        <v>5410.18</v>
       </c>
       <c r="M55" s="4" t="n">
-        <v>3871.69</v>
+        <v>5350.88</v>
       </c>
       <c r="N55" s="4" t="n">
-        <v>3554.51</v>
+        <v>5177.17</v>
       </c>
       <c r="O55" s="4" t="inlineStr">
         <is>
@@ -7666,71 +7664,71 @@
       </c>
       <c r="P55" s="4" t="inlineStr">
         <is>
-          <t>Buy</t>
+          <t>Sell</t>
         </is>
       </c>
       <c r="Q55" s="4" t="n">
-        <v>95.36</v>
+        <v>84.55</v>
       </c>
       <c r="R55" s="4" t="n">
-        <v>51.18</v>
+        <v>39.04</v>
       </c>
       <c r="S55" s="4" t="n">
-        <v>26.3831</v>
+        <v>-57.624</v>
       </c>
       <c r="T55" s="4" t="n">
-        <v>47.9326</v>
+        <v>-5.0728</v>
       </c>
       <c r="U55" s="4" t="n">
-        <v>-21.5495</v>
+        <v>-52.5512</v>
       </c>
       <c r="V55" s="4" t="inlineStr"/>
       <c r="W55" s="4" t="n">
-        <v>23.5</v>
+        <v>33.38</v>
       </c>
       <c r="X55" s="4" t="n">
-        <v>172514</v>
+        <v>251663</v>
       </c>
       <c r="Y55" s="4" t="n">
-        <v>338996</v>
+        <v>535409</v>
       </c>
       <c r="Z55" s="4" t="n">
-        <v>0.51</v>
+        <v>0.47</v>
       </c>
       <c r="AA55" s="4" t="n">
-        <v>140917</v>
+        <v>103393</v>
       </c>
       <c r="AB55" s="4" t="n">
-        <v>83.340355</v>
+        <v>18.989853</v>
       </c>
       <c r="AC55" s="4" t="n">
-        <v>58.388645</v>
+        <v>15.865028</v>
       </c>
       <c r="AD55" s="4" t="inlineStr"/>
       <c r="AE55" s="4" t="n">
-        <v>2.213</v>
+        <v>3.57</v>
       </c>
       <c r="AF55" s="4" t="n">
-        <v>14.8</v>
+        <v>34.9</v>
       </c>
       <c r="AG55" s="4" t="n">
-        <v>406.1</v>
+        <v>-17.2</v>
       </c>
       <c r="AH55" s="4" t="n">
-        <v>10.181711</v>
+        <v>4.7830014</v>
       </c>
       <c r="AI55" s="4" t="n">
-        <v>46</v>
+        <v>354</v>
       </c>
       <c r="AJ55" s="4" t="inlineStr"/>
       <c r="AK55" s="4" t="inlineStr">
         <is>
-          <t>https://www.screener.in/company/SIEMENS/</t>
+          <t>https://www.screener.in/company/HEROMOTOCO/</t>
         </is>
       </c>
       <c r="AL55" s="4" t="inlineStr">
         <is>
-          <t>https://www.tradingview.com/chart/?symbol=NSE:SIEMENS</t>
+          <t>https://www.tradingview.com/chart/?symbol=NSE:HEROMOTOCO</t>
         </is>
       </c>
     </row>
@@ -7828,13 +7826,13 @@
         <v>1.49</v>
       </c>
       <c r="AA56" s="2" t="n">
-        <v>157652</v>
+        <v>153014</v>
       </c>
       <c r="AB56" s="2" t="n">
-        <v>27.24978</v>
+        <v>26.448185</v>
       </c>
       <c r="AC56" s="2" t="n">
-        <v>18.800514</v>
+        <v>18.247467</v>
       </c>
       <c r="AD56" s="2" t="inlineStr"/>
       <c r="AE56" s="2" t="n">
@@ -7847,7 +7845,7 @@
         <v>43.7</v>
       </c>
       <c r="AH56" s="2" t="n">
-        <v>5.163689</v>
+        <v>5.011791</v>
       </c>
       <c r="AI56" s="2" t="n">
         <v>11</v>
@@ -7958,13 +7956,13 @@
         <v>0.43</v>
       </c>
       <c r="AA57" s="4" t="n">
-        <v>29987</v>
+        <v>27428</v>
       </c>
       <c r="AB57" s="4" t="n">
-        <v>110.2623</v>
+        <v>100.85246</v>
       </c>
       <c r="AC57" s="4" t="n">
-        <v>60.872673</v>
+        <v>55.67777</v>
       </c>
       <c r="AD57" s="4" t="inlineStr"/>
       <c r="AE57" s="4" t="n">
@@ -7977,7 +7975,7 @@
         <v>178.4</v>
       </c>
       <c r="AH57" s="4" t="n">
-        <v>39.608818</v>
+        <v>36.228584</v>
       </c>
       <c r="AI57" s="4" t="n">
         <v>6</v>
@@ -8088,13 +8086,13 @@
         <v>0.38</v>
       </c>
       <c r="AA58" s="2" t="n">
-        <v>43080</v>
+        <v>42593</v>
       </c>
       <c r="AB58" s="2" t="n">
-        <v>10.23521</v>
+        <v>10.119388</v>
       </c>
       <c r="AC58" s="2" t="n">
-        <v>10.125611</v>
+        <v>10.011028</v>
       </c>
       <c r="AD58" s="2" t="inlineStr"/>
       <c r="AE58" s="2" t="n">
@@ -8107,7 +8105,7 @@
         <v>35.1</v>
       </c>
       <c r="AH58" s="2" t="n">
-        <v>1.9327835</v>
+        <v>1.9109118</v>
       </c>
       <c r="AI58" s="2" t="n">
         <v>348</v>
@@ -8218,13 +8216,13 @@
         <v>1.53</v>
       </c>
       <c r="AA59" s="4" t="n">
-        <v>217877</v>
+        <v>212816</v>
       </c>
       <c r="AB59" s="4" t="n">
-        <v>13.315697</v>
+        <v>13.006376</v>
       </c>
       <c r="AC59" s="4" t="n">
-        <v>8.830985999999999</v>
+        <v>8.625845</v>
       </c>
       <c r="AD59" s="4" t="inlineStr"/>
       <c r="AE59" s="4" t="n">
@@ -8237,10 +8235,10 @@
         <v>75.09999999999999</v>
       </c>
       <c r="AH59" s="4" t="n">
-        <v>1.5951983</v>
+        <v>1.5581423</v>
       </c>
       <c r="AI59" s="4" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="AJ59" s="4" t="inlineStr"/>
       <c r="AK59" s="4" t="inlineStr">
@@ -8348,13 +8346,13 @@
         <v>0.75</v>
       </c>
       <c r="AA60" s="2" t="n">
-        <v>79356</v>
+        <v>77040</v>
       </c>
       <c r="AB60" s="2" t="n">
-        <v>28.087534</v>
+        <v>27.267904</v>
       </c>
       <c r="AC60" s="2" t="n">
-        <v>17.505682</v>
+        <v>16.994844</v>
       </c>
       <c r="AD60" s="2" t="inlineStr"/>
       <c r="AE60" s="2" t="inlineStr"/>
@@ -8365,7 +8363,7 @@
         <v>35.1</v>
       </c>
       <c r="AH60" s="2" t="n">
-        <v>3.9624155</v>
+        <v>3.8467872</v>
       </c>
       <c r="AI60" s="2" t="n">
         <v>9</v>
@@ -8476,13 +8474,13 @@
         <v>0.57</v>
       </c>
       <c r="AA61" s="4" t="n">
-        <v>159492</v>
+        <v>154830</v>
       </c>
       <c r="AB61" s="4" t="n">
-        <v>60.242214</v>
+        <v>58.481354</v>
       </c>
       <c r="AC61" s="4" t="n">
-        <v>49.3847</v>
+        <v>47.9412</v>
       </c>
       <c r="AD61" s="4" t="inlineStr"/>
       <c r="AE61" s="4" t="n">
@@ -8495,7 +8493,7 @@
         <v>29.6</v>
       </c>
       <c r="AH61" s="4" t="n">
-        <v>14.722215</v>
+        <v>14.291888</v>
       </c>
       <c r="AI61" s="4" t="n">
         <v>73</v>
@@ -8606,13 +8604,13 @@
         <v>0.72</v>
       </c>
       <c r="AA62" s="2" t="n">
-        <v>140540</v>
+        <v>135107</v>
       </c>
       <c r="AB62" s="2" t="n">
-        <v>59.521015</v>
+        <v>57.220005</v>
       </c>
       <c r="AC62" s="2" t="n">
-        <v>42.950027</v>
+        <v>41.28963</v>
       </c>
       <c r="AD62" s="2" t="inlineStr"/>
       <c r="AE62" s="2" t="n">
@@ -8625,10 +8623,10 @@
         <v>0.9</v>
       </c>
       <c r="AH62" s="2" t="n">
-        <v>16.58261</v>
+        <v>15.9415455</v>
       </c>
       <c r="AI62" s="2" t="n">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="AJ62" s="2" t="inlineStr"/>
       <c r="AK62" s="2" t="inlineStr">
@@ -8736,13 +8734,13 @@
         <v>0.45</v>
       </c>
       <c r="AA63" s="4" t="n">
-        <v>20941</v>
+        <v>19969</v>
       </c>
       <c r="AB63" s="4" t="n">
-        <v>32.42677</v>
+        <v>30.921719</v>
       </c>
       <c r="AC63" s="4" t="n">
-        <v>17.18282</v>
+        <v>16.3853</v>
       </c>
       <c r="AD63" s="4" t="inlineStr"/>
       <c r="AE63" s="4" t="n">
@@ -8755,7 +8753,7 @@
         <v>33.8</v>
       </c>
       <c r="AH63" s="4" t="n">
-        <v>30.700998</v>
+        <v>29.276049</v>
       </c>
       <c r="AI63" s="4" t="n">
         <v>31</v>
@@ -8866,13 +8864,13 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="AA64" s="2" t="n">
-        <v>86177</v>
+        <v>85576</v>
       </c>
       <c r="AB64" s="2" t="n">
-        <v>45.250206</v>
+        <v>44.934372</v>
       </c>
       <c r="AC64" s="2" t="n">
-        <v>31.187147</v>
+        <v>30.964218</v>
       </c>
       <c r="AD64" s="2" t="n">
         <v>25.2</v>
@@ -8887,7 +8885,7 @@
         <v>12.1</v>
       </c>
       <c r="AH64" s="2" t="n">
-        <v>10.250102</v>
+        <v>10.178559</v>
       </c>
       <c r="AI64" s="2" t="n">
         <v>65</v>
@@ -9000,13 +8998,13 @@
         <v>0.79</v>
       </c>
       <c r="AA65" s="4" t="n">
-        <v>28424</v>
+        <v>27400</v>
       </c>
       <c r="AB65" s="4" t="n">
-        <v>60.230293</v>
+        <v>58.06023</v>
       </c>
       <c r="AC65" s="4" t="n">
-        <v>45.702793</v>
+        <v>44.05615</v>
       </c>
       <c r="AD65" s="4" t="n">
         <v>23.91</v>
@@ -9021,7 +9019,7 @@
         <v>-19.9</v>
       </c>
       <c r="AH65" s="4" t="n">
-        <v>14.503728</v>
+        <v>13.981167</v>
       </c>
       <c r="AI65" s="4" t="n">
         <v>94</v>
@@ -9134,13 +9132,13 @@
         <v>0.95</v>
       </c>
       <c r="AA66" s="2" t="n">
-        <v>308784</v>
+        <v>300045</v>
       </c>
       <c r="AB66" s="2" t="n">
-        <v>12.483963</v>
+        <v>12.130662</v>
       </c>
       <c r="AC66" s="2" t="n">
-        <v>17.36253</v>
+        <v>16.871162</v>
       </c>
       <c r="AD66" s="2" t="inlineStr"/>
       <c r="AE66" s="2" t="n">
@@ -9153,7 +9151,7 @@
         <v>113</v>
       </c>
       <c r="AH66" s="2" t="n">
-        <v>3.086013</v>
+        <v>2.9986777</v>
       </c>
       <c r="AI66" s="2" t="n">
         <v>56</v>
@@ -9264,13 +9262,13 @@
         <v>0.47</v>
       </c>
       <c r="AA67" s="4" t="n">
-        <v>22489</v>
+        <v>22590</v>
       </c>
       <c r="AB67" s="4" t="n">
-        <v>18.62623</v>
+        <v>18.709848</v>
       </c>
       <c r="AC67" s="4" t="n">
-        <v>10.850162</v>
+        <v>10.898871</v>
       </c>
       <c r="AD67" s="4" t="n">
         <v>16.36</v>
@@ -9285,7 +9283,7 @@
         <v>715.2</v>
       </c>
       <c r="AH67" s="4" t="n">
-        <v>2.8665628</v>
+        <v>2.879432</v>
       </c>
       <c r="AI67" s="4" t="n">
         <v>0</v>
@@ -9519,14 +9517,12 @@
       <c r="Z69" s="4" t="n">
         <v>0.58</v>
       </c>
-      <c r="AA69" s="4" t="n">
-        <v>19293</v>
-      </c>
+      <c r="AA69" s="4" t="inlineStr"/>
       <c r="AB69" s="4" t="n">
-        <v>36.525703</v>
+        <v>35.039387</v>
       </c>
       <c r="AC69" s="4" t="n">
-        <v>27.95237</v>
+        <v>26.814922</v>
       </c>
       <c r="AD69" s="4" t="inlineStr"/>
       <c r="AE69" s="4" t="n">
@@ -9539,7 +9535,7 @@
         <v>-57.7</v>
       </c>
       <c r="AH69" s="4" t="n">
-        <v>5.2135115</v>
+        <v>5.0013614</v>
       </c>
       <c r="AI69" s="4" t="n">
         <v>23</v>
@@ -9650,13 +9646,13 @@
         <v>1.45</v>
       </c>
       <c r="AA70" s="2" t="n">
-        <v>81627</v>
+        <v>80137</v>
       </c>
       <c r="AB70" s="2" t="n">
-        <v>43.66848</v>
+        <v>42.871548</v>
       </c>
       <c r="AC70" s="2" t="n">
-        <v>47.731304</v>
+        <v>46.86023</v>
       </c>
       <c r="AD70" s="2" t="inlineStr"/>
       <c r="AE70" s="2" t="n">
@@ -9669,7 +9665,7 @@
         <v>154.6</v>
       </c>
       <c r="AH70" s="2" t="n">
-        <v>14.954469</v>
+        <v>14.681557</v>
       </c>
       <c r="AI70" s="2" t="n">
         <v>7</v>
@@ -9780,13 +9776,13 @@
         <v>1.06</v>
       </c>
       <c r="AA71" s="4" t="n">
-        <v>8797</v>
+        <v>8666</v>
       </c>
       <c r="AB71" s="4" t="n">
-        <v>50.0181</v>
+        <v>49.271492</v>
       </c>
       <c r="AC71" s="4" t="n">
-        <v>34.752262</v>
+        <v>34.23353</v>
       </c>
       <c r="AD71" s="4" t="inlineStr"/>
       <c r="AE71" s="4" t="n">
@@ -9799,7 +9795,7 @@
         <v>31.8</v>
       </c>
       <c r="AH71" s="4" t="n">
-        <v>15.024738</v>
+        <v>14.800468</v>
       </c>
       <c r="AI71" s="4" t="n">
         <v>297</v>
@@ -9910,13 +9906,13 @@
         <v>1.94</v>
       </c>
       <c r="AA72" s="2" t="n">
-        <v>76216</v>
+        <v>74525</v>
       </c>
       <c r="AB72" s="2" t="n">
-        <v>57.575047</v>
+        <v>56.53073</v>
       </c>
       <c r="AC72" s="2" t="n">
-        <v>12.375846</v>
+        <v>12.101305</v>
       </c>
       <c r="AD72" s="2" t="inlineStr"/>
       <c r="AE72" s="2" t="inlineStr"/>
@@ -9927,7 +9923,7 @@
         <v>71.7</v>
       </c>
       <c r="AH72" s="2" t="n">
-        <v>1.1587411</v>
+        <v>1.133036</v>
       </c>
       <c r="AI72" s="2" t="n">
         <v>15</v>
@@ -10038,13 +10034,13 @@
         <v>0.96</v>
       </c>
       <c r="AA73" s="4" t="n">
-        <v>99053</v>
+        <v>97320</v>
       </c>
       <c r="AB73" s="4" t="n">
-        <v>58.490566</v>
+        <v>57.467503</v>
       </c>
       <c r="AC73" s="4" t="n">
-        <v>46.156593</v>
+        <v>45.349266</v>
       </c>
       <c r="AD73" s="4" t="inlineStr"/>
       <c r="AE73" s="4" t="n">
@@ -10057,10 +10053,10 @@
         <v>11.2</v>
       </c>
       <c r="AH73" s="4" t="n">
-        <v>11.063614</v>
+        <v>10.8701</v>
       </c>
       <c r="AI73" s="4" t="n">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="AJ73" s="4" t="inlineStr"/>
       <c r="AK73" s="4" t="inlineStr">
@@ -10168,13 +10164,13 @@
         <v>1.09</v>
       </c>
       <c r="AA74" s="2" t="n">
-        <v>136517</v>
+        <v>139609</v>
       </c>
       <c r="AB74" s="2" t="n">
-        <v>26.665512</v>
+        <v>27.269424</v>
       </c>
       <c r="AC74" s="2" t="n">
-        <v>17.69093</v>
+        <v>18.091587</v>
       </c>
       <c r="AD74" s="2" t="inlineStr"/>
       <c r="AE74" s="2" t="n">
@@ -10187,7 +10183,7 @@
         <v>28.3</v>
       </c>
       <c r="AH74" s="2" t="n">
-        <v>4.6081433</v>
+        <v>4.7125072</v>
       </c>
       <c r="AI74" s="2" t="n">
         <v>331</v>
@@ -10298,13 +10294,13 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="AA75" s="4" t="n">
-        <v>38054</v>
+        <v>38369</v>
       </c>
       <c r="AB75" s="4" t="n">
-        <v>41.563786</v>
+        <v>41.907967</v>
       </c>
       <c r="AC75" s="4" t="n">
-        <v>30.310017</v>
+        <v>30.561008</v>
       </c>
       <c r="AD75" s="4" t="inlineStr"/>
       <c r="AE75" s="4" t="n">
@@ -10317,10 +10313,10 @@
         <v>21.5</v>
       </c>
       <c r="AH75" s="4" t="n">
-        <v>6.665187</v>
+        <v>6.72038</v>
       </c>
       <c r="AI75" s="4" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AJ75" s="4" t="inlineStr"/>
       <c r="AK75" s="4" t="inlineStr">
@@ -10428,13 +10424,13 @@
         <v>0.44</v>
       </c>
       <c r="AA76" s="2" t="n">
-        <v>58525</v>
+        <v>58416</v>
       </c>
       <c r="AB76" s="2" t="n">
-        <v>82.99639000000001</v>
+        <v>83.17435999999999</v>
       </c>
       <c r="AC76" s="2" t="n">
-        <v>54.789986</v>
+        <v>54.688385</v>
       </c>
       <c r="AD76" s="2" t="inlineStr"/>
       <c r="AE76" s="2" t="n">
@@ -10447,7 +10443,7 @@
         <v>62.1</v>
       </c>
       <c r="AH76" s="2" t="n">
-        <v>17.639553</v>
+        <v>17.606842</v>
       </c>
       <c r="AI76" s="2" t="n">
         <v>15</v>
@@ -10558,13 +10554,13 @@
         <v>0.54</v>
       </c>
       <c r="AA77" s="4" t="n">
-        <v>49802</v>
+        <v>47587</v>
       </c>
       <c r="AB77" s="4" t="n">
-        <v>43.904522</v>
+        <v>41.952263</v>
       </c>
       <c r="AC77" s="4" t="n">
-        <v>24.879227</v>
+        <v>23.772945</v>
       </c>
       <c r="AD77" s="4" t="inlineStr"/>
       <c r="AE77" s="4" t="n">
@@ -10577,10 +10573,10 @@
         <v>161.9</v>
       </c>
       <c r="AH77" s="4" t="n">
-        <v>14.914568</v>
+        <v>14.251376</v>
       </c>
       <c r="AI77" s="4" t="n">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AJ77" s="4" t="inlineStr"/>
       <c r="AK77" s="4" t="inlineStr">
@@ -10688,13 +10684,13 @@
         <v>0.35</v>
       </c>
       <c r="AA78" s="2" t="n">
-        <v>73936</v>
+        <v>71458</v>
       </c>
       <c r="AB78" s="2" t="n">
-        <v>17.294685</v>
+        <v>16.714975</v>
       </c>
       <c r="AC78" s="2" t="n">
-        <v>11.2849455</v>
+        <v>10.906679</v>
       </c>
       <c r="AD78" s="2" t="inlineStr"/>
       <c r="AE78" s="2" t="n">
@@ -10707,10 +10703,10 @@
         <v>121.1</v>
       </c>
       <c r="AH78" s="2" t="n">
-        <v>1.2260189</v>
+        <v>1.1849233</v>
       </c>
       <c r="AI78" s="2" t="n">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="AJ78" s="2" t="inlineStr"/>
       <c r="AK78" s="2" t="inlineStr">
@@ -10818,13 +10814,13 @@
         <v>0.95</v>
       </c>
       <c r="AA79" s="4" t="n">
-        <v>104111</v>
+        <v>102702</v>
       </c>
       <c r="AB79" s="4" t="n">
-        <v>55.241043</v>
+        <v>54.4938</v>
       </c>
       <c r="AC79" s="4" t="n">
-        <v>41.19163</v>
+        <v>40.634434</v>
       </c>
       <c r="AD79" s="4" t="inlineStr"/>
       <c r="AE79" s="4" t="n">
@@ -10837,7 +10833,7 @@
         <v>24.7</v>
       </c>
       <c r="AH79" s="4" t="n">
-        <v>24.732508</v>
+        <v>24.397953</v>
       </c>
       <c r="AI79" s="4" t="n">
         <v>50</v>
@@ -10948,13 +10944,13 @@
         <v>0.47</v>
       </c>
       <c r="AA80" s="2" t="n">
-        <v>1260</v>
+        <v>1196</v>
       </c>
       <c r="AB80" s="2" t="n">
-        <v>135.29411</v>
+        <v>128.41176</v>
       </c>
       <c r="AC80" s="2" t="n">
-        <v>29.67742</v>
+        <v>28.167742</v>
       </c>
       <c r="AD80" s="2" t="inlineStr"/>
       <c r="AE80" s="2" t="n">
@@ -10967,7 +10963,7 @@
         <v>87.09999999999999</v>
       </c>
       <c r="AH80" s="2" t="n">
-        <v>1.1871427</v>
+        <v>1.1267532</v>
       </c>
       <c r="AI80" s="2" t="n">
         <v>108</v>
@@ -11078,13 +11074,13 @@
         <v>0.66</v>
       </c>
       <c r="AA81" s="4" t="n">
-        <v>30904</v>
+        <v>29951</v>
       </c>
       <c r="AB81" s="4" t="n">
-        <v>20.122324</v>
+        <v>19.50153</v>
       </c>
       <c r="AC81" s="4" t="n">
-        <v>10.683004</v>
+        <v>10.353423</v>
       </c>
       <c r="AD81" s="4" t="inlineStr"/>
       <c r="AE81" s="4" t="n">
@@ -11097,7 +11093,7 @@
         <v>288.5</v>
       </c>
       <c r="AH81" s="4" t="n">
-        <v>1.9254066</v>
+        <v>1.8660058</v>
       </c>
       <c r="AI81" s="4" t="n">
         <v>122</v>
@@ -11208,13 +11204,13 @@
         <v>0.6</v>
       </c>
       <c r="AA82" s="2" t="n">
-        <v>10404</v>
+        <v>10405</v>
       </c>
       <c r="AB82" s="2" t="n">
-        <v>42.939884</v>
+        <v>42.944775</v>
       </c>
       <c r="AC82" s="2" t="n">
-        <v>23.92916</v>
+        <v>23.931885</v>
       </c>
       <c r="AD82" s="2" t="inlineStr"/>
       <c r="AE82" s="2" t="n">
@@ -11227,7 +11223,7 @@
         <v>101.5</v>
       </c>
       <c r="AH82" s="2" t="n">
-        <v>5.1725965</v>
+        <v>5.1731853</v>
       </c>
       <c r="AI82" s="2" t="n">
         <v>0</v>
@@ -11338,13 +11334,13 @@
         <v>0.42</v>
       </c>
       <c r="AA83" s="4" t="n">
-        <v>25756</v>
+        <v>24922</v>
       </c>
       <c r="AB83" s="4" t="n">
-        <v>76.06112</v>
+        <v>73.724495</v>
       </c>
       <c r="AC83" s="4" t="n">
-        <v>33.52816</v>
+        <v>32.442986</v>
       </c>
       <c r="AD83" s="4" t="inlineStr"/>
       <c r="AE83" s="4" t="n">
@@ -11357,7 +11353,7 @@
         <v>40.6</v>
       </c>
       <c r="AH83" s="4" t="n">
-        <v>14.126551</v>
+        <v>13.66933</v>
       </c>
       <c r="AI83" s="4" t="n">
         <v>37</v>
@@ -11464,11 +11460,11 @@
         <v>0.53</v>
       </c>
       <c r="AA84" s="2" t="n">
-        <v>7207</v>
+        <v>7155</v>
       </c>
       <c r="AB84" s="2" t="inlineStr"/>
       <c r="AC84" s="2" t="n">
-        <v>94.644104</v>
+        <v>93.96378</v>
       </c>
       <c r="AD84" s="2" t="inlineStr"/>
       <c r="AE84" s="2" t="n">
@@ -11479,7 +11475,7 @@
       </c>
       <c r="AG84" s="2" t="inlineStr"/>
       <c r="AH84" s="2" t="n">
-        <v>5.176454</v>
+        <v>5.139245</v>
       </c>
       <c r="AI84" s="2" t="n">
         <v>0</v>
@@ -11590,13 +11586,13 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="AA85" s="4" t="n">
-        <v>103939</v>
+        <v>103432</v>
       </c>
       <c r="AB85" s="4" t="n">
-        <v>47.614315</v>
+        <v>47.382374</v>
       </c>
       <c r="AC85" s="4" t="n">
-        <v>38.42579</v>
+        <v>38.23861</v>
       </c>
       <c r="AD85" s="4" t="inlineStr"/>
       <c r="AE85" s="4" t="n">
@@ -11609,7 +11605,7 @@
         <v>20.7</v>
       </c>
       <c r="AH85" s="4" t="n">
-        <v>7.8356743</v>
+        <v>7.797505</v>
       </c>
       <c r="AI85" s="4" t="n">
         <v>45</v>
@@ -11720,13 +11716,13 @@
         <v>0.27</v>
       </c>
       <c r="AA86" s="2" t="n">
-        <v>167912</v>
+        <v>164793</v>
       </c>
       <c r="AB86" s="2" t="n">
-        <v>56.50206</v>
+        <v>55.452675</v>
       </c>
       <c r="AC86" s="2" t="n">
-        <v>37.97552</v>
+        <v>37.27022</v>
       </c>
       <c r="AD86" s="2" t="inlineStr"/>
       <c r="AE86" s="2" t="n">
@@ -11739,7 +11735,7 @@
         <v>124.1</v>
       </c>
       <c r="AH86" s="2" t="n">
-        <v>6.486512</v>
+        <v>6.3660417</v>
       </c>
       <c r="AI86" s="2" t="n">
         <v>0</v>
@@ -11850,13 +11846,13 @@
         <v>1.3</v>
       </c>
       <c r="AA87" s="4" t="n">
-        <v>5772</v>
+        <v>5447</v>
       </c>
       <c r="AB87" s="4" t="n">
-        <v>59.36699</v>
+        <v>56.01356</v>
       </c>
       <c r="AC87" s="4" t="n">
-        <v>18.7795</v>
+        <v>17.718712</v>
       </c>
       <c r="AD87" s="4" t="inlineStr"/>
       <c r="AE87" s="4" t="n">
@@ -11869,7 +11865,7 @@
         <v>3.4</v>
       </c>
       <c r="AH87" s="4" t="n">
-        <v>2.6707983</v>
+        <v>2.5199344</v>
       </c>
       <c r="AI87" s="4" t="n">
         <v>0</v>
@@ -11980,13 +11976,13 @@
         <v>0.25</v>
       </c>
       <c r="AA88" s="2" t="n">
-        <v>30711</v>
+        <v>30685</v>
       </c>
       <c r="AB88" s="2" t="n">
-        <v>151.08267</v>
+        <v>150.95473</v>
       </c>
       <c r="AC88" s="2" t="n">
-        <v>45.157528</v>
+        <v>45.11928</v>
       </c>
       <c r="AD88" s="2" t="inlineStr"/>
       <c r="AE88" s="2" t="n">
@@ -11999,7 +11995,7 @@
         <v>-46.9</v>
       </c>
       <c r="AH88" s="2" t="n">
-        <v>13.665093</v>
+        <v>13.653521</v>
       </c>
       <c r="AI88" s="2" t="n">
         <v>0</v>
@@ -12110,13 +12106,13 @@
         <v>1.83</v>
       </c>
       <c r="AA89" s="4" t="n">
-        <v>67601</v>
+        <v>65584</v>
       </c>
       <c r="AB89" s="4" t="n">
-        <v>52.911533</v>
+        <v>51.332584</v>
       </c>
       <c r="AC89" s="4" t="n">
-        <v>37.85819</v>
+        <v>36.72845</v>
       </c>
       <c r="AD89" s="4" t="inlineStr"/>
       <c r="AE89" s="4" t="n">
@@ -12129,7 +12125,7 @@
         <v>23.3</v>
       </c>
       <c r="AH89" s="4" t="n">
-        <v>6.1502013</v>
+        <v>5.9666715</v>
       </c>
       <c r="AI89" s="4" t="n">
         <v>13</v>
@@ -12240,13 +12236,13 @@
         <v>0.67</v>
       </c>
       <c r="AA90" s="2" t="n">
-        <v>211053</v>
+        <v>206721</v>
       </c>
       <c r="AB90" s="2" t="n">
-        <v>123.43931</v>
+        <v>120.90559</v>
       </c>
       <c r="AC90" s="2" t="n">
-        <v>42.950077</v>
+        <v>42.06848</v>
       </c>
       <c r="AD90" s="2" t="inlineStr"/>
       <c r="AE90" s="2" t="n">
@@ -12259,7 +12255,7 @@
         <v>18.5</v>
       </c>
       <c r="AH90" s="2" t="n">
-        <v>10.940996</v>
+        <v>10.71642</v>
       </c>
       <c r="AI90" s="2" t="n">
         <v>0</v>
@@ -12370,13 +12366,13 @@
         <v>0.91</v>
       </c>
       <c r="AA91" s="4" t="n">
-        <v>266744</v>
+        <v>262636</v>
       </c>
       <c r="AB91" s="4" t="n">
-        <v>69.93428</v>
+        <v>68.85742999999999</v>
       </c>
       <c r="AC91" s="4" t="n">
-        <v>55.71974</v>
+        <v>54.86177</v>
       </c>
       <c r="AD91" s="4" t="inlineStr"/>
       <c r="AE91" s="4" t="n">
@@ -12389,7 +12385,7 @@
         <v>48.1</v>
       </c>
       <c r="AH91" s="4" t="n">
-        <v>51.725685</v>
+        <v>50.929214</v>
       </c>
       <c r="AI91" s="4" t="n">
         <v>87</v>
@@ -12500,13 +12496,13 @@
         <v>0.95</v>
       </c>
       <c r="AA92" s="2" t="n">
-        <v>441478</v>
+        <v>440278</v>
       </c>
       <c r="AB92" s="2" t="n">
-        <v>36.493458</v>
+        <v>36.39429</v>
       </c>
       <c r="AC92" s="2" t="n">
-        <v>28.512602</v>
+        <v>28.435123</v>
       </c>
       <c r="AD92" s="2" t="inlineStr"/>
       <c r="AE92" s="2" t="n">
@@ -12519,7 +12515,7 @@
         <v>27.4</v>
       </c>
       <c r="AH92" s="2" t="n">
-        <v>5.2827263</v>
+        <v>5.268371</v>
       </c>
       <c r="AI92" s="2" t="n">
         <v>87</v>
@@ -12626,13 +12622,13 @@
         <v>0.4</v>
       </c>
       <c r="AA93" s="4" t="n">
-        <v>3653</v>
+        <v>3501</v>
       </c>
       <c r="AB93" s="4" t="n">
-        <v>835</v>
+        <v>800.2841</v>
       </c>
       <c r="AC93" s="4" t="n">
-        <v>37.29949</v>
+        <v>35.74873</v>
       </c>
       <c r="AD93" s="4" t="inlineStr"/>
       <c r="AE93" s="4" t="n">
@@ -12643,7 +12639,7 @@
       </c>
       <c r="AG93" s="4" t="inlineStr"/>
       <c r="AH93" s="4" t="n">
-        <v>5.308328</v>
+        <v>5.0876293</v>
       </c>
       <c r="AI93" s="4" t="n">
         <v>0</v>
@@ -12754,13 +12750,13 @@
         <v>0.92</v>
       </c>
       <c r="AA94" s="2" t="n">
-        <v>540812</v>
+        <v>529805</v>
       </c>
       <c r="AB94" s="2" t="n">
-        <v>32.573963</v>
+        <v>31.910997</v>
       </c>
       <c r="AC94" s="2" t="n">
-        <v>21.852234</v>
+        <v>21.407484</v>
       </c>
       <c r="AD94" s="2" t="inlineStr"/>
       <c r="AE94" s="2" t="n">
@@ -12773,10 +12769,10 @@
         <v>14</v>
       </c>
       <c r="AH94" s="2" t="n">
-        <v>4.947575</v>
+        <v>4.846879</v>
       </c>
       <c r="AI94" s="2" t="n">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="AJ94" s="2" t="inlineStr"/>
       <c r="AK94" s="2" t="inlineStr">
@@ -13382,13 +13378,13 @@
         <v>9.32</v>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>3908</v>
+        <v>3659</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>20.465115</v>
+        <v>19.165115</v>
       </c>
       <c r="AC2" s="2" t="n">
-        <v>6.62152</v>
+        <v>6.2009034</v>
       </c>
       <c r="AD2" s="2" t="inlineStr"/>
       <c r="AE2" s="2" t="n">
@@ -13401,7 +13397,7 @@
         <v>17</v>
       </c>
       <c r="AH2" s="2" t="n">
-        <v>4.0618505</v>
+        <v>3.803831</v>
       </c>
       <c r="AI2" s="2" t="n">
         <v>62</v>
@@ -13512,13 +13508,13 @@
         <v>1.16</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>247470</v>
+        <v>244178</v>
       </c>
       <c r="AB3" s="4" t="n">
-        <v>84.74545000000001</v>
+        <v>83.61818</v>
       </c>
       <c r="AC3" s="4" t="n">
-        <v>61.95091</v>
+        <v>61.126846</v>
       </c>
       <c r="AD3" s="4" t="inlineStr"/>
       <c r="AE3" s="4" t="n">
@@ -13531,7 +13527,7 @@
         <v>65.7</v>
       </c>
       <c r="AH3" s="4" t="n">
-        <v>14.764624</v>
+        <v>14.568227</v>
       </c>
       <c r="AI3" s="4" t="n">
         <v>32</v>
@@ -13642,13 +13638,13 @@
         <v>0.95</v>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>63950</v>
+        <v>62596</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>34.010715</v>
+        <v>33.272877</v>
       </c>
       <c r="AC4" s="2" t="n">
-        <v>20.596039</v>
+        <v>20.149221</v>
       </c>
       <c r="AD4" s="2" t="inlineStr"/>
       <c r="AE4" s="2" t="inlineStr"/>
@@ -13659,7 +13655,7 @@
         <v>367.9</v>
       </c>
       <c r="AH4" s="2" t="n">
-        <v>1.5225495</v>
+        <v>1.4895188</v>
       </c>
       <c r="AI4" s="2" t="n">
         <v>33</v>
@@ -13770,13 +13766,13 @@
         <v>1.24</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>416807</v>
+        <v>407655</v>
       </c>
       <c r="AB5" s="4" t="n">
-        <v>20.529152</v>
+        <v>20.078392</v>
       </c>
       <c r="AC5" s="4" t="n">
-        <v>16.399218</v>
+        <v>16.039139</v>
       </c>
       <c r="AD5" s="4" t="inlineStr"/>
       <c r="AE5" s="4" t="inlineStr"/>
@@ -13787,7 +13783,7 @@
         <v>22.5</v>
       </c>
       <c r="AH5" s="4" t="n">
-        <v>2.299658</v>
+        <v>2.2491643</v>
       </c>
       <c r="AI5" s="4" t="n">
         <v>16</v>
@@ -13897,14 +13893,12 @@
       <c r="Z6" s="2" t="n">
         <v>0.73</v>
       </c>
-      <c r="AA6" s="2" t="n">
-        <v>83379</v>
-      </c>
+      <c r="AA6" s="2" t="inlineStr"/>
       <c r="AB6" s="2" t="n">
-        <v>54.050488</v>
+        <v>52.359344</v>
       </c>
       <c r="AC6" s="2" t="n">
-        <v>40.93824</v>
+        <v>39.65736</v>
       </c>
       <c r="AD6" s="2" t="inlineStr"/>
       <c r="AE6" s="2" t="n">
@@ -13917,7 +13911,7 @@
         <v>103.4</v>
       </c>
       <c r="AH6" s="2" t="n">
-        <v>19.813597</v>
+        <v>19.193666</v>
       </c>
       <c r="AI6" s="2" t="n">
         <v>24</v>
@@ -14028,13 +14022,13 @@
         <v>1.17</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>30741</v>
+        <v>29235</v>
       </c>
       <c r="AB7" s="4" t="n">
-        <v>9.787946</v>
+        <v>9.308593999999999</v>
       </c>
       <c r="AC7" s="4" t="n">
-        <v>3.425781</v>
+        <v>3.2580078</v>
       </c>
       <c r="AD7" s="4" t="inlineStr"/>
       <c r="AE7" s="4" t="n">
@@ -14045,10 +14039,10 @@
       </c>
       <c r="AG7" s="4" t="inlineStr"/>
       <c r="AH7" s="4" t="n">
-        <v>2.1573088</v>
+        <v>2.0516572</v>
       </c>
       <c r="AI7" s="4" t="n">
-        <v>221</v>
+        <v>227</v>
       </c>
       <c r="AJ7" s="4" t="inlineStr"/>
       <c r="AK7" s="4" t="inlineStr">
@@ -14160,13 +14154,13 @@
         <v>1.35</v>
       </c>
       <c r="AA8" s="2" t="n">
-        <v>47490</v>
+        <v>46455</v>
       </c>
       <c r="AB8" s="2" t="n">
-        <v>38.00562</v>
+        <v>37.176968</v>
       </c>
       <c r="AC8" s="2" t="n">
-        <v>32.17346</v>
+        <v>31.471966</v>
       </c>
       <c r="AD8" s="2" t="inlineStr"/>
       <c r="AE8" s="2" t="n">
@@ -14179,7 +14173,7 @@
         <v>269</v>
       </c>
       <c r="AH8" s="2" t="n">
-        <v>7.843115</v>
+        <v>7.672108</v>
       </c>
       <c r="AI8" s="2" t="n">
         <v>99</v>
@@ -14290,13 +14284,13 @@
         <v>0.83</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>328034</v>
+        <v>313990</v>
       </c>
       <c r="AB9" s="4" t="n">
-        <v>35.211773</v>
+        <v>33.704235</v>
       </c>
       <c r="AC9" s="4" t="n">
-        <v>28.519903</v>
+        <v>27.298868</v>
       </c>
       <c r="AD9" s="4" t="inlineStr"/>
       <c r="AE9" s="4" t="n">
@@ -14309,10 +14303,10 @@
         <v>14.9</v>
       </c>
       <c r="AH9" s="4" t="n">
-        <v>7.992817</v>
+        <v>7.6506166</v>
       </c>
       <c r="AI9" s="4" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="AJ9" s="4" t="inlineStr"/>
       <c r="AK9" s="4" t="inlineStr">
@@ -14671,13 +14665,13 @@
         <v>9.32</v>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>3908</v>
+        <v>3659</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>20.465115</v>
+        <v>19.165115</v>
       </c>
       <c r="AC2" s="2" t="n">
-        <v>6.62152</v>
+        <v>6.2009034</v>
       </c>
       <c r="AD2" s="2" t="inlineStr"/>
       <c r="AE2" s="2" t="n">
@@ -14690,7 +14684,7 @@
         <v>17</v>
       </c>
       <c r="AH2" s="2" t="n">
-        <v>4.0618505</v>
+        <v>3.803831</v>
       </c>
       <c r="AI2" s="2" t="n">
         <v>62</v>
@@ -14801,13 +14795,13 @@
         <v>1.16</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>247470</v>
+        <v>244178</v>
       </c>
       <c r="AB3" s="4" t="n">
-        <v>84.74545000000001</v>
+        <v>83.61818</v>
       </c>
       <c r="AC3" s="4" t="n">
-        <v>61.95091</v>
+        <v>61.126846</v>
       </c>
       <c r="AD3" s="4" t="inlineStr"/>
       <c r="AE3" s="4" t="n">
@@ -14820,7 +14814,7 @@
         <v>65.7</v>
       </c>
       <c r="AH3" s="4" t="n">
-        <v>14.764624</v>
+        <v>14.568227</v>
       </c>
       <c r="AI3" s="4" t="n">
         <v>32</v>
@@ -14931,13 +14925,13 @@
         <v>0.95</v>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>63950</v>
+        <v>62596</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>34.010715</v>
+        <v>33.272877</v>
       </c>
       <c r="AC4" s="2" t="n">
-        <v>20.596039</v>
+        <v>20.149221</v>
       </c>
       <c r="AD4" s="2" t="inlineStr"/>
       <c r="AE4" s="2" t="inlineStr"/>
@@ -14948,7 +14942,7 @@
         <v>367.9</v>
       </c>
       <c r="AH4" s="2" t="n">
-        <v>1.5225495</v>
+        <v>1.4895188</v>
       </c>
       <c r="AI4" s="2" t="n">
         <v>33</v>
@@ -15059,13 +15053,13 @@
         <v>1.24</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>416807</v>
+        <v>407655</v>
       </c>
       <c r="AB5" s="4" t="n">
-        <v>20.529152</v>
+        <v>20.078392</v>
       </c>
       <c r="AC5" s="4" t="n">
-        <v>16.399218</v>
+        <v>16.039139</v>
       </c>
       <c r="AD5" s="4" t="inlineStr"/>
       <c r="AE5" s="4" t="inlineStr"/>
@@ -15076,7 +15070,7 @@
         <v>22.5</v>
       </c>
       <c r="AH5" s="4" t="n">
-        <v>2.299658</v>
+        <v>2.2491643</v>
       </c>
       <c r="AI5" s="4" t="n">
         <v>16</v>
@@ -15186,14 +15180,12 @@
       <c r="Z6" s="2" t="n">
         <v>0.73</v>
       </c>
-      <c r="AA6" s="2" t="n">
-        <v>83379</v>
-      </c>
+      <c r="AA6" s="2" t="inlineStr"/>
       <c r="AB6" s="2" t="n">
-        <v>54.050488</v>
+        <v>52.359344</v>
       </c>
       <c r="AC6" s="2" t="n">
-        <v>40.93824</v>
+        <v>39.65736</v>
       </c>
       <c r="AD6" s="2" t="inlineStr"/>
       <c r="AE6" s="2" t="n">
@@ -15206,7 +15198,7 @@
         <v>103.4</v>
       </c>
       <c r="AH6" s="2" t="n">
-        <v>19.813597</v>
+        <v>19.193666</v>
       </c>
       <c r="AI6" s="2" t="n">
         <v>24</v>
@@ -15317,13 +15309,13 @@
         <v>1.17</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>30741</v>
+        <v>29235</v>
       </c>
       <c r="AB7" s="4" t="n">
-        <v>9.787946</v>
+        <v>9.308593999999999</v>
       </c>
       <c r="AC7" s="4" t="n">
-        <v>3.425781</v>
+        <v>3.2580078</v>
       </c>
       <c r="AD7" s="4" t="inlineStr"/>
       <c r="AE7" s="4" t="n">
@@ -15334,10 +15326,10 @@
       </c>
       <c r="AG7" s="4" t="inlineStr"/>
       <c r="AH7" s="4" t="n">
-        <v>2.1573088</v>
+        <v>2.0516572</v>
       </c>
       <c r="AI7" s="4" t="n">
-        <v>221</v>
+        <v>227</v>
       </c>
       <c r="AJ7" s="4" t="inlineStr"/>
       <c r="AK7" s="4" t="inlineStr">
@@ -15449,13 +15441,13 @@
         <v>1.35</v>
       </c>
       <c r="AA8" s="2" t="n">
-        <v>47490</v>
+        <v>46455</v>
       </c>
       <c r="AB8" s="2" t="n">
-        <v>38.00562</v>
+        <v>37.176968</v>
       </c>
       <c r="AC8" s="2" t="n">
-        <v>32.17346</v>
+        <v>31.471966</v>
       </c>
       <c r="AD8" s="2" t="inlineStr"/>
       <c r="AE8" s="2" t="n">
@@ -15468,7 +15460,7 @@
         <v>269</v>
       </c>
       <c r="AH8" s="2" t="n">
-        <v>7.843115</v>
+        <v>7.672108</v>
       </c>
       <c r="AI8" s="2" t="n">
         <v>99</v>
@@ -15579,13 +15571,13 @@
         <v>0.83</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>328034</v>
+        <v>313990</v>
       </c>
       <c r="AB9" s="4" t="n">
-        <v>35.211773</v>
+        <v>33.704235</v>
       </c>
       <c r="AC9" s="4" t="n">
-        <v>28.519903</v>
+        <v>27.298868</v>
       </c>
       <c r="AD9" s="4" t="inlineStr"/>
       <c r="AE9" s="4" t="n">
@@ -15598,10 +15590,10 @@
         <v>14.9</v>
       </c>
       <c r="AH9" s="4" t="n">
-        <v>7.992817</v>
+        <v>7.6506166</v>
       </c>
       <c r="AI9" s="4" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="AJ9" s="4" t="inlineStr"/>
       <c r="AK9" s="4" t="inlineStr">
@@ -15641,7 +15633,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Run Date: 14-Sep-2026 15:28 IST</t>
+          <t>Run Date: 15-Sep-2026 14:04 IST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
@@ -15745,7 +15737,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>44.2</v>
+        <v>44.3</v>
       </c>
     </row>
     <row r="14">

</xml_diff>

<commit_message>
📈 Daily Screener Report — 05-Oct-2026 23:07 IST
</commit_message>
<xml_diff>
--- a/output/swing_screener_report.xlsx
+++ b/output/swing_screener_report.xlsx
@@ -517,7 +517,7 @@
     <col width="16" customWidth="1" min="25" max="25"/>
     <col width="14" customWidth="1" min="26" max="26"/>
     <col width="17" customWidth="1" min="27" max="27"/>
-    <col width="12" customWidth="1" min="28" max="28"/>
+    <col width="11" customWidth="1" min="28" max="28"/>
     <col width="13" customWidth="1" min="29" max="29"/>
     <col width="8" customWidth="1" min="30" max="30"/>
     <col width="13" customWidth="1" min="31" max="31"/>
@@ -775,7 +775,7 @@
         <v>406.67</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>399.74</v>
+        <v>399.9</v>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
@@ -816,13 +816,13 @@
         <v>4.73</v>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>416170</v>
+        <v>413832</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>20.487268</v>
+        <v>20.392157</v>
       </c>
       <c r="AC2" s="2" t="n">
-        <v>17.80935</v>
+        <v>17.709309</v>
       </c>
       <c r="AD2" s="2" t="inlineStr"/>
       <c r="AE2" s="2" t="inlineStr"/>
@@ -833,7 +833,7 @@
         <v>22.5</v>
       </c>
       <c r="AH2" s="2" t="n">
-        <v>2.2960906</v>
+        <v>2.2831926</v>
       </c>
       <c r="AI2" s="2" t="n">
         <v>16</v>
@@ -903,7 +903,7 @@
         <v>197.46</v>
       </c>
       <c r="N3" s="4" t="n">
-        <v>159.68</v>
+        <v>159.85</v>
       </c>
       <c r="O3" s="4" t="inlineStr">
         <is>
@@ -944,13 +944,13 @@
         <v>4.27</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>22501</v>
+        <v>21679</v>
       </c>
       <c r="AB3" s="4" t="n">
-        <v>78.10457599999999</v>
+        <v>79.40345000000001</v>
       </c>
       <c r="AC3" s="4" t="n">
-        <v>25.921907</v>
+        <v>24.975054</v>
       </c>
       <c r="AD3" s="4" t="inlineStr"/>
       <c r="AE3" s="4" t="n">
@@ -963,7 +963,7 @@
         <v>83.7</v>
       </c>
       <c r="AH3" s="4" t="n">
-        <v>4.6616864</v>
+        <v>4.491408</v>
       </c>
       <c r="AI3" s="4" t="n">
         <v>4</v>
@@ -1033,7 +1033,7 @@
         <v>218.67</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>163.47</v>
+        <v>163.55</v>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
@@ -1078,13 +1078,13 @@
         <v>3.43</v>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>36477</v>
+        <v>38298</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>62.07552</v>
+        <v>65.17448400000001</v>
       </c>
       <c r="AC4" s="2" t="n">
-        <v>45.840385</v>
+        <v>48.12885</v>
       </c>
       <c r="AD4" s="2" t="inlineStr"/>
       <c r="AE4" s="2" t="n">
@@ -1095,7 +1095,7 @@
       </c>
       <c r="AG4" s="2" t="inlineStr"/>
       <c r="AH4" s="2" t="n">
-        <v>7.1899977</v>
+        <v>7.5489397</v>
       </c>
       <c r="AI4" s="2" t="n">
         <v>8</v>
@@ -1210,13 +1210,13 @@
         <v>1.53</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>3797</v>
+        <v>3853</v>
       </c>
       <c r="AB5" s="4" t="n">
-        <v>38.48101</v>
+        <v>38.994946</v>
       </c>
       <c r="AC5" s="4" t="n">
-        <v>18.164751</v>
+        <v>18.43065</v>
       </c>
       <c r="AD5" s="4" t="inlineStr"/>
       <c r="AE5" s="4" t="n">
@@ -1229,7 +1229,7 @@
         <v>32</v>
       </c>
       <c r="AH5" s="4" t="n">
-        <v>4.2089524</v>
+        <v>4.270564</v>
       </c>
       <c r="AI5" s="4" t="n">
         <v>16</v>
@@ -1299,7 +1299,7 @@
         <v>417.57</v>
       </c>
       <c r="N6" s="2" t="n">
-        <v>414.55</v>
+        <v>414.64</v>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
@@ -1340,13 +1340,13 @@
         <v>1.01</v>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>259081</v>
+        <v>261978</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>8.31981</v>
+        <v>8.396208</v>
       </c>
       <c r="AC6" s="2" t="n">
-        <v>7.418175</v>
+        <v>7.501109</v>
       </c>
       <c r="AD6" s="2" t="inlineStr"/>
       <c r="AE6" s="2" t="n">
@@ -1359,7 +1359,7 @@
         <v>1.2</v>
       </c>
       <c r="AH6" s="2" t="n">
-        <v>2.1750827</v>
+        <v>2.1994</v>
       </c>
       <c r="AI6" s="2" t="n">
         <v>500</v>
@@ -1429,7 +1429,7 @@
         <v>8812.860000000001</v>
       </c>
       <c r="N7" s="4" t="n">
-        <v>7434.25</v>
+        <v>7438.03</v>
       </c>
       <c r="O7" s="4" t="inlineStr">
         <is>
@@ -1470,13 +1470,13 @@
         <v>1.18</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>245532</v>
+        <v>244125</v>
       </c>
       <c r="AB7" s="4" t="n">
-        <v>83.82273000000001</v>
+        <v>83.440704</v>
       </c>
       <c r="AC7" s="4" t="n">
-        <v>61.465775</v>
+        <v>60.902584</v>
       </c>
       <c r="AD7" s="4" t="inlineStr"/>
       <c r="AE7" s="4" t="n">
@@ -1489,7 +1489,7 @@
         <v>65.7</v>
       </c>
       <c r="AH7" s="4" t="n">
-        <v>14.649003</v>
+        <v>14.565059</v>
       </c>
       <c r="AI7" s="4" t="n">
         <v>32</v>
@@ -1559,7 +1559,7 @@
         <v>85.43000000000001</v>
       </c>
       <c r="N8" s="2" t="n">
-        <v>64.48</v>
+        <v>64.44</v>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
@@ -1600,13 +1600,13 @@
         <v>0.51</v>
       </c>
       <c r="AA8" s="2" t="n">
-        <v>4695</v>
+        <v>4613</v>
       </c>
       <c r="AB8" s="2" t="n">
-        <v>24.590696</v>
+        <v>24.160463</v>
       </c>
       <c r="AC8" s="2" t="n">
-        <v>7.956358</v>
+        <v>7.817156</v>
       </c>
       <c r="AD8" s="2" t="inlineStr"/>
       <c r="AE8" s="2" t="n">
@@ -1619,7 +1619,7 @@
         <v>18.5</v>
       </c>
       <c r="AH8" s="2" t="n">
-        <v>4.880683</v>
+        <v>4.795292</v>
       </c>
       <c r="AI8" s="2" t="n">
         <v>28</v>
@@ -1689,7 +1689,7 @@
         <v>1544.15</v>
       </c>
       <c r="N9" s="4" t="n">
-        <v>1211.83</v>
+        <v>1213</v>
       </c>
       <c r="O9" s="4" t="inlineStr">
         <is>
@@ -1730,13 +1730,13 @@
         <v>0.63</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>33131</v>
+        <v>32754</v>
       </c>
       <c r="AB9" s="4" t="n">
-        <v>89.39709000000001</v>
+        <v>88.42434</v>
       </c>
       <c r="AC9" s="4" t="n">
-        <v>55.04849</v>
+        <v>54.421196</v>
       </c>
       <c r="AD9" s="4" t="inlineStr"/>
       <c r="AE9" s="4" t="n">
@@ -1749,7 +1749,7 @@
         <v>86</v>
       </c>
       <c r="AH9" s="4" t="n">
-        <v>11.495559</v>
+        <v>11.364563</v>
       </c>
       <c r="AI9" s="4" t="n">
         <v>9</v>
@@ -1819,7 +1819,7 @@
         <v>1773.21</v>
       </c>
       <c r="N10" s="2" t="n">
-        <v>1605.89</v>
+        <v>1607.86</v>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
@@ -1860,13 +1860,13 @@
         <v>1.42</v>
       </c>
       <c r="AA10" s="2" t="n">
-        <v>80899</v>
+        <v>82051</v>
       </c>
       <c r="AB10" s="2" t="n">
-        <v>35.839058</v>
+        <v>37.9275</v>
       </c>
       <c r="AC10" s="2" t="n">
-        <v>25.635433</v>
+        <v>25.904682</v>
       </c>
       <c r="AD10" s="2" t="inlineStr"/>
       <c r="AE10" s="2" t="n">
@@ -1879,7 +1879,7 @@
         <v>30.9</v>
       </c>
       <c r="AH10" s="2" t="n">
-        <v>6.430415</v>
+        <v>6.521976</v>
       </c>
       <c r="AI10" s="2" t="n">
         <v>88</v>
@@ -1949,7 +1949,7 @@
         <v>1306.15</v>
       </c>
       <c r="N11" s="4" t="n">
-        <v>1032.94</v>
+        <v>1031.11</v>
       </c>
       <c r="O11" s="4" t="inlineStr">
         <is>
@@ -1990,13 +1990,13 @@
         <v>1.14</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>49196</v>
+        <v>47718</v>
       </c>
       <c r="AB11" s="4" t="n">
-        <v>39.3266</v>
+        <v>38.13464</v>
       </c>
       <c r="AC11" s="4" t="n">
-        <v>33.329132</v>
+        <v>32.328022</v>
       </c>
       <c r="AD11" s="4" t="inlineStr"/>
       <c r="AE11" s="4" t="n">
@@ -2009,7 +2009,7 @@
         <v>269</v>
       </c>
       <c r="AH11" s="4" t="n">
-        <v>8.124841</v>
+        <v>7.880794</v>
       </c>
       <c r="AI11" s="4" t="n">
         <v>96</v>
@@ -2079,7 +2079,7 @@
         <v>554.54</v>
       </c>
       <c r="N12" s="2" t="n">
-        <v>533.5599999999999</v>
+        <v>532.96</v>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
@@ -2120,13 +2120,13 @@
         <v>0.23</v>
       </c>
       <c r="AA12" s="2" t="n">
-        <v>9080</v>
+        <v>9172</v>
       </c>
       <c r="AB12" s="2" t="n">
-        <v>291.04477</v>
+        <v>289.6814</v>
       </c>
       <c r="AC12" s="2" t="n">
-        <v>113.65712</v>
+        <v>111.54862</v>
       </c>
       <c r="AD12" s="2" t="inlineStr"/>
       <c r="AE12" s="2" t="n">
@@ -2139,7 +2139,7 @@
         <v>-50</v>
       </c>
       <c r="AH12" s="2" t="n">
-        <v>14.961253</v>
+        <v>15.113424</v>
       </c>
       <c r="AI12" s="2" t="n">
         <v>14</v>
@@ -2209,7 +2209,7 @@
         <v>1921.83</v>
       </c>
       <c r="N13" s="4" t="n">
-        <v>1823.77</v>
+        <v>1826.94</v>
       </c>
       <c r="O13" s="4" t="inlineStr">
         <is>
@@ -2250,13 +2250,13 @@
         <v>1.46</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>69032</v>
+        <v>69211</v>
       </c>
       <c r="AB13" s="4" t="n">
-        <v>53.94075</v>
+        <v>53.89972</v>
       </c>
       <c r="AC13" s="4" t="n">
-        <v>38.688435</v>
+        <v>38.788662</v>
       </c>
       <c r="AD13" s="4" t="inlineStr"/>
       <c r="AE13" s="4" t="n">
@@ -2269,7 +2269,7 @@
         <v>23.3</v>
       </c>
       <c r="AH13" s="4" t="n">
-        <v>6.2803645</v>
+        <v>6.2966347</v>
       </c>
       <c r="AI13" s="4" t="n">
         <v>13</v>
@@ -2339,7 +2339,7 @@
         <v>3145.56</v>
       </c>
       <c r="N14" s="2" t="n">
-        <v>2756.57</v>
+        <v>2756.24</v>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
@@ -2379,14 +2379,12 @@
       <c r="Z14" s="2" t="n">
         <v>1.09</v>
       </c>
-      <c r="AA14" s="2" t="n">
-        <v>81546</v>
-      </c>
+      <c r="AA14" s="2" t="inlineStr"/>
       <c r="AB14" s="2" t="n">
-        <v>52.906208</v>
+        <v>66.45154599999999</v>
       </c>
       <c r="AC14" s="2" t="n">
-        <v>39.583183</v>
+        <v>39.307682</v>
       </c>
       <c r="AD14" s="2" t="inlineStr"/>
       <c r="AE14" s="2" t="n">
@@ -2399,7 +2397,7 @@
         <v>103.4</v>
       </c>
       <c r="AH14" s="2" t="n">
-        <v>19.378134</v>
+        <v>19.24326</v>
       </c>
       <c r="AI14" s="2" t="n">
         <v>25</v>
@@ -2469,7 +2467,7 @@
         <v>857.49</v>
       </c>
       <c r="N15" s="4" t="n">
-        <v>631.58</v>
+        <v>631.72</v>
       </c>
       <c r="O15" s="4" t="inlineStr">
         <is>
@@ -2510,13 +2508,13 @@
         <v>0.2</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>7953</v>
+        <v>8656</v>
       </c>
       <c r="AB15" s="4" t="n">
-        <v>184.98451</v>
+        <v>184.23512</v>
       </c>
       <c r="AC15" s="4" t="n">
-        <v>70.71006</v>
+        <v>76.96449</v>
       </c>
       <c r="AD15" s="4" t="inlineStr"/>
       <c r="AE15" s="4" t="n">
@@ -2529,7 +2527,7 @@
         <v>-99.59999999999999</v>
       </c>
       <c r="AH15" s="4" t="n">
-        <v>2.7963943</v>
+        <v>3.0437407</v>
       </c>
       <c r="AI15" s="4" t="n">
         <v>0</v>
@@ -2599,7 +2597,7 @@
         <v>336.95</v>
       </c>
       <c r="N16" s="2" t="n">
-        <v>305.07</v>
+        <v>305.04</v>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
@@ -2640,13 +2638,13 @@
         <v>2.01</v>
       </c>
       <c r="AA16" s="2" t="n">
-        <v>78604</v>
+        <v>80865</v>
       </c>
       <c r="AB16" s="2" t="n">
-        <v>17.034262</v>
+        <v>17.514713</v>
       </c>
       <c r="AC16" s="2" t="n">
-        <v>12.975972</v>
+        <v>11.623477</v>
       </c>
       <c r="AD16" s="2" t="inlineStr"/>
       <c r="AE16" s="2" t="inlineStr"/>
@@ -2657,7 +2655,7 @@
         <v>32.7</v>
       </c>
       <c r="AH16" s="2" t="n">
-        <v>1.9588168</v>
+        <v>2.0151436</v>
       </c>
       <c r="AI16" s="2" t="n">
         <v>38</v>
@@ -2727,7 +2725,7 @@
         <v>395.51</v>
       </c>
       <c r="N17" s="4" t="n">
-        <v>351.92</v>
+        <v>352.24</v>
       </c>
       <c r="O17" s="4" t="inlineStr">
         <is>
@@ -2768,13 +2766,13 @@
         <v>1.49</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>63835</v>
+        <v>64634</v>
       </c>
       <c r="AB17" s="4" t="n">
-        <v>34</v>
+        <v>30.316593</v>
       </c>
       <c r="AC17" s="4" t="n">
-        <v>20.045412</v>
+        <v>20.244125</v>
       </c>
       <c r="AD17" s="4" t="inlineStr"/>
       <c r="AE17" s="4" t="inlineStr"/>
@@ -2785,7 +2783,7 @@
         <v>-11.7</v>
       </c>
       <c r="AH17" s="4" t="n">
-        <v>1.5183053</v>
+        <v>1.5373118</v>
       </c>
       <c r="AI17" s="4" t="n">
         <v>24</v>
@@ -2855,7 +2853,7 @@
         <v>417.62</v>
       </c>
       <c r="N18" s="2" t="n">
-        <v>362.05</v>
+        <v>361.62</v>
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
@@ -2896,13 +2894,13 @@
         <v>2</v>
       </c>
       <c r="AA18" s="2" t="n">
-        <v>146595</v>
+        <v>149381</v>
       </c>
       <c r="AB18" s="2" t="n">
-        <v>60.315186</v>
+        <v>61.373394</v>
       </c>
       <c r="AC18" s="2" t="n">
-        <v>30.107279</v>
+        <v>30.679388</v>
       </c>
       <c r="AD18" s="2" t="inlineStr"/>
       <c r="AE18" s="2" t="n">
@@ -2913,7 +2911,7 @@
       </c>
       <c r="AG18" s="2" t="inlineStr"/>
       <c r="AH18" s="2" t="n">
-        <v>5.6066804</v>
+        <v>5.7132206</v>
       </c>
       <c r="AI18" s="2" t="n">
         <v>33</v>
@@ -2983,7 +2981,7 @@
         <v>2366.94</v>
       </c>
       <c r="N19" s="4" t="n">
-        <v>2230.61</v>
+        <v>2227.34</v>
       </c>
       <c r="O19" s="4" t="inlineStr">
         <is>
@@ -3024,13 +3022,13 @@
         <v>1.76</v>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>65787</v>
+        <v>64771</v>
       </c>
       <c r="AB19" s="4" t="n">
-        <v>36.627907</v>
+        <v>36.033916</v>
       </c>
       <c r="AC19" s="4" t="n">
-        <v>23.86682</v>
+        <v>23.585155</v>
       </c>
       <c r="AD19" s="4" t="inlineStr"/>
       <c r="AE19" s="4" t="n">
@@ -3043,10 +3041,10 @@
         <v>930.7</v>
       </c>
       <c r="AH19" s="4" t="n">
-        <v>6.258138</v>
+        <v>6.161487</v>
       </c>
       <c r="AI19" s="4" t="n">
-        <v>32</v>
+        <v>21</v>
       </c>
       <c r="AJ19" s="4" t="inlineStr"/>
       <c r="AK19" s="4" t="inlineStr">
@@ -3113,7 +3111,7 @@
         <v>4751.56</v>
       </c>
       <c r="N20" s="2" t="n">
-        <v>4530.51</v>
+        <v>4529.9</v>
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
@@ -3154,13 +3152,13 @@
         <v>0.87</v>
       </c>
       <c r="AA20" s="2" t="n">
-        <v>307703</v>
+        <v>312987</v>
       </c>
       <c r="AB20" s="2" t="n">
-        <v>33.003372</v>
+        <v>33.57727</v>
       </c>
       <c r="AC20" s="2" t="n">
-        <v>26.64076</v>
+        <v>27.095772</v>
       </c>
       <c r="AD20" s="2" t="inlineStr"/>
       <c r="AE20" s="2" t="n">
@@ -3173,7 +3171,7 @@
         <v>14.9</v>
       </c>
       <c r="AH20" s="2" t="n">
-        <v>7.4974413</v>
+        <v>7.626174</v>
       </c>
       <c r="AI20" s="2" t="n">
         <v>43</v>
@@ -3243,7 +3241,7 @@
         <v>657.1</v>
       </c>
       <c r="N21" s="4" t="n">
-        <v>646.17</v>
+        <v>646.83</v>
       </c>
       <c r="O21" s="4" t="inlineStr">
         <is>
@@ -3284,13 +3282,13 @@
         <v>1.57</v>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>162975</v>
+        <v>166588</v>
       </c>
       <c r="AB21" s="4" t="n">
-        <v>36.72058</v>
+        <v>37.472164</v>
       </c>
       <c r="AC21" s="4" t="n">
-        <v>25.900347</v>
+        <v>26.474686</v>
       </c>
       <c r="AD21" s="4" t="n">
         <v>10.1</v>
@@ -3305,7 +3303,7 @@
         <v>4.2</v>
       </c>
       <c r="AH21" s="4" t="n">
-        <v>3.5839486</v>
+        <v>3.6634226</v>
       </c>
       <c r="AI21" s="4" t="n">
         <v>122</v>
@@ -3375,7 +3373,7 @@
         <v>2146.58</v>
       </c>
       <c r="N22" s="2" t="n">
-        <v>1608.24</v>
+        <v>1607.31</v>
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
@@ -3416,13 +3414,13 @@
         <v>0.44</v>
       </c>
       <c r="AA22" s="2" t="n">
-        <v>15196</v>
+        <v>15091</v>
       </c>
       <c r="AB22" s="2" t="n">
-        <v>114.51613</v>
+        <v>113.21124</v>
       </c>
       <c r="AC22" s="2" t="n">
-        <v>62.062138</v>
+        <v>61.633278</v>
       </c>
       <c r="AD22" s="2" t="inlineStr"/>
       <c r="AE22" s="2" t="n">
@@ -3435,7 +3433,7 @@
         <v>145.3</v>
       </c>
       <c r="AH22" s="2" t="n">
-        <v>21.030416</v>
+        <v>20.885094</v>
       </c>
       <c r="AI22" s="2" t="n">
         <v>0</v>
@@ -3455,32 +3453,32 @@
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>OFSS</t>
+          <t>BEML</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>Oracle Financial Services Software Limited</t>
+          <t>BEML Limited</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>Software - Infrastructure</t>
+          <t>Conglomerates</t>
         </is>
       </c>
       <c r="E23" s="6" t="n">
-        <v>42.6</v>
+        <v>42.8</v>
       </c>
       <c r="F23" s="4" t="n">
-        <v>3.6</v>
+        <v>21.6</v>
       </c>
       <c r="G23" s="4" t="n">
-        <v>39</v>
+        <v>21.2</v>
       </c>
       <c r="H23" s="6" t="inlineStr">
         <is>
@@ -3489,27 +3487,27 @@
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>📉 Tight Base | 💎 High ROE | 👤 High Promoter</t>
+          <t>📈 EMA Bull Stack | 📉 Tight Base</t>
         </is>
       </c>
       <c r="J23" s="4" t="n">
-        <v>10420</v>
+        <v>1962.3</v>
       </c>
       <c r="K23" s="4" t="n">
-        <v>-1.98</v>
+        <v>-1.51</v>
       </c>
       <c r="L23" s="4" t="n">
-        <v>11142.27</v>
+        <v>2008.6</v>
       </c>
       <c r="M23" s="4" t="n">
-        <v>11270.24</v>
+        <v>1950.92</v>
       </c>
       <c r="N23" s="4" t="n">
-        <v>9889.139999999999</v>
+        <v>1856.07</v>
       </c>
       <c r="O23" s="4" t="inlineStr">
         <is>
-          <t>✗</t>
+          <t>✓</t>
         </is>
       </c>
       <c r="P23" s="4" t="inlineStr">
@@ -3518,103 +3516,97 @@
         </is>
       </c>
       <c r="Q23" s="4" t="n">
-        <v>83.09</v>
+        <v>86.97</v>
       </c>
       <c r="R23" s="4" t="n">
-        <v>33.38</v>
+        <v>45.98</v>
       </c>
       <c r="S23" s="4" t="n">
-        <v>-320.1535</v>
+        <v>13.8206</v>
       </c>
       <c r="T23" s="4" t="n">
-        <v>-205.253</v>
+        <v>30.6456</v>
       </c>
       <c r="U23" s="4" t="n">
-        <v>-114.9005</v>
+        <v>-16.825</v>
       </c>
       <c r="V23" s="4" t="inlineStr"/>
       <c r="W23" s="4" t="n">
-        <v>19.47</v>
+        <v>20.78</v>
       </c>
       <c r="X23" s="4" t="n">
-        <v>194062</v>
+        <v>198724</v>
       </c>
       <c r="Y23" s="4" t="n">
-        <v>214902</v>
+        <v>398370</v>
       </c>
       <c r="Z23" s="4" t="n">
-        <v>0.9</v>
+        <v>0.5</v>
       </c>
       <c r="AA23" s="4" t="n">
-        <v>90760</v>
+        <v>16411</v>
       </c>
       <c r="AB23" s="4" t="n">
-        <v>26.631227</v>
+        <v>27.585049</v>
       </c>
       <c r="AC23" s="4" t="n">
-        <v>22.98445</v>
-      </c>
-      <c r="AD23" s="4" t="n">
-        <v>49.9</v>
-      </c>
+        <v>27.19669</v>
+      </c>
+      <c r="AD23" s="4" t="inlineStr"/>
       <c r="AE23" s="4" t="n">
-        <v>0.5669999999999999</v>
+        <v>10.529</v>
       </c>
       <c r="AF23" s="4" t="n">
-        <v>68.7</v>
-      </c>
-      <c r="AG23" s="4" t="n">
-        <v>120.2</v>
-      </c>
+        <v>29.3</v>
+      </c>
+      <c r="AG23" s="4" t="inlineStr"/>
       <c r="AH23" s="4" t="n">
-        <v>13.09733</v>
+        <v>5.593818</v>
       </c>
       <c r="AI23" s="4" t="n">
-        <v>638</v>
-      </c>
-      <c r="AJ23" s="4" t="n">
-        <v>4.413</v>
-      </c>
+        <v>90</v>
+      </c>
+      <c r="AJ23" s="4" t="inlineStr"/>
       <c r="AK23" s="4" t="inlineStr">
         <is>
-          <t>https://www.screener.in/company/OFSS/</t>
+          <t>https://www.screener.in/company/BEML/</t>
         </is>
       </c>
       <c r="AL23" s="4" t="inlineStr">
         <is>
-          <t>https://www.tradingview.com/chart/?symbol=NSE:OFSS</t>
+          <t>https://www.tradingview.com/chart/?symbol=NSE:BEML</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>LAURUSLABS</t>
+          <t>OFSS</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Laurus Labs Limited</t>
+          <t>Oracle Financial Services Software Limited</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Drug Manufacturers - Specialty &amp; Generic</t>
+          <t>Software - Infrastructure</t>
         </is>
       </c>
       <c r="E24" s="6" t="n">
-        <v>41.9</v>
+        <v>42.6</v>
       </c>
       <c r="F24" s="2" t="n">
-        <v>27.4</v>
+        <v>3.6</v>
       </c>
       <c r="G24" s="2" t="n">
-        <v>14.5</v>
+        <v>39</v>
       </c>
       <c r="H24" s="6" t="inlineStr">
         <is>
@@ -3623,108 +3615,112 @@
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>✅ Supertrend Buy | 📈 EMA Bull Stack | 🏆 Near 52W High | 📉 Tight Base</t>
+          <t>📉 Tight Base | 💎 High ROE | 👤 High Promoter</t>
         </is>
       </c>
       <c r="J24" s="2" t="n">
-        <v>1984</v>
+        <v>10420</v>
       </c>
       <c r="K24" s="2" t="n">
-        <v>0.2</v>
+        <v>-1.98</v>
       </c>
       <c r="L24" s="2" t="n">
-        <v>1961.42</v>
+        <v>11142.27</v>
       </c>
       <c r="M24" s="2" t="n">
-        <v>1857.88</v>
+        <v>11270.24</v>
       </c>
       <c r="N24" s="2" t="n">
-        <v>1464.64</v>
+        <v>9886.77</v>
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>✗</t>
         </is>
       </c>
       <c r="P24" s="2" t="inlineStr">
         <is>
-          <t>Buy</t>
+          <t>Sell</t>
         </is>
       </c>
       <c r="Q24" s="2" t="n">
-        <v>96.53</v>
+        <v>83.09</v>
       </c>
       <c r="R24" s="2" t="n">
-        <v>58.38</v>
+        <v>33.38</v>
       </c>
       <c r="S24" s="2" t="n">
-        <v>39.5147</v>
+        <v>-320.1535</v>
       </c>
       <c r="T24" s="2" t="n">
-        <v>45.8215</v>
+        <v>-205.253</v>
       </c>
       <c r="U24" s="2" t="n">
-        <v>-6.3068</v>
+        <v>-114.9005</v>
       </c>
       <c r="V24" s="2" t="inlineStr"/>
       <c r="W24" s="2" t="n">
-        <v>19.29</v>
+        <v>19.47</v>
       </c>
       <c r="X24" s="2" t="n">
-        <v>1459687</v>
+        <v>194062</v>
       </c>
       <c r="Y24" s="2" t="n">
-        <v>1615452</v>
+        <v>214902</v>
       </c>
       <c r="Z24" s="2" t="n">
         <v>0.9</v>
       </c>
       <c r="AA24" s="2" t="n">
-        <v>107198</v>
+        <v>91196</v>
       </c>
       <c r="AB24" s="2" t="n">
-        <v>98.02372</v>
+        <v>26.759016</v>
       </c>
       <c r="AC24" s="2" t="n">
-        <v>67.46165499999999</v>
-      </c>
-      <c r="AD24" s="2" t="inlineStr"/>
+        <v>23.120237</v>
+      </c>
+      <c r="AD24" s="2" t="n">
+        <v>49.9</v>
+      </c>
       <c r="AE24" s="2" t="n">
-        <v>46.369</v>
+        <v>0.5669999999999999</v>
       </c>
       <c r="AF24" s="2" t="n">
-        <v>29.1</v>
+        <v>68.7</v>
       </c>
       <c r="AG24" s="2" t="n">
-        <v>125.2</v>
+        <v>120.2</v>
       </c>
       <c r="AH24" s="2" t="n">
-        <v>20.20881</v>
+        <v>13.160177</v>
       </c>
       <c r="AI24" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AJ24" s="2" t="inlineStr"/>
+        <v>384</v>
+      </c>
+      <c r="AJ24" s="2" t="n">
+        <v>4.413</v>
+      </c>
       <c r="AK24" s="2" t="inlineStr">
         <is>
-          <t>https://www.screener.in/company/LAURUSLABS/</t>
+          <t>https://www.screener.in/company/OFSS/</t>
         </is>
       </c>
       <c r="AL24" s="2" t="inlineStr">
         <is>
-          <t>https://www.tradingview.com/chart/?symbol=NSE:LAURUSLABS</t>
+          <t>https://www.tradingview.com/chart/?symbol=NSE:OFSS</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>AUROPHARMA</t>
+          <t>LAURUSLABS</t>
         </is>
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>Aurobindo Pharma Limited</t>
+          <t>Laurus Labs Limited</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
@@ -3738,13 +3734,13 @@
         </is>
       </c>
       <c r="E25" s="6" t="n">
-        <v>41.59999999999999</v>
+        <v>41.9</v>
       </c>
       <c r="F25" s="4" t="n">
-        <v>22.4</v>
+        <v>27.4</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>19.2</v>
+        <v>14.5</v>
       </c>
       <c r="H25" s="6" t="inlineStr">
         <is>
@@ -3757,19 +3753,19 @@
         </is>
       </c>
       <c r="J25" s="4" t="n">
-        <v>1676.8</v>
+        <v>1984</v>
       </c>
       <c r="K25" s="4" t="n">
-        <v>0.29</v>
+        <v>0.2</v>
       </c>
       <c r="L25" s="4" t="n">
-        <v>1684.48</v>
+        <v>1961.42</v>
       </c>
       <c r="M25" s="4" t="n">
-        <v>1645.98</v>
+        <v>1857.88</v>
       </c>
       <c r="N25" s="4" t="n">
-        <v>1462.28</v>
+        <v>1464.79</v>
       </c>
       <c r="O25" s="4" t="inlineStr">
         <is>
@@ -3782,89 +3778,89 @@
         </is>
       </c>
       <c r="Q25" s="4" t="n">
-        <v>96.37</v>
+        <v>96.53</v>
       </c>
       <c r="R25" s="4" t="n">
-        <v>50.08</v>
+        <v>58.38</v>
       </c>
       <c r="S25" s="4" t="n">
-        <v>13.4115</v>
+        <v>39.5147</v>
       </c>
       <c r="T25" s="4" t="n">
-        <v>18.5697</v>
+        <v>45.8215</v>
       </c>
       <c r="U25" s="4" t="n">
-        <v>-5.1582</v>
+        <v>-6.3068</v>
       </c>
       <c r="V25" s="4" t="inlineStr"/>
       <c r="W25" s="4" t="n">
-        <v>17.96</v>
+        <v>19.29</v>
       </c>
       <c r="X25" s="4" t="n">
-        <v>1074057</v>
+        <v>1459687</v>
       </c>
       <c r="Y25" s="4" t="n">
-        <v>759336</v>
+        <v>1615452</v>
       </c>
       <c r="Z25" s="4" t="n">
-        <v>1.41</v>
+        <v>0.9</v>
       </c>
       <c r="AA25" s="4" t="n">
-        <v>96479</v>
+        <v>106517</v>
       </c>
       <c r="AB25" s="4" t="n">
-        <v>26.183636</v>
+        <v>97.44933</v>
       </c>
       <c r="AC25" s="4" t="n">
-        <v>18.013765</v>
+        <v>66.83839999999999</v>
       </c>
       <c r="AD25" s="4" t="inlineStr"/>
       <c r="AE25" s="4" t="n">
-        <v>21.31</v>
+        <v>46.369</v>
       </c>
       <c r="AF25" s="4" t="n">
-        <v>16.3</v>
+        <v>29.1</v>
       </c>
       <c r="AG25" s="4" t="n">
-        <v>25.8</v>
+        <v>125.2</v>
       </c>
       <c r="AH25" s="4" t="n">
-        <v>2.5702379</v>
+        <v>20.080467</v>
       </c>
       <c r="AI25" s="4" t="n">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="AJ25" s="4" t="inlineStr"/>
       <c r="AK25" s="4" t="inlineStr">
         <is>
-          <t>https://www.screener.in/company/AUROPHARMA/</t>
+          <t>https://www.screener.in/company/LAURUSLABS/</t>
         </is>
       </c>
       <c r="AL25" s="4" t="inlineStr">
         <is>
-          <t>https://www.tradingview.com/chart/?symbol=NSE:AUROPHARMA</t>
+          <t>https://www.tradingview.com/chart/?symbol=NSE:LAURUSLABS</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>MOTHERSON</t>
+          <t>AUROPHARMA</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Samvardhana Motherson International Limited</t>
+          <t>Aurobindo Pharma Limited</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Consumer Cyclical</t>
+          <t>Healthcare</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Auto Parts</t>
+          <t>Drug Manufacturers - Specialty &amp; Generic</t>
         </is>
       </c>
       <c r="E26" s="6" t="n">
@@ -3883,23 +3879,23 @@
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>📈 EMA Bull Stack | 📊 High Volume | 🏆 Near 52W High | 📉 Tight Base</t>
+          <t>✅ Supertrend Buy | 📈 EMA Bull Stack | 🏆 Near 52W High | 📉 Tight Base</t>
         </is>
       </c>
       <c r="J26" s="2" t="n">
-        <v>157.03</v>
+        <v>1676.8</v>
       </c>
       <c r="K26" s="2" t="n">
-        <v>-3.82</v>
+        <v>0.29</v>
       </c>
       <c r="L26" s="2" t="n">
-        <v>162.1</v>
+        <v>1684.48</v>
       </c>
       <c r="M26" s="2" t="n">
-        <v>159.66</v>
+        <v>1645.98</v>
       </c>
       <c r="N26" s="2" t="n">
-        <v>139.69</v>
+        <v>1462.94</v>
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
@@ -3908,103 +3904,103 @@
       </c>
       <c r="P26" s="2" t="inlineStr">
         <is>
-          <t>Sell</t>
+          <t>Buy</t>
         </is>
       </c>
       <c r="Q26" s="2" t="n">
-        <v>90.63</v>
+        <v>96.37</v>
       </c>
       <c r="R26" s="2" t="n">
-        <v>42.52</v>
+        <v>50.08</v>
       </c>
       <c r="S26" s="2" t="n">
-        <v>-0.4109</v>
+        <v>13.4115</v>
       </c>
       <c r="T26" s="2" t="n">
-        <v>0.136</v>
+        <v>18.5697</v>
       </c>
       <c r="U26" s="2" t="n">
-        <v>-0.5468</v>
+        <v>-5.1582</v>
       </c>
       <c r="V26" s="2" t="inlineStr"/>
       <c r="W26" s="2" t="n">
-        <v>18.66</v>
+        <v>17.96</v>
       </c>
       <c r="X26" s="2" t="n">
-        <v>23039471</v>
+        <v>1074057</v>
       </c>
       <c r="Y26" s="2" t="n">
-        <v>11388720</v>
+        <v>759336</v>
       </c>
       <c r="Z26" s="2" t="n">
-        <v>2.02</v>
+        <v>1.41</v>
       </c>
       <c r="AA26" s="2" t="n">
-        <v>165372</v>
+        <v>96370</v>
       </c>
       <c r="AB26" s="2" t="n">
-        <v>37.035378</v>
+        <v>26.170313</v>
       </c>
       <c r="AC26" s="2" t="n">
-        <v>22.609306</v>
+        <v>17.945934</v>
       </c>
       <c r="AD26" s="2" t="inlineStr"/>
       <c r="AE26" s="2" t="n">
-        <v>43.908</v>
+        <v>21.31</v>
       </c>
       <c r="AF26" s="2" t="n">
-        <v>16.6</v>
+        <v>16.3</v>
       </c>
       <c r="AG26" s="2" t="n">
-        <v>104.2</v>
+        <v>25.8</v>
       </c>
       <c r="AH26" s="2" t="n">
-        <v>4.0355163</v>
+        <v>2.5673256</v>
       </c>
       <c r="AI26" s="2" t="n">
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="AJ26" s="2" t="inlineStr"/>
       <c r="AK26" s="2" t="inlineStr">
         <is>
-          <t>https://www.screener.in/company/MOTHERSON/</t>
+          <t>https://www.screener.in/company/AUROPHARMA/</t>
         </is>
       </c>
       <c r="AL26" s="2" t="inlineStr">
         <is>
-          <t>https://www.tradingview.com/chart/?symbol=NSE:MOTHERSON</t>
+          <t>https://www.tradingview.com/chart/?symbol=NSE:AUROPHARMA</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>SIEMENS</t>
+          <t>MOTHERSON</t>
         </is>
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>Siemens Limited</t>
+          <t>Samvardhana Motherson International Limited</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Consumer Cyclical</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>Specialty Industrial Machinery</t>
+          <t>Auto Parts</t>
         </is>
       </c>
       <c r="E27" s="6" t="n">
-        <v>41.3</v>
+        <v>41.59999999999999</v>
       </c>
       <c r="F27" s="4" t="n">
-        <v>24</v>
+        <v>22.4</v>
       </c>
       <c r="G27" s="4" t="n">
-        <v>17.3</v>
+        <v>19.2</v>
       </c>
       <c r="H27" s="6" t="inlineStr">
         <is>
@@ -4013,23 +4009,23 @@
       </c>
       <c r="I27" s="4" t="inlineStr">
         <is>
-          <t>📈 EMA Bull Stack | 🏆 Near 52W High | 📉 Tight Base | 👤 High Promoter</t>
+          <t>📈 EMA Bull Stack | 📊 High Volume | 🏆 Near 52W High | 📉 Tight Base</t>
         </is>
       </c>
       <c r="J27" s="4" t="n">
-        <v>3804</v>
+        <v>157.03</v>
       </c>
       <c r="K27" s="4" t="n">
-        <v>2.1</v>
+        <v>-3.82</v>
       </c>
       <c r="L27" s="4" t="n">
-        <v>3850.01</v>
+        <v>162.1</v>
       </c>
       <c r="M27" s="4" t="n">
-        <v>3848.93</v>
+        <v>159.66</v>
       </c>
       <c r="N27" s="4" t="n">
-        <v>3594.58</v>
+        <v>139.73</v>
       </c>
       <c r="O27" s="4" t="inlineStr">
         <is>
@@ -4042,99 +4038,99 @@
         </is>
       </c>
       <c r="Q27" s="4" t="n">
-        <v>91.68000000000001</v>
+        <v>90.63</v>
       </c>
       <c r="R27" s="4" t="n">
-        <v>45.38</v>
+        <v>42.52</v>
       </c>
       <c r="S27" s="4" t="n">
-        <v>-40.3953</v>
+        <v>-0.4109</v>
       </c>
       <c r="T27" s="4" t="n">
-        <v>-25.8195</v>
+        <v>0.136</v>
       </c>
       <c r="U27" s="4" t="n">
-        <v>-14.5758</v>
+        <v>-0.5468</v>
       </c>
       <c r="V27" s="4" t="inlineStr"/>
       <c r="W27" s="4" t="n">
-        <v>22.06</v>
+        <v>18.66</v>
       </c>
       <c r="X27" s="4" t="n">
-        <v>243713</v>
+        <v>23039471</v>
       </c>
       <c r="Y27" s="4" t="n">
-        <v>242322</v>
+        <v>11388720</v>
       </c>
       <c r="Z27" s="4" t="n">
-        <v>1.01</v>
+        <v>2.02</v>
       </c>
       <c r="AA27" s="4" t="n">
-        <v>135468</v>
+        <v>164814</v>
       </c>
       <c r="AB27" s="4" t="n">
-        <v>80.38884</v>
+        <v>37.710842</v>
       </c>
       <c r="AC27" s="4" t="n">
-        <v>56.13101</v>
+        <v>22.532995</v>
       </c>
       <c r="AD27" s="4" t="inlineStr"/>
       <c r="AE27" s="4" t="n">
-        <v>2.213</v>
+        <v>43.908</v>
       </c>
       <c r="AF27" s="4" t="n">
-        <v>14.8</v>
+        <v>16.6</v>
       </c>
       <c r="AG27" s="4" t="n">
-        <v>406.1</v>
+        <v>104.2</v>
       </c>
       <c r="AH27" s="4" t="n">
-        <v>9.788029</v>
+        <v>4.021896</v>
       </c>
       <c r="AI27" s="4" t="n">
-        <v>47</v>
+        <v>32</v>
       </c>
       <c r="AJ27" s="4" t="inlineStr"/>
       <c r="AK27" s="4" t="inlineStr">
         <is>
-          <t>https://www.screener.in/company/SIEMENS/</t>
+          <t>https://www.screener.in/company/MOTHERSON/</t>
         </is>
       </c>
       <c r="AL27" s="4" t="inlineStr">
         <is>
-          <t>https://www.tradingview.com/chart/?symbol=NSE:SIEMENS</t>
+          <t>https://www.tradingview.com/chart/?symbol=NSE:MOTHERSON</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>PERSISTENT</t>
+          <t>SIEMENS</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Persistent Systems Limited</t>
+          <t>Siemens Limited</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Information Technology Services</t>
+          <t>Specialty Industrial Machinery</t>
         </is>
       </c>
       <c r="E28" s="6" t="n">
-        <v>40.6</v>
+        <v>41.3</v>
       </c>
       <c r="F28" s="2" t="n">
-        <v>16.8</v>
+        <v>24</v>
       </c>
       <c r="G28" s="2" t="n">
-        <v>23.8</v>
+        <v>17.3</v>
       </c>
       <c r="H28" s="6" t="inlineStr">
         <is>
@@ -4143,23 +4139,23 @@
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>📈 EMA Bull Stack | 📉 Tight Base | 💎 High ROE</t>
+          <t>📈 EMA Bull Stack | 🏆 Near 52W High | 📉 Tight Base | 👤 High Promoter</t>
         </is>
       </c>
       <c r="J28" s="2" t="n">
-        <v>5367</v>
+        <v>3804</v>
       </c>
       <c r="K28" s="2" t="n">
-        <v>1.67</v>
+        <v>2.1</v>
       </c>
       <c r="L28" s="2" t="n">
-        <v>5396.68</v>
+        <v>3850.01</v>
       </c>
       <c r="M28" s="2" t="n">
-        <v>5396</v>
+        <v>3848.92</v>
       </c>
       <c r="N28" s="2" t="n">
-        <v>5321.51</v>
+        <v>3592.63</v>
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
@@ -4172,103 +4168,99 @@
         </is>
       </c>
       <c r="Q28" s="2" t="n">
-        <v>81.91</v>
+        <v>91.68000000000001</v>
       </c>
       <c r="R28" s="2" t="n">
-        <v>47.66</v>
+        <v>45.38</v>
       </c>
       <c r="S28" s="2" t="n">
-        <v>-62.5577</v>
+        <v>-40.3953</v>
       </c>
       <c r="T28" s="2" t="n">
-        <v>-45.3151</v>
+        <v>-25.8195</v>
       </c>
       <c r="U28" s="2" t="n">
-        <v>-17.2426</v>
+        <v>-14.5758</v>
       </c>
       <c r="V28" s="2" t="inlineStr"/>
       <c r="W28" s="2" t="n">
-        <v>14.41</v>
+        <v>22.06</v>
       </c>
       <c r="X28" s="2" t="n">
-        <v>506268</v>
+        <v>243713</v>
       </c>
       <c r="Y28" s="2" t="n">
-        <v>400031</v>
+        <v>242322</v>
       </c>
       <c r="Z28" s="2" t="n">
-        <v>1.27</v>
+        <v>1.01</v>
       </c>
       <c r="AA28" s="2" t="n">
-        <v>83849</v>
+        <v>131804</v>
       </c>
       <c r="AB28" s="2" t="n">
-        <v>43.858788</v>
+        <v>90.73547000000001</v>
       </c>
       <c r="AC28" s="2" t="n">
-        <v>30.282188</v>
-      </c>
-      <c r="AD28" s="2" t="n">
-        <v>25.2</v>
-      </c>
+        <v>54.61264</v>
+      </c>
+      <c r="AD28" s="2" t="inlineStr"/>
       <c r="AE28" s="2" t="n">
-        <v>6.94</v>
+        <v>2.213</v>
       </c>
       <c r="AF28" s="2" t="n">
-        <v>29.1</v>
+        <v>14.8</v>
       </c>
       <c r="AG28" s="2" t="n">
-        <v>12.1</v>
+        <v>406.1</v>
       </c>
       <c r="AH28" s="2" t="n">
-        <v>9.973223000000001</v>
+        <v>9.523258</v>
       </c>
       <c r="AI28" s="2" t="n">
-        <v>67</v>
-      </c>
-      <c r="AJ28" s="2" t="n">
-        <v>2.711</v>
-      </c>
+        <v>47</v>
+      </c>
+      <c r="AJ28" s="2" t="inlineStr"/>
       <c r="AK28" s="2" t="inlineStr">
         <is>
-          <t>https://www.screener.in/company/PERSISTENT/</t>
+          <t>https://www.screener.in/company/SIEMENS/</t>
         </is>
       </c>
       <c r="AL28" s="2" t="inlineStr">
         <is>
-          <t>https://www.tradingview.com/chart/?symbol=NSE:PERSISTENT</t>
+          <t>https://www.tradingview.com/chart/?symbol=NSE:SIEMENS</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>PERSISTENT</t>
         </is>
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>Adani Ports and Special Economic Zone Limited</t>
+          <t>Persistent Systems Limited</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>Marine Shipping</t>
+          <t>Information Technology Services</t>
         </is>
       </c>
       <c r="E29" s="6" t="n">
-        <v>39.9</v>
+        <v>40.6</v>
       </c>
       <c r="F29" s="4" t="n">
-        <v>19.2</v>
+        <v>16.8</v>
       </c>
       <c r="G29" s="4" t="n">
-        <v>20.7</v>
+        <v>23.8</v>
       </c>
       <c r="H29" s="6" t="inlineStr">
         <is>
@@ -4277,23 +4269,23 @@
       </c>
       <c r="I29" s="4" t="inlineStr">
         <is>
-          <t>✅ Supertrend Buy | 📈 EMA Bull Stack | 🏆 Near 52W High | 📉 Tight Base</t>
+          <t>📈 EMA Bull Stack | 📉 Tight Base | 💎 High ROE</t>
         </is>
       </c>
       <c r="J29" s="4" t="n">
-        <v>1737.8</v>
+        <v>5367</v>
       </c>
       <c r="K29" s="4" t="n">
-        <v>-3.36</v>
+        <v>1.67</v>
       </c>
       <c r="L29" s="4" t="n">
-        <v>1761.16</v>
+        <v>5396.68</v>
       </c>
       <c r="M29" s="4" t="n">
-        <v>1744.7</v>
+        <v>5396</v>
       </c>
       <c r="N29" s="4" t="n">
-        <v>1649.82</v>
+        <v>5320.61</v>
       </c>
       <c r="O29" s="4" t="inlineStr">
         <is>
@@ -4302,103 +4294,107 @@
       </c>
       <c r="P29" s="4" t="inlineStr">
         <is>
-          <t>Buy</t>
+          <t>Sell</t>
         </is>
       </c>
       <c r="Q29" s="4" t="n">
-        <v>91.89</v>
+        <v>81.91</v>
       </c>
       <c r="R29" s="4" t="n">
-        <v>47.93</v>
+        <v>47.66</v>
       </c>
       <c r="S29" s="4" t="n">
-        <v>17.2875</v>
+        <v>-62.5577</v>
       </c>
       <c r="T29" s="4" t="n">
-        <v>18.3936</v>
+        <v>-45.3151</v>
       </c>
       <c r="U29" s="4" t="n">
-        <v>-1.1061</v>
+        <v>-17.2426</v>
       </c>
       <c r="V29" s="4" t="inlineStr"/>
       <c r="W29" s="4" t="n">
-        <v>17.51</v>
+        <v>14.41</v>
       </c>
       <c r="X29" s="4" t="n">
-        <v>2157928</v>
+        <v>506268</v>
       </c>
       <c r="Y29" s="4" t="n">
-        <v>1947992</v>
+        <v>400031</v>
       </c>
       <c r="Z29" s="4" t="n">
-        <v>1.11</v>
+        <v>1.27</v>
       </c>
       <c r="AA29" s="4" t="n">
-        <v>400382</v>
+        <v>86396</v>
       </c>
       <c r="AB29" s="4" t="n">
-        <v>29.675547</v>
+        <v>45.272205</v>
       </c>
       <c r="AC29" s="4" t="n">
-        <v>22.230867</v>
-      </c>
-      <c r="AD29" s="4" t="inlineStr"/>
+        <v>31.18118</v>
+      </c>
+      <c r="AD29" s="4" t="n">
+        <v>25.2</v>
+      </c>
       <c r="AE29" s="4" t="n">
-        <v>64.051</v>
+        <v>6.94</v>
       </c>
       <c r="AF29" s="4" t="n">
-        <v>18.6</v>
+        <v>29.1</v>
       </c>
       <c r="AG29" s="4" t="n">
-        <v>2.4</v>
+        <v>12.1</v>
       </c>
       <c r="AH29" s="4" t="n">
-        <v>4.172439</v>
+        <v>10.276117</v>
       </c>
       <c r="AI29" s="4" t="n">
-        <v>43</v>
-      </c>
-      <c r="AJ29" s="4" t="inlineStr"/>
+        <v>67</v>
+      </c>
+      <c r="AJ29" s="4" t="n">
+        <v>2.711</v>
+      </c>
       <c r="AK29" s="4" t="inlineStr">
         <is>
-          <t>https://www.screener.in/company/ADANIPORTS/</t>
+          <t>https://www.screener.in/company/PERSISTENT/</t>
         </is>
       </c>
       <c r="AL29" s="4" t="inlineStr">
         <is>
-          <t>https://www.tradingview.com/chart/?symbol=NSE:ADANIPORTS</t>
+          <t>https://www.tradingview.com/chart/?symbol=NSE:PERSISTENT</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>IDFCFIRSTB</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>IDFC First Bank Limited</t>
+          <t>Adani Ports and Special Economic Zone Limited</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Financial Services</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Banks - Regional</t>
+          <t>Marine Shipping</t>
         </is>
       </c>
       <c r="E30" s="6" t="n">
-        <v>39.7</v>
+        <v>39.9</v>
       </c>
       <c r="F30" s="2" t="n">
-        <v>21.6</v>
+        <v>19.2</v>
       </c>
       <c r="G30" s="2" t="n">
-        <v>18.1</v>
+        <v>20.7</v>
       </c>
       <c r="H30" s="6" t="inlineStr">
         <is>
@@ -4407,23 +4403,23 @@
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>📈 EMA Bull Stack | 📉 Tight Base</t>
+          <t>✅ Supertrend Buy | 📈 EMA Bull Stack | 🏆 Near 52W High | 📉 Tight Base</t>
         </is>
       </c>
       <c r="J30" s="2" t="n">
-        <v>80.39</v>
+        <v>1737.8</v>
       </c>
       <c r="K30" s="2" t="n">
-        <v>-1.29</v>
+        <v>-3.36</v>
       </c>
       <c r="L30" s="2" t="n">
-        <v>83.83</v>
+        <v>1761.16</v>
       </c>
       <c r="M30" s="2" t="n">
-        <v>83.55</v>
+        <v>1744.7</v>
       </c>
       <c r="N30" s="2" t="n">
-        <v>78.40000000000001</v>
+        <v>1650.28</v>
       </c>
       <c r="O30" s="2" t="inlineStr">
         <is>
@@ -4432,103 +4428,103 @@
       </c>
       <c r="P30" s="2" t="inlineStr">
         <is>
-          <t>Sell</t>
+          <t>Buy</t>
         </is>
       </c>
       <c r="Q30" s="2" t="n">
-        <v>89.70999999999999</v>
+        <v>91.89</v>
       </c>
       <c r="R30" s="2" t="n">
-        <v>38.17</v>
+        <v>47.93</v>
       </c>
       <c r="S30" s="2" t="n">
-        <v>-1.0337</v>
+        <v>17.2875</v>
       </c>
       <c r="T30" s="2" t="n">
-        <v>-0.3093</v>
+        <v>18.3936</v>
       </c>
       <c r="U30" s="2" t="n">
-        <v>-0.7244</v>
+        <v>-1.1061</v>
       </c>
       <c r="V30" s="2" t="inlineStr"/>
       <c r="W30" s="2" t="n">
-        <v>20.63</v>
+        <v>17.51</v>
       </c>
       <c r="X30" s="2" t="n">
-        <v>24434109</v>
+        <v>2157928</v>
       </c>
       <c r="Y30" s="2" t="n">
-        <v>21412158</v>
+        <v>1947992</v>
       </c>
       <c r="Z30" s="2" t="n">
-        <v>1.14</v>
+        <v>1.11</v>
       </c>
       <c r="AA30" s="2" t="n">
-        <v>69319</v>
+        <v>408722</v>
       </c>
       <c r="AB30" s="2" t="n">
-        <v>31.03861</v>
+        <v>30.278204</v>
       </c>
       <c r="AC30" s="2" t="n">
-        <v>11.817558</v>
-      </c>
-      <c r="AD30" s="2" t="n">
-        <v>5.26</v>
-      </c>
-      <c r="AE30" s="2" t="inlineStr"/>
+        <v>22.692484</v>
+      </c>
+      <c r="AD30" s="2" t="inlineStr"/>
+      <c r="AE30" s="2" t="n">
+        <v>64.051</v>
+      </c>
       <c r="AF30" s="2" t="n">
-        <v>29.8</v>
+        <v>18.6</v>
       </c>
       <c r="AG30" s="2" t="n">
-        <v>116.4</v>
+        <v>2.4</v>
       </c>
       <c r="AH30" s="2" t="n">
-        <v>1.4223787</v>
+        <v>4.259355</v>
       </c>
       <c r="AI30" s="2" t="n">
-        <v>31</v>
+        <v>43</v>
       </c>
       <c r="AJ30" s="2" t="inlineStr"/>
       <c r="AK30" s="2" t="inlineStr">
         <is>
-          <t>https://www.screener.in/company/IDFCFIRSTB/</t>
+          <t>https://www.screener.in/company/ADANIPORTS/</t>
         </is>
       </c>
       <c r="AL30" s="2" t="inlineStr">
         <is>
-          <t>https://www.tradingview.com/chart/?symbol=NSE:IDFCFIRSTB</t>
+          <t>https://www.tradingview.com/chart/?symbol=NSE:ADANIPORTS</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>NYKAA</t>
+          <t>IDFCFIRSTB</t>
         </is>
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>FSN E-Commerce Ventures Limited</t>
+          <t>IDFC First Bank Limited</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>Consumer Cyclical</t>
+          <t>Financial Services</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>Internet Retail</t>
+          <t>Banks - Regional</t>
         </is>
       </c>
       <c r="E31" s="6" t="n">
-        <v>39</v>
+        <v>39.7</v>
       </c>
       <c r="F31" s="4" t="n">
-        <v>22.4</v>
+        <v>21.6</v>
       </c>
       <c r="G31" s="4" t="n">
-        <v>16.6</v>
+        <v>18.1</v>
       </c>
       <c r="H31" s="6" t="inlineStr">
         <is>
@@ -4537,23 +4533,23 @@
       </c>
       <c r="I31" s="4" t="inlineStr">
         <is>
-          <t>📈 EMA Bull Stack | 📊 High Volume | 🏆 Near 52W High | 📉 Tight Base</t>
+          <t>📈 EMA Bull Stack | 📉 Tight Base</t>
         </is>
       </c>
       <c r="J31" s="4" t="n">
-        <v>324.95</v>
+        <v>80.39</v>
       </c>
       <c r="K31" s="4" t="n">
-        <v>1.55</v>
+        <v>-1.29</v>
       </c>
       <c r="L31" s="4" t="n">
-        <v>331.59</v>
+        <v>83.83</v>
       </c>
       <c r="M31" s="4" t="n">
-        <v>328.46</v>
+        <v>83.55</v>
       </c>
       <c r="N31" s="4" t="n">
-        <v>293.6</v>
+        <v>78.40000000000001</v>
       </c>
       <c r="O31" s="4" t="inlineStr">
         <is>
@@ -4566,99 +4562,99 @@
         </is>
       </c>
       <c r="Q31" s="4" t="n">
-        <v>92.95999999999999</v>
+        <v>89.70999999999999</v>
       </c>
       <c r="R31" s="4" t="n">
-        <v>44.32</v>
+        <v>38.17</v>
       </c>
       <c r="S31" s="4" t="n">
-        <v>-1.9872</v>
+        <v>-1.0337</v>
       </c>
       <c r="T31" s="4" t="n">
-        <v>-0.2497</v>
+        <v>-0.3093</v>
       </c>
       <c r="U31" s="4" t="n">
-        <v>-1.7375</v>
+        <v>-0.7244</v>
       </c>
       <c r="V31" s="4" t="inlineStr"/>
       <c r="W31" s="4" t="n">
-        <v>18.23</v>
+        <v>20.63</v>
       </c>
       <c r="X31" s="4" t="n">
-        <v>7907193</v>
+        <v>24434109</v>
       </c>
       <c r="Y31" s="4" t="n">
-        <v>3778052</v>
+        <v>21412158</v>
       </c>
       <c r="Z31" s="4" t="n">
-        <v>2.09</v>
+        <v>1.14</v>
       </c>
       <c r="AA31" s="4" t="n">
-        <v>93107</v>
+        <v>70897</v>
       </c>
       <c r="AB31" s="4" t="n">
-        <v>365.11237</v>
+        <v>31.745174</v>
       </c>
       <c r="AC31" s="4" t="n">
-        <v>110.70344</v>
-      </c>
-      <c r="AD31" s="4" t="inlineStr"/>
-      <c r="AE31" s="4" t="n">
-        <v>82.82899999999999</v>
-      </c>
+        <v>12.086182</v>
+      </c>
+      <c r="AD31" s="4" t="n">
+        <v>5.26</v>
+      </c>
+      <c r="AE31" s="4" t="inlineStr"/>
       <c r="AF31" s="4" t="n">
-        <v>29.1</v>
+        <v>29.8</v>
       </c>
       <c r="AG31" s="4" t="n">
-        <v>250</v>
+        <v>116.4</v>
       </c>
       <c r="AH31" s="4" t="n">
-        <v>64.70529999999999</v>
+        <v>1.4547578</v>
       </c>
       <c r="AI31" s="4" t="n">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="AJ31" s="4" t="inlineStr"/>
       <c r="AK31" s="4" t="inlineStr">
         <is>
-          <t>https://www.screener.in/company/NYKAA/</t>
+          <t>https://www.screener.in/company/IDFCFIRSTB/</t>
         </is>
       </c>
       <c r="AL31" s="4" t="inlineStr">
         <is>
-          <t>https://www.tradingview.com/chart/?symbol=NSE:NYKAA</t>
+          <t>https://www.tradingview.com/chart/?symbol=NSE:IDFCFIRSTB</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>TORNTPHARM</t>
+          <t>NYKAA</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Torrent Pharmaceuticals Limited</t>
+          <t>FSN E-Commerce Ventures Limited</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Consumer Cyclical</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Drug Manufacturers - Specialty &amp; Generic</t>
+          <t>Internet Retail</t>
         </is>
       </c>
       <c r="E32" s="6" t="n">
-        <v>38.5</v>
+        <v>39</v>
       </c>
       <c r="F32" s="2" t="n">
-        <v>16.8</v>
+        <v>22.4</v>
       </c>
       <c r="G32" s="2" t="n">
-        <v>21.7</v>
+        <v>16.6</v>
       </c>
       <c r="H32" s="6" t="inlineStr">
         <is>
@@ -4667,23 +4663,23 @@
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>✅ Supertrend Buy | 📈 EMA Bull Stack | 🏆 Near 52W High | 📉 Tight Base</t>
+          <t>📈 EMA Bull Stack | 📊 High Volume | 🏆 Near 52W High | 📉 Tight Base</t>
         </is>
       </c>
       <c r="J32" s="2" t="n">
-        <v>4767.3</v>
+        <v>324.95</v>
       </c>
       <c r="K32" s="2" t="n">
-        <v>-0.68</v>
+        <v>1.55</v>
       </c>
       <c r="L32" s="2" t="n">
-        <v>4897.78</v>
+        <v>331.59</v>
       </c>
       <c r="M32" s="2" t="n">
-        <v>4883.86</v>
+        <v>328.46</v>
       </c>
       <c r="N32" s="2" t="n">
-        <v>4501.02</v>
+        <v>293.85</v>
       </c>
       <c r="O32" s="2" t="inlineStr">
         <is>
@@ -4692,83 +4688,83 @@
       </c>
       <c r="P32" s="2" t="inlineStr">
         <is>
-          <t>Buy</t>
+          <t>Sell</t>
         </is>
       </c>
       <c r="Q32" s="2" t="n">
-        <v>90.81</v>
+        <v>92.95999999999999</v>
       </c>
       <c r="R32" s="2" t="n">
-        <v>40.85</v>
+        <v>44.32</v>
       </c>
       <c r="S32" s="2" t="n">
-        <v>-22.6091</v>
+        <v>-1.9872</v>
       </c>
       <c r="T32" s="2" t="n">
-        <v>-7.9207</v>
+        <v>-0.2497</v>
       </c>
       <c r="U32" s="2" t="n">
-        <v>-14.6885</v>
+        <v>-1.7375</v>
       </c>
       <c r="V32" s="2" t="inlineStr"/>
       <c r="W32" s="2" t="n">
-        <v>16.73</v>
+        <v>18.23</v>
       </c>
       <c r="X32" s="2" t="n">
-        <v>357701</v>
+        <v>7907193</v>
       </c>
       <c r="Y32" s="2" t="n">
-        <v>340691</v>
+        <v>3778052</v>
       </c>
       <c r="Z32" s="2" t="n">
-        <v>1.05</v>
+        <v>2.09</v>
       </c>
       <c r="AA32" s="2" t="n">
-        <v>181333</v>
+        <v>97290</v>
       </c>
       <c r="AB32" s="2" t="n">
-        <v>76.10632</v>
+        <v>381.51685</v>
       </c>
       <c r="AC32" s="2" t="n">
-        <v>51.178196</v>
+        <v>115.656456</v>
       </c>
       <c r="AD32" s="2" t="inlineStr"/>
       <c r="AE32" s="2" t="n">
-        <v>85.446</v>
+        <v>82.82899999999999</v>
       </c>
       <c r="AF32" s="2" t="n">
-        <v>54.8</v>
+        <v>29.1</v>
       </c>
       <c r="AG32" s="2" t="n">
-        <v>-8.199999999999999</v>
+        <v>250</v>
       </c>
       <c r="AH32" s="2" t="n">
-        <v>19.23446</v>
+        <v>67.6125</v>
       </c>
       <c r="AI32" s="2" t="n">
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="AJ32" s="2" t="inlineStr"/>
       <c r="AK32" s="2" t="inlineStr">
         <is>
-          <t>https://www.screener.in/company/TORNTPHARM/</t>
+          <t>https://www.screener.in/company/NYKAA/</t>
         </is>
       </c>
       <c r="AL32" s="2" t="inlineStr">
         <is>
-          <t>https://www.tradingview.com/chart/?symbol=NSE:TORNTPHARM</t>
+          <t>https://www.tradingview.com/chart/?symbol=NSE:NYKAA</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>GRANULES</t>
+          <t>TORNTPHARM</t>
         </is>
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>Granules India Limited</t>
+          <t>Torrent Pharmaceuticals Limited</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr">
@@ -4782,13 +4778,13 @@
         </is>
       </c>
       <c r="E33" s="6" t="n">
-        <v>38.3</v>
+        <v>38.5</v>
       </c>
       <c r="F33" s="4" t="n">
-        <v>19.2</v>
+        <v>16.8</v>
       </c>
       <c r="G33" s="4" t="n">
-        <v>19.1</v>
+        <v>21.7</v>
       </c>
       <c r="H33" s="6" t="inlineStr">
         <is>
@@ -4797,23 +4793,23 @@
       </c>
       <c r="I33" s="4" t="inlineStr">
         <is>
-          <t>📈 EMA Bull Stack | 📉 Tight Base</t>
+          <t>✅ Supertrend Buy | 📈 EMA Bull Stack | 🏆 Near 52W High | 📉 Tight Base</t>
         </is>
       </c>
       <c r="J33" s="4" t="n">
-        <v>821.75</v>
+        <v>4767.3</v>
       </c>
       <c r="K33" s="4" t="n">
-        <v>-2.93</v>
+        <v>-0.68</v>
       </c>
       <c r="L33" s="4" t="n">
-        <v>858.76</v>
+        <v>4897.78</v>
       </c>
       <c r="M33" s="4" t="n">
-        <v>850.74</v>
+        <v>4883.86</v>
       </c>
       <c r="N33" s="4" t="n">
-        <v>743.41</v>
+        <v>4502.99</v>
       </c>
       <c r="O33" s="4" t="inlineStr">
         <is>
@@ -4822,103 +4818,103 @@
       </c>
       <c r="P33" s="4" t="inlineStr">
         <is>
-          <t>Sell</t>
+          <t>Buy</t>
         </is>
       </c>
       <c r="Q33" s="4" t="n">
-        <v>88.97</v>
+        <v>90.81</v>
       </c>
       <c r="R33" s="4" t="n">
-        <v>40.27</v>
+        <v>40.85</v>
       </c>
       <c r="S33" s="4" t="n">
-        <v>-2.9133</v>
+        <v>-22.6091</v>
       </c>
       <c r="T33" s="4" t="n">
-        <v>2.3115</v>
+        <v>-7.9207</v>
       </c>
       <c r="U33" s="4" t="n">
-        <v>-5.2248</v>
+        <v>-14.6885</v>
       </c>
       <c r="V33" s="4" t="inlineStr"/>
       <c r="W33" s="4" t="n">
-        <v>20.15</v>
+        <v>16.73</v>
       </c>
       <c r="X33" s="4" t="n">
-        <v>783432</v>
+        <v>357701</v>
       </c>
       <c r="Y33" s="4" t="n">
-        <v>1389889</v>
+        <v>340691</v>
       </c>
       <c r="Z33" s="4" t="n">
-        <v>0.5600000000000001</v>
+        <v>1.05</v>
       </c>
       <c r="AA33" s="4" t="n">
-        <v>22491</v>
+        <v>181512</v>
       </c>
       <c r="AB33" s="4" t="n">
-        <v>30.59369</v>
+        <v>76.230034</v>
       </c>
       <c r="AC33" s="4" t="n">
-        <v>20.760788</v>
+        <v>51.237114</v>
       </c>
       <c r="AD33" s="4" t="inlineStr"/>
       <c r="AE33" s="4" t="n">
-        <v>29.735</v>
+        <v>85.446</v>
       </c>
       <c r="AF33" s="4" t="n">
-        <v>22</v>
+        <v>54.8</v>
       </c>
       <c r="AG33" s="4" t="n">
-        <v>53.4</v>
+        <v>-8.199999999999999</v>
       </c>
       <c r="AH33" s="4" t="n">
-        <v>4.0178747</v>
+        <v>19.253426</v>
       </c>
       <c r="AI33" s="4" t="n">
-        <v>21</v>
+        <v>80</v>
       </c>
       <c r="AJ33" s="4" t="inlineStr"/>
       <c r="AK33" s="4" t="inlineStr">
         <is>
-          <t>https://www.screener.in/company/GRANULES/</t>
+          <t>https://www.screener.in/company/TORNTPHARM/</t>
         </is>
       </c>
       <c r="AL33" s="4" t="inlineStr">
         <is>
-          <t>https://www.tradingview.com/chart/?symbol=NSE:GRANULES</t>
+          <t>https://www.tradingview.com/chart/?symbol=NSE:TORNTPHARM</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>BEML</t>
+          <t>GRANULES</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>BEML Limited</t>
+          <t>Granules India Limited</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Healthcare</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Conglomerates</t>
+          <t>Drug Manufacturers - Specialty &amp; Generic</t>
         </is>
       </c>
       <c r="E34" s="6" t="n">
-        <v>38.2</v>
+        <v>38.3</v>
       </c>
       <c r="F34" s="2" t="n">
-        <v>21.6</v>
+        <v>19.2</v>
       </c>
       <c r="G34" s="2" t="n">
-        <v>16.6</v>
+        <v>19.1</v>
       </c>
       <c r="H34" s="6" t="inlineStr">
         <is>
@@ -4931,19 +4927,19 @@
         </is>
       </c>
       <c r="J34" s="2" t="n">
-        <v>1962.3</v>
+        <v>821.75</v>
       </c>
       <c r="K34" s="2" t="n">
-        <v>-1.51</v>
+        <v>-2.93</v>
       </c>
       <c r="L34" s="2" t="n">
-        <v>2008.6</v>
+        <v>858.76</v>
       </c>
       <c r="M34" s="2" t="n">
-        <v>1950.92</v>
+        <v>850.74</v>
       </c>
       <c r="N34" s="2" t="n">
-        <v>1855.54</v>
+        <v>743.47</v>
       </c>
       <c r="O34" s="2" t="inlineStr">
         <is>
@@ -4956,65 +4952,67 @@
         </is>
       </c>
       <c r="Q34" s="2" t="n">
-        <v>86.97</v>
+        <v>88.97</v>
       </c>
       <c r="R34" s="2" t="n">
-        <v>45.98</v>
+        <v>40.27</v>
       </c>
       <c r="S34" s="2" t="n">
-        <v>13.8206</v>
+        <v>-2.9133</v>
       </c>
       <c r="T34" s="2" t="n">
-        <v>30.6456</v>
+        <v>2.3115</v>
       </c>
       <c r="U34" s="2" t="n">
-        <v>-16.825</v>
+        <v>-5.2248</v>
       </c>
       <c r="V34" s="2" t="inlineStr"/>
       <c r="W34" s="2" t="n">
-        <v>20.78</v>
+        <v>20.15</v>
       </c>
       <c r="X34" s="2" t="n">
-        <v>198724</v>
+        <v>783432</v>
       </c>
       <c r="Y34" s="2" t="n">
-        <v>398370</v>
+        <v>1389889</v>
       </c>
       <c r="Z34" s="2" t="n">
-        <v>0.5</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="AA34" s="2" t="n">
-        <v>16325</v>
+        <v>22293</v>
       </c>
       <c r="AB34" s="2" t="n">
-        <v>90.95128</v>
+        <v>30.358469</v>
       </c>
       <c r="AC34" s="2" t="n">
-        <v>27.05314</v>
+        <v>20.878649</v>
       </c>
       <c r="AD34" s="2" t="inlineStr"/>
       <c r="AE34" s="2" t="n">
-        <v>10.529</v>
+        <v>29.735</v>
       </c>
       <c r="AF34" s="2" t="n">
-        <v>29.3</v>
-      </c>
-      <c r="AG34" s="2" t="inlineStr"/>
+        <v>22</v>
+      </c>
+      <c r="AG34" s="2" t="n">
+        <v>53.4</v>
+      </c>
       <c r="AH34" s="2" t="n">
-        <v>5.564293</v>
+        <v>3.9825447</v>
       </c>
       <c r="AI34" s="2" t="n">
-        <v>90</v>
+        <v>21</v>
       </c>
       <c r="AJ34" s="2" t="inlineStr"/>
       <c r="AK34" s="2" t="inlineStr">
         <is>
-          <t>https://www.screener.in/company/BEML/</t>
+          <t>https://www.screener.in/company/GRANULES/</t>
         </is>
       </c>
       <c r="AL34" s="2" t="inlineStr">
         <is>
-          <t>https://www.tradingview.com/chart/?symbol=NSE:BEML</t>
+          <t>https://www.tradingview.com/chart/?symbol=NSE:GRANULES</t>
         </is>
       </c>
     </row>
@@ -5071,7 +5069,7 @@
         <v>1146.49</v>
       </c>
       <c r="N35" s="4" t="n">
-        <v>1002.86</v>
+        <v>1005.15</v>
       </c>
       <c r="O35" s="4" t="inlineStr">
         <is>
@@ -5112,13 +5110,13 @@
         <v>0.53</v>
       </c>
       <c r="AA35" s="4" t="n">
-        <v>23723</v>
+        <v>23442</v>
       </c>
       <c r="AB35" s="4" t="n">
-        <v>38.86403</v>
+        <v>38.363136</v>
       </c>
       <c r="AC35" s="4" t="n">
-        <v>27.106842</v>
+        <v>26.785112</v>
       </c>
       <c r="AD35" s="4" t="inlineStr"/>
       <c r="AE35" s="4" t="n">
@@ -5131,7 +5129,7 @@
         <v>13.5</v>
       </c>
       <c r="AH35" s="4" t="n">
-        <v>5.549302</v>
+        <v>5.483438</v>
       </c>
       <c r="AI35" s="4" t="n">
         <v>76</v>
@@ -5201,7 +5199,7 @@
         <v>173.27</v>
       </c>
       <c r="N36" s="2" t="n">
-        <v>166.55</v>
+        <v>166.62</v>
       </c>
       <c r="O36" s="2" t="inlineStr">
         <is>
@@ -5245,7 +5243,7 @@
         <v>13342</v>
       </c>
       <c r="AB36" s="2" t="n">
-        <v>22.4096</v>
+        <v>22.700161</v>
       </c>
       <c r="AC36" s="2" t="n">
         <v>16.813925</v>
@@ -5325,7 +5323,7 @@
         <v>570.91</v>
       </c>
       <c r="N37" s="4" t="n">
-        <v>536.25</v>
+        <v>536.86</v>
       </c>
       <c r="O37" s="4" t="inlineStr">
         <is>
@@ -5366,13 +5364,13 @@
         <v>1.95</v>
       </c>
       <c r="AA37" s="4" t="n">
-        <v>11161</v>
+        <v>11485</v>
       </c>
       <c r="AB37" s="4" t="n">
-        <v>55.23614</v>
+        <v>57.013386</v>
       </c>
       <c r="AC37" s="4" t="n">
-        <v>34.707214</v>
+        <v>35.713593</v>
       </c>
       <c r="AD37" s="4" t="inlineStr"/>
       <c r="AE37" s="4" t="n">
@@ -5385,7 +5383,7 @@
         <v>12.7</v>
       </c>
       <c r="AH37" s="4" t="n">
-        <v>7.3714786</v>
+        <v>7.5852237</v>
       </c>
       <c r="AI37" s="4" t="n">
         <v>37</v>
@@ -5455,7 +5453,7 @@
         <v>177.66</v>
       </c>
       <c r="N38" s="2" t="n">
-        <v>166.32</v>
+        <v>166.23</v>
       </c>
       <c r="O38" s="2" t="inlineStr">
         <is>
@@ -5496,13 +5494,13 @@
         <v>1.68</v>
       </c>
       <c r="AA38" s="2" t="n">
-        <v>72078</v>
+        <v>73090</v>
       </c>
       <c r="AB38" s="2" t="n">
-        <v>17.53769</v>
+        <v>17.113152</v>
       </c>
       <c r="AC38" s="2" t="n">
-        <v>11.0012455</v>
+        <v>11.1557045</v>
       </c>
       <c r="AD38" s="2" t="inlineStr"/>
       <c r="AE38" s="2" t="n">
@@ -5515,7 +5513,7 @@
         <v>121.1</v>
       </c>
       <c r="AH38" s="2" t="n">
-        <v>1.1951972</v>
+        <v>1.211978</v>
       </c>
       <c r="AI38" s="2" t="n">
         <v>135</v>
@@ -5585,7 +5583,7 @@
         <v>516.25</v>
       </c>
       <c r="N39" s="4" t="n">
-        <v>496.04</v>
+        <v>497.6</v>
       </c>
       <c r="O39" s="4" t="inlineStr">
         <is>
@@ -5626,13 +5624,13 @@
         <v>0.34</v>
       </c>
       <c r="AA39" s="4" t="n">
-        <v>12583</v>
+        <v>12666</v>
       </c>
       <c r="AB39" s="4" t="n">
-        <v>32.589676</v>
+        <v>32.827454</v>
       </c>
       <c r="AC39" s="4" t="n">
-        <v>27.888237</v>
+        <v>28.074034</v>
       </c>
       <c r="AD39" s="4" t="inlineStr"/>
       <c r="AE39" s="4" t="n">
@@ -5645,7 +5643,7 @@
         <v>14.9</v>
       </c>
       <c r="AH39" s="4" t="n">
-        <v>6.3977118</v>
+        <v>6.4403343</v>
       </c>
       <c r="AI39" s="4" t="n">
         <v>149</v>
@@ -5715,7 +5713,7 @@
         <v>1319.84</v>
       </c>
       <c r="N40" s="2" t="n">
-        <v>1245.56</v>
+        <v>1246.6</v>
       </c>
       <c r="O40" s="2" t="inlineStr">
         <is>
@@ -5756,13 +5754,13 @@
         <v>4.54</v>
       </c>
       <c r="AA40" s="2" t="n">
-        <v>210196</v>
+        <v>211497</v>
       </c>
       <c r="AB40" s="2" t="n">
-        <v>121.998085</v>
+        <v>122.98851</v>
       </c>
       <c r="AC40" s="2" t="n">
-        <v>42.77577</v>
+        <v>43.040585</v>
       </c>
       <c r="AD40" s="2" t="inlineStr"/>
       <c r="AE40" s="2" t="n">
@@ -5775,7 +5773,7 @@
         <v>18.5</v>
       </c>
       <c r="AH40" s="2" t="n">
-        <v>10.896593</v>
+        <v>10.964051</v>
       </c>
       <c r="AI40" s="2" t="n">
         <v>0</v>
@@ -5845,7 +5843,7 @@
         <v>284.97</v>
       </c>
       <c r="N41" s="4" t="n">
-        <v>278.82</v>
+        <v>278.75</v>
       </c>
       <c r="O41" s="4" t="inlineStr">
         <is>
@@ -5886,13 +5884,13 @@
         <v>1.07</v>
       </c>
       <c r="AA41" s="4" t="n">
-        <v>42825</v>
+        <v>43500</v>
       </c>
       <c r="AB41" s="4" t="n">
-        <v>10.181883</v>
+        <v>10.334996</v>
       </c>
       <c r="AC41" s="4" t="n">
-        <v>10.044428</v>
+        <v>10.202746</v>
       </c>
       <c r="AD41" s="4" t="inlineStr"/>
       <c r="AE41" s="4" t="n">
@@ -5905,7 +5903,7 @@
         <v>35.1</v>
       </c>
       <c r="AH41" s="4" t="n">
-        <v>1.9213428</v>
+        <v>1.9516267</v>
       </c>
       <c r="AI41" s="4" t="n">
         <v>350</v>
@@ -5975,7 +5973,7 @@
         <v>4380.32</v>
       </c>
       <c r="N42" s="2" t="n">
-        <v>3760.81</v>
+        <v>3762.42</v>
       </c>
       <c r="O42" s="2" t="inlineStr">
         <is>
@@ -6016,13 +6014,13 @@
         <v>1.81</v>
       </c>
       <c r="AA42" s="2" t="n">
-        <v>56771</v>
+        <v>57469</v>
       </c>
       <c r="AB42" s="2" t="n">
-        <v>80.87421399999999</v>
+        <v>81.65049</v>
       </c>
       <c r="AC42" s="2" t="n">
-        <v>53.159748</v>
+        <v>53.80277</v>
       </c>
       <c r="AD42" s="2" t="inlineStr"/>
       <c r="AE42" s="2" t="n">
@@ -6035,7 +6033,7 @@
         <v>76</v>
       </c>
       <c r="AH42" s="2" t="n">
-        <v>17.110136</v>
+        <v>17.32053</v>
       </c>
       <c r="AI42" s="2" t="n">
         <v>21</v>
@@ -6105,7 +6103,7 @@
         <v>722.48</v>
       </c>
       <c r="N43" s="4" t="n">
-        <v>706.37</v>
+        <v>706.71</v>
       </c>
       <c r="O43" s="4" t="inlineStr">
         <is>
@@ -6146,13 +6144,13 @@
         <v>1.32</v>
       </c>
       <c r="AA43" s="4" t="n">
-        <v>103866</v>
+        <v>104879</v>
       </c>
       <c r="AB43" s="4" t="n">
-        <v>47.612732</v>
+        <v>48.108826</v>
       </c>
       <c r="AC43" s="4" t="n">
-        <v>38.487392</v>
+        <v>38.862617</v>
       </c>
       <c r="AD43" s="4" t="inlineStr"/>
       <c r="AE43" s="4" t="n">
@@ -6165,7 +6163,7 @@
         <v>20.7</v>
       </c>
       <c r="AH43" s="4" t="n">
-        <v>7.8302217</v>
+        <v>7.906561</v>
       </c>
       <c r="AI43" s="4" t="n">
         <v>45</v>
@@ -6235,7 +6233,7 @@
         <v>169.07</v>
       </c>
       <c r="N44" s="2" t="n">
-        <v>163.09</v>
+        <v>163.02</v>
       </c>
       <c r="O44" s="2" t="inlineStr">
         <is>
@@ -6276,13 +6274,13 @@
         <v>1.11</v>
       </c>
       <c r="AA44" s="2" t="n">
-        <v>28730</v>
+        <v>30220</v>
       </c>
       <c r="AB44" s="2" t="n">
-        <v>9.1427765</v>
+        <v>9.616842</v>
       </c>
       <c r="AC44" s="2" t="n">
-        <v>3.2017577</v>
+        <v>3.3677733</v>
       </c>
       <c r="AD44" s="2" t="inlineStr"/>
       <c r="AE44" s="2" t="n">
@@ -6293,7 +6291,7 @@
       </c>
       <c r="AG44" s="2" t="inlineStr"/>
       <c r="AH44" s="2" t="n">
-        <v>2.016235</v>
+        <v>2.1207798</v>
       </c>
       <c r="AI44" s="2" t="n">
         <v>243</v>
@@ -6363,7 +6361,7 @@
         <v>541.73</v>
       </c>
       <c r="N45" s="4" t="n">
-        <v>462.29</v>
+        <v>462.38</v>
       </c>
       <c r="O45" s="4" t="inlineStr">
         <is>
@@ -6404,13 +6402,13 @@
         <v>0.89</v>
       </c>
       <c r="AA45" s="4" t="n">
-        <v>14595</v>
+        <v>13904</v>
       </c>
       <c r="AB45" s="4" t="n">
-        <v>33.93422</v>
+        <v>33.569622</v>
       </c>
       <c r="AC45" s="4" t="n">
-        <v>20.840729</v>
+        <v>20.603771</v>
       </c>
       <c r="AD45" s="4" t="inlineStr"/>
       <c r="AE45" s="4" t="n">
@@ -6423,7 +6421,7 @@
         <v>0.5</v>
       </c>
       <c r="AH45" s="4" t="n">
-        <v>3.4771957</v>
+        <v>3.4376602</v>
       </c>
       <c r="AI45" s="4" t="n">
         <v>84</v>
@@ -6493,7 +6491,7 @@
         <v>4846.5</v>
       </c>
       <c r="N46" s="2" t="n">
-        <v>4448.31</v>
+        <v>4453.47</v>
       </c>
       <c r="O46" s="2" t="inlineStr">
         <is>
@@ -6534,13 +6532,13 @@
         <v>1.17</v>
       </c>
       <c r="AA46" s="2" t="n">
-        <v>400684</v>
+        <v>406389</v>
       </c>
       <c r="AB46" s="2" t="n">
-        <v>69.44025999999999</v>
+        <v>70.591866</v>
       </c>
       <c r="AC46" s="2" t="n">
-        <v>50.779655</v>
+        <v>51.485996</v>
       </c>
       <c r="AD46" s="2" t="inlineStr"/>
       <c r="AE46" s="2" t="n">
@@ -6553,7 +6551,7 @@
         <v>62.8</v>
       </c>
       <c r="AH46" s="2" t="n">
-        <v>25.530027</v>
+        <v>25.893553</v>
       </c>
       <c r="AI46" s="2" t="n">
         <v>33</v>
@@ -6623,7 +6621,7 @@
         <v>1353.4</v>
       </c>
       <c r="N47" s="4" t="n">
-        <v>1212.11</v>
+        <v>1214.3</v>
       </c>
       <c r="O47" s="4" t="inlineStr">
         <is>
@@ -6664,13 +6662,13 @@
         <v>0.5600000000000001</v>
       </c>
       <c r="AA47" s="4" t="n">
-        <v>25104</v>
+        <v>24981</v>
       </c>
       <c r="AB47" s="4" t="n">
-        <v>73.96951</v>
+        <v>67.50906000000001</v>
       </c>
       <c r="AC47" s="4" t="n">
-        <v>32.883587</v>
+        <v>32.794968</v>
       </c>
       <c r="AD47" s="4" t="inlineStr"/>
       <c r="AE47" s="4" t="n">
@@ -6683,7 +6681,7 @@
         <v>40.6</v>
       </c>
       <c r="AH47" s="4" t="n">
-        <v>13.769182</v>
+        <v>13.701913</v>
       </c>
       <c r="AI47" s="4" t="n">
         <v>38</v>
@@ -6753,7 +6751,7 @@
         <v>172.51</v>
       </c>
       <c r="N48" s="2" t="n">
-        <v>168.48</v>
+        <v>168.5</v>
       </c>
       <c r="O48" s="2" t="inlineStr">
         <is>
@@ -6794,13 +6792,13 @@
         <v>1.11</v>
       </c>
       <c r="AA48" s="2" t="n">
-        <v>112579</v>
+        <v>110133</v>
       </c>
       <c r="AB48" s="2" t="n">
-        <v>11.391883</v>
+        <v>11.144378</v>
       </c>
       <c r="AC48" s="2" t="n">
-        <v>9.30889</v>
+        <v>9.106642000000001</v>
       </c>
       <c r="AD48" s="2" t="inlineStr"/>
       <c r="AE48" s="2" t="n">
@@ -6813,7 +6811,7 @@
         <v>97.2</v>
       </c>
       <c r="AH48" s="2" t="n">
-        <v>1.2631595</v>
+        <v>1.2357155</v>
       </c>
       <c r="AI48" s="2" t="n">
         <v>321</v>
@@ -6883,7 +6881,7 @@
         <v>872.66</v>
       </c>
       <c r="N49" s="4" t="n">
-        <v>765.89</v>
+        <v>765.5700000000001</v>
       </c>
       <c r="O49" s="4" t="inlineStr">
         <is>
@@ -6924,13 +6922,13 @@
         <v>1.34</v>
       </c>
       <c r="AA49" s="4" t="n">
-        <v>9902</v>
+        <v>10060</v>
       </c>
       <c r="AB49" s="4" t="n">
-        <v>40.767918</v>
+        <v>41.47705</v>
       </c>
       <c r="AC49" s="4" t="n">
-        <v>22.710249</v>
+        <v>23.071484</v>
       </c>
       <c r="AD49" s="4" t="inlineStr"/>
       <c r="AE49" s="4" t="n">
@@ -6943,7 +6941,7 @@
         <v>101.5</v>
       </c>
       <c r="AH49" s="4" t="n">
-        <v>4.9229603</v>
+        <v>5.001266</v>
       </c>
       <c r="AI49" s="4" t="n">
         <v>0</v>
@@ -7013,7 +7011,7 @@
         <v>1809.08</v>
       </c>
       <c r="N50" s="2" t="n">
-        <v>1726.9</v>
+        <v>1728.07</v>
       </c>
       <c r="O50" s="2" t="inlineStr">
         <is>
@@ -7054,13 +7052,13 @@
         <v>0.65</v>
       </c>
       <c r="AA50" s="2" t="n">
-        <v>63798</v>
+        <v>63674</v>
       </c>
       <c r="AB50" s="2" t="n">
-        <v>24.238153</v>
+        <v>24.21795</v>
       </c>
       <c r="AC50" s="2" t="n">
-        <v>16.492826</v>
+        <v>16.460867</v>
       </c>
       <c r="AD50" s="2" t="inlineStr"/>
       <c r="AE50" s="2" t="n">
@@ -7073,7 +7071,7 @@
         <v>28.9</v>
       </c>
       <c r="AH50" s="2" t="n">
-        <v>3.5598135</v>
+        <v>3.5529153</v>
       </c>
       <c r="AI50" s="2" t="n">
         <v>46</v>
@@ -7139,7 +7137,7 @@
         <v>773.16</v>
       </c>
       <c r="N51" s="4" t="n">
-        <v>693.21</v>
+        <v>692.76</v>
       </c>
       <c r="O51" s="4" t="inlineStr">
         <is>
@@ -7180,13 +7178,13 @@
         <v>1.64</v>
       </c>
       <c r="AA51" s="4" t="n">
-        <v>3635</v>
+        <v>3488</v>
       </c>
       <c r="AB51" s="4" t="n">
-        <v>830.9091</v>
+        <v>89.38217</v>
       </c>
       <c r="AC51" s="4" t="n">
-        <v>37.11675</v>
+        <v>35.616753</v>
       </c>
       <c r="AD51" s="4" t="inlineStr"/>
       <c r="AE51" s="4" t="n">
@@ -7197,7 +7195,7 @@
       </c>
       <c r="AG51" s="4" t="inlineStr"/>
       <c r="AH51" s="4" t="n">
-        <v>5.2823215</v>
+        <v>5.0688467</v>
       </c>
       <c r="AI51" s="4" t="n">
         <v>0</v>
@@ -7267,7 +7265,7 @@
         <v>2969.73</v>
       </c>
       <c r="N52" s="2" t="n">
-        <v>2719.38</v>
+        <v>2722.54</v>
       </c>
       <c r="O52" s="2" t="inlineStr">
         <is>
@@ -7308,13 +7306,13 @@
         <v>1.41</v>
       </c>
       <c r="AA52" s="2" t="n">
-        <v>381317</v>
+        <v>387706</v>
       </c>
       <c r="AB52" s="2" t="n">
-        <v>49.02193</v>
+        <v>46.156326</v>
       </c>
       <c r="AC52" s="2" t="n">
-        <v>42.782505</v>
+        <v>43.499393</v>
       </c>
       <c r="AD52" s="2" t="inlineStr"/>
       <c r="AE52" s="2" t="n">
@@ -7325,7 +7323,7 @@
       </c>
       <c r="AG52" s="2" t="inlineStr"/>
       <c r="AH52" s="2" t="n">
-        <v>4.499458</v>
+        <v>4.5748534</v>
       </c>
       <c r="AI52" s="2" t="n">
         <v>5</v>
@@ -7395,7 +7393,7 @@
         <v>4783.38</v>
       </c>
       <c r="N53" s="4" t="n">
-        <v>4169.99</v>
+        <v>4173.46</v>
       </c>
       <c r="O53" s="4" t="inlineStr">
         <is>
@@ -7436,13 +7434,13 @@
         <v>0.75</v>
       </c>
       <c r="AA53" s="4" t="n">
-        <v>26858</v>
+        <v>28327</v>
       </c>
       <c r="AB53" s="4" t="n">
-        <v>97.983086</v>
+        <v>103.81481</v>
       </c>
       <c r="AC53" s="4" t="n">
-        <v>54.143642</v>
+        <v>57.104885</v>
       </c>
       <c r="AD53" s="4" t="inlineStr"/>
       <c r="AE53" s="4" t="n">
@@ -7455,7 +7453,7 @@
         <v>178.4</v>
       </c>
       <c r="AH53" s="4" t="n">
-        <v>35.474804</v>
+        <v>37.415005</v>
       </c>
       <c r="AI53" s="4" t="n">
         <v>7</v>
@@ -7525,7 +7523,7 @@
         <v>511.42</v>
       </c>
       <c r="N54" s="2" t="n">
-        <v>460.71</v>
+        <v>460.88</v>
       </c>
       <c r="O54" s="2" t="inlineStr">
         <is>
@@ -7566,13 +7564,13 @@
         <v>0.79</v>
       </c>
       <c r="AA54" s="2" t="n">
-        <v>6492</v>
+        <v>6274</v>
       </c>
       <c r="AB54" s="2" t="n">
-        <v>29.495548</v>
+        <v>28.763472</v>
       </c>
       <c r="AC54" s="2" t="n">
-        <v>21.894272</v>
+        <v>21.160793</v>
       </c>
       <c r="AD54" s="2" t="inlineStr"/>
       <c r="AE54" s="2" t="n">
@@ -7585,7 +7583,7 @@
         <v>95.7</v>
       </c>
       <c r="AH54" s="2" t="n">
-        <v>8.81362</v>
+        <v>8.518354</v>
       </c>
       <c r="AI54" s="2" t="n">
         <v>0</v>
@@ -7655,7 +7653,7 @@
         <v>562.91</v>
       </c>
       <c r="N55" s="4" t="n">
-        <v>506.78</v>
+        <v>507.24</v>
       </c>
       <c r="O55" s="4" t="inlineStr">
         <is>
@@ -7696,13 +7694,13 @@
         <v>1.01</v>
       </c>
       <c r="AA55" s="4" t="n">
-        <v>8451</v>
+        <v>8627</v>
       </c>
       <c r="AB55" s="4" t="n">
-        <v>48.185116</v>
+        <v>49.187836</v>
       </c>
       <c r="AC55" s="4" t="n">
-        <v>33.387825</v>
+        <v>34.08262</v>
       </c>
       <c r="AD55" s="4" t="inlineStr"/>
       <c r="AE55" s="4" t="n">
@@ -7715,10 +7713,10 @@
         <v>31.8</v>
       </c>
       <c r="AH55" s="4" t="n">
-        <v>14.434839</v>
+        <v>14.735226</v>
       </c>
       <c r="AI55" s="4" t="n">
-        <v>306</v>
+        <v>175</v>
       </c>
       <c r="AJ55" s="4" t="inlineStr"/>
       <c r="AK55" s="4" t="inlineStr">
@@ -7782,10 +7780,10 @@
         <v>1550.61</v>
       </c>
       <c r="M56" s="2" t="n">
-        <v>1554.52</v>
+        <v>1554.51</v>
       </c>
       <c r="N56" s="2" t="n">
-        <v>1500.05</v>
+        <v>1498.06</v>
       </c>
       <c r="O56" s="2" t="inlineStr">
         <is>
@@ -7826,13 +7824,13 @@
         <v>1.53</v>
       </c>
       <c r="AA56" s="2" t="n">
-        <v>135812</v>
+        <v>136069</v>
       </c>
       <c r="AB56" s="2" t="n">
-        <v>26.385542</v>
+        <v>26.554289</v>
       </c>
       <c r="AC56" s="2" t="n">
-        <v>17.49139</v>
+        <v>17.495626</v>
       </c>
       <c r="AD56" s="2" t="inlineStr"/>
       <c r="AE56" s="2" t="n">
@@ -7845,7 +7843,7 @@
         <v>28.3</v>
       </c>
       <c r="AH56" s="2" t="n">
-        <v>4.5842204</v>
+        <v>4.5928926</v>
       </c>
       <c r="AI56" s="2" t="n">
         <v>333</v>
@@ -8409,7 +8407,7 @@
         <v>406.67</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>399.74</v>
+        <v>399.9</v>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
@@ -8450,13 +8448,13 @@
         <v>4.73</v>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>416170</v>
+        <v>413832</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>20.487268</v>
+        <v>20.392157</v>
       </c>
       <c r="AC2" s="2" t="n">
-        <v>17.80935</v>
+        <v>17.709309</v>
       </c>
       <c r="AD2" s="2" t="inlineStr"/>
       <c r="AE2" s="2" t="inlineStr"/>
@@ -8467,7 +8465,7 @@
         <v>22.5</v>
       </c>
       <c r="AH2" s="2" t="n">
-        <v>2.2960906</v>
+        <v>2.2831926</v>
       </c>
       <c r="AI2" s="2" t="n">
         <v>16</v>
@@ -8537,7 +8535,7 @@
         <v>197.46</v>
       </c>
       <c r="N3" s="4" t="n">
-        <v>159.68</v>
+        <v>159.85</v>
       </c>
       <c r="O3" s="4" t="inlineStr">
         <is>
@@ -8578,13 +8576,13 @@
         <v>4.27</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>22501</v>
+        <v>21679</v>
       </c>
       <c r="AB3" s="4" t="n">
-        <v>78.10457599999999</v>
+        <v>79.40345000000001</v>
       </c>
       <c r="AC3" s="4" t="n">
-        <v>25.921907</v>
+        <v>24.975054</v>
       </c>
       <c r="AD3" s="4" t="inlineStr"/>
       <c r="AE3" s="4" t="n">
@@ -8597,7 +8595,7 @@
         <v>83.7</v>
       </c>
       <c r="AH3" s="4" t="n">
-        <v>4.6616864</v>
+        <v>4.491408</v>
       </c>
       <c r="AI3" s="4" t="n">
         <v>4</v>
@@ -8667,7 +8665,7 @@
         <v>218.67</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>163.47</v>
+        <v>163.55</v>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
@@ -8712,13 +8710,13 @@
         <v>3.43</v>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>36477</v>
+        <v>38298</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>62.07552</v>
+        <v>65.17448400000001</v>
       </c>
       <c r="AC4" s="2" t="n">
-        <v>45.840385</v>
+        <v>48.12885</v>
       </c>
       <c r="AD4" s="2" t="inlineStr"/>
       <c r="AE4" s="2" t="n">
@@ -8729,7 +8727,7 @@
       </c>
       <c r="AG4" s="2" t="inlineStr"/>
       <c r="AH4" s="2" t="n">
-        <v>7.1899977</v>
+        <v>7.5489397</v>
       </c>
       <c r="AI4" s="2" t="n">
         <v>8</v>
@@ -8844,13 +8842,13 @@
         <v>1.53</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>3797</v>
+        <v>3853</v>
       </c>
       <c r="AB5" s="4" t="n">
-        <v>38.48101</v>
+        <v>38.994946</v>
       </c>
       <c r="AC5" s="4" t="n">
-        <v>18.164751</v>
+        <v>18.43065</v>
       </c>
       <c r="AD5" s="4" t="inlineStr"/>
       <c r="AE5" s="4" t="n">
@@ -8863,7 +8861,7 @@
         <v>32</v>
       </c>
       <c r="AH5" s="4" t="n">
-        <v>4.2089524</v>
+        <v>4.270564</v>
       </c>
       <c r="AI5" s="4" t="n">
         <v>16</v>
@@ -9180,7 +9178,7 @@
         <v>406.67</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>399.74</v>
+        <v>399.9</v>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
@@ -9221,13 +9219,13 @@
         <v>4.73</v>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>416170</v>
+        <v>413832</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>20.487268</v>
+        <v>20.392157</v>
       </c>
       <c r="AC2" s="2" t="n">
-        <v>17.80935</v>
+        <v>17.709309</v>
       </c>
       <c r="AD2" s="2" t="inlineStr"/>
       <c r="AE2" s="2" t="inlineStr"/>
@@ -9238,7 +9236,7 @@
         <v>22.5</v>
       </c>
       <c r="AH2" s="2" t="n">
-        <v>2.2960906</v>
+        <v>2.2831926</v>
       </c>
       <c r="AI2" s="2" t="n">
         <v>16</v>
@@ -9308,7 +9306,7 @@
         <v>197.46</v>
       </c>
       <c r="N3" s="4" t="n">
-        <v>159.68</v>
+        <v>159.85</v>
       </c>
       <c r="O3" s="4" t="inlineStr">
         <is>
@@ -9349,13 +9347,13 @@
         <v>4.27</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>22501</v>
+        <v>21679</v>
       </c>
       <c r="AB3" s="4" t="n">
-        <v>78.10457599999999</v>
+        <v>79.40345000000001</v>
       </c>
       <c r="AC3" s="4" t="n">
-        <v>25.921907</v>
+        <v>24.975054</v>
       </c>
       <c r="AD3" s="4" t="inlineStr"/>
       <c r="AE3" s="4" t="n">
@@ -9368,7 +9366,7 @@
         <v>83.7</v>
       </c>
       <c r="AH3" s="4" t="n">
-        <v>4.6616864</v>
+        <v>4.491408</v>
       </c>
       <c r="AI3" s="4" t="n">
         <v>4</v>
@@ -9438,7 +9436,7 @@
         <v>218.67</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>163.47</v>
+        <v>163.55</v>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
@@ -9483,13 +9481,13 @@
         <v>3.43</v>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>36477</v>
+        <v>38298</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>62.07552</v>
+        <v>65.17448400000001</v>
       </c>
       <c r="AC4" s="2" t="n">
-        <v>45.840385</v>
+        <v>48.12885</v>
       </c>
       <c r="AD4" s="2" t="inlineStr"/>
       <c r="AE4" s="2" t="n">
@@ -9500,7 +9498,7 @@
       </c>
       <c r="AG4" s="2" t="inlineStr"/>
       <c r="AH4" s="2" t="n">
-        <v>7.1899977</v>
+        <v>7.5489397</v>
       </c>
       <c r="AI4" s="2" t="n">
         <v>8</v>
@@ -9615,13 +9613,13 @@
         <v>1.53</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>3797</v>
+        <v>3853</v>
       </c>
       <c r="AB5" s="4" t="n">
-        <v>38.48101</v>
+        <v>38.994946</v>
       </c>
       <c r="AC5" s="4" t="n">
-        <v>18.164751</v>
+        <v>18.43065</v>
       </c>
       <c r="AD5" s="4" t="inlineStr"/>
       <c r="AE5" s="4" t="n">
@@ -9634,7 +9632,7 @@
         <v>32</v>
       </c>
       <c r="AH5" s="4" t="n">
-        <v>4.2089524</v>
+        <v>4.270564</v>
       </c>
       <c r="AI5" s="4" t="n">
         <v>16</v>
@@ -9677,7 +9675,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Run Date: 02-Oct-2026 15:15 IST</t>
+          <t>Run Date: 05-Oct-2026 17:37 IST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
@@ -9781,7 +9779,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>41.7</v>
+        <v>41.8</v>
       </c>
     </row>
     <row r="14">

</xml_diff>

<commit_message>
📈 Daily Screener Report — 13-Oct-2026 22:09 IST
</commit_message>
<xml_diff>
--- a/output/swing_screener_report.xlsx
+++ b/output/swing_screener_report.xlsx
@@ -816,13 +816,13 @@
         <v>1.44</v>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>441089</v>
+        <v>436712</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>21.735294</v>
+        <v>21.636272</v>
       </c>
       <c r="AC2" s="2" t="n">
-        <v>18.875738</v>
+        <v>18.688429</v>
       </c>
       <c r="AD2" s="2" t="inlineStr"/>
       <c r="AE2" s="2" t="inlineStr"/>
@@ -833,7 +833,7 @@
         <v>22.5</v>
       </c>
       <c r="AH2" s="2" t="n">
-        <v>2.433576</v>
+        <v>2.409427</v>
       </c>
       <c r="AI2" s="2" t="n">
         <v>15</v>
@@ -944,13 +944,13 @@
         <v>1.76</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>90785</v>
+        <v>93938</v>
       </c>
       <c r="AB3" s="4" t="n">
-        <v>47.376175</v>
+        <v>49.1666</v>
       </c>
       <c r="AC3" s="4" t="n">
-        <v>32.53733</v>
+        <v>33.667515</v>
       </c>
       <c r="AD3" s="4" t="n">
         <v>25.2</v>
@@ -965,7 +965,7 @@
         <v>12.1</v>
       </c>
       <c r="AH3" s="4" t="n">
-        <v>10.753688</v>
+        <v>11.127195</v>
       </c>
       <c r="AI3" s="4" t="n">
         <v>62</v>
@@ -1082,13 +1082,13 @@
         <v>0.9</v>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>133318</v>
+        <v>133950</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>6.0479665</v>
+        <v>6.0263705</v>
       </c>
       <c r="AC4" s="2" t="n">
-        <v>6.671329</v>
+        <v>6.7029605</v>
       </c>
       <c r="AD4" s="2" t="n">
         <v>14.97</v>
@@ -1101,10 +1101,10 @@
         <v>175</v>
       </c>
       <c r="AH4" s="2" t="n">
-        <v>0.85260266</v>
+        <v>0.85664517</v>
       </c>
       <c r="AI4" s="2" t="n">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="AJ4" s="2" t="inlineStr"/>
       <c r="AK4" s="2" t="inlineStr">
@@ -1212,13 +1212,13 @@
         <v>0.47</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>30446</v>
+        <v>30826</v>
       </c>
       <c r="AB5" s="4" t="n">
-        <v>9.688789</v>
+        <v>9.898142999999999</v>
       </c>
       <c r="AC5" s="4" t="n">
-        <v>3.3830576</v>
+        <v>3.4253166</v>
       </c>
       <c r="AD5" s="4" t="inlineStr"/>
       <c r="AE5" s="4" t="n">
@@ -1229,10 +1229,10 @@
       </c>
       <c r="AG5" s="4" t="inlineStr"/>
       <c r="AH5" s="4" t="n">
-        <v>2.136646</v>
+        <v>2.1633356</v>
       </c>
       <c r="AI5" s="4" t="n">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="AJ5" s="4" t="inlineStr"/>
       <c r="AK5" s="4" t="inlineStr">
@@ -1340,13 +1340,13 @@
         <v>1.04</v>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>81812</v>
+        <v>85462</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>37.816914</v>
+        <v>39.056488</v>
       </c>
       <c r="AC6" s="2" t="n">
-        <v>25.854103</v>
+        <v>27.007778</v>
       </c>
       <c r="AD6" s="2" t="inlineStr"/>
       <c r="AE6" s="2" t="n">
@@ -1359,10 +1359,10 @@
         <v>30.9</v>
       </c>
       <c r="AH6" s="2" t="n">
-        <v>6.5029597</v>
+        <v>6.793138</v>
       </c>
       <c r="AI6" s="2" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="AJ6" s="2" t="inlineStr"/>
       <c r="AK6" s="2" t="inlineStr">
@@ -1470,13 +1470,13 @@
         <v>1.24</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>40625</v>
+        <v>40093</v>
       </c>
       <c r="AB7" s="4" t="n">
-        <v>69.13542</v>
+        <v>69.496025</v>
       </c>
       <c r="AC7" s="4" t="n">
-        <v>51.05385</v>
+        <v>50.384617</v>
       </c>
       <c r="AD7" s="4" t="inlineStr"/>
       <c r="AE7" s="4" t="n">
@@ -1487,7 +1487,7 @@
       </c>
       <c r="AG7" s="4" t="inlineStr"/>
       <c r="AH7" s="4" t="n">
-        <v>8.007721999999999</v>
+        <v>7.902754</v>
       </c>
       <c r="AI7" s="4" t="n">
         <v>8</v>
@@ -1598,13 +1598,13 @@
         <v>0.59</v>
       </c>
       <c r="AA8" s="2" t="n">
-        <v>50895</v>
+        <v>48859</v>
       </c>
       <c r="AB8" s="2" t="n">
-        <v>40.67321</v>
+        <v>40.761345</v>
       </c>
       <c r="AC8" s="2" t="n">
-        <v>34.444744</v>
+        <v>33.06695</v>
       </c>
       <c r="AD8" s="2" t="inlineStr"/>
       <c r="AE8" s="2" t="n">
@@ -1617,10 +1617,10 @@
         <v>269</v>
       </c>
       <c r="AH8" s="2" t="n">
-        <v>8.405408</v>
+        <v>8.069191</v>
       </c>
       <c r="AI8" s="2" t="n">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="AJ8" s="2" t="inlineStr"/>
       <c r="AK8" s="2" t="inlineStr">
@@ -1728,13 +1728,13 @@
         <v>0.51</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>21343</v>
+        <v>21289</v>
       </c>
       <c r="AB9" s="4" t="n">
-        <v>78.17241</v>
+        <v>79.06644</v>
       </c>
       <c r="AC9" s="4" t="n">
-        <v>24.45523</v>
+        <v>24.393744</v>
       </c>
       <c r="AD9" s="4" t="inlineStr"/>
       <c r="AE9" s="4" t="n">
@@ -1747,7 +1747,7 @@
         <v>83.7</v>
       </c>
       <c r="AH9" s="4" t="n">
-        <v>4.4217753</v>
+        <v>4.4106574</v>
       </c>
       <c r="AI9" s="4" t="n">
         <v>4</v>
@@ -1858,13 +1858,13 @@
         <v>0.77</v>
       </c>
       <c r="AA10" s="2" t="n">
-        <v>250231</v>
+        <v>246488</v>
       </c>
       <c r="AB10" s="2" t="n">
-        <v>85.527626</v>
+        <v>85.02746999999999</v>
       </c>
       <c r="AC10" s="2" t="n">
-        <v>62.37426</v>
+        <v>61.39353</v>
       </c>
       <c r="AD10" s="2" t="inlineStr"/>
       <c r="AE10" s="2" t="n">
@@ -1877,7 +1877,7 @@
         <v>65.7</v>
       </c>
       <c r="AH10" s="2" t="n">
-        <v>14.929344</v>
+        <v>14.706021</v>
       </c>
       <c r="AI10" s="2" t="n">
         <v>32</v>
@@ -1897,32 +1897,32 @@
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>BHEL</t>
+          <t>FILATEX</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Bharat Heavy Electricals Limited</t>
+          <t>Filatex India Limited</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Consumer Cyclical</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Specialty Industrial Machinery</t>
+          <t>Textile Manufacturing</t>
         </is>
       </c>
       <c r="E11" s="5" t="n">
-        <v>53.90000000000001</v>
+        <v>54.3</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>32.2</v>
+        <v>35.4</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>21.7</v>
+        <v>18.9</v>
       </c>
       <c r="H11" s="5" t="inlineStr">
         <is>
@@ -1931,23 +1931,23 @@
       </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>✅ Supertrend Buy | 📈 EMA Bull Stack | 🏆 Near 52W High | 📉 Tight Base</t>
+          <t>✅ Supertrend Buy | 📈 EMA Bull Stack | 🏆 Near 52W High</t>
         </is>
       </c>
       <c r="J11" s="4" t="n">
-        <v>433.6</v>
+        <v>109.06</v>
       </c>
       <c r="K11" s="4" t="n">
-        <v>0.93</v>
+        <v>-0.62</v>
       </c>
       <c r="L11" s="4" t="n">
-        <v>427.96</v>
+        <v>101.73</v>
       </c>
       <c r="M11" s="4" t="n">
-        <v>420.93</v>
+        <v>89.47</v>
       </c>
       <c r="N11" s="4" t="n">
-        <v>363.41</v>
+        <v>66.42</v>
       </c>
       <c r="O11" s="4" t="inlineStr">
         <is>
@@ -1960,77 +1960,79 @@
         </is>
       </c>
       <c r="Q11" s="4" t="n">
-        <v>95.09999999999999</v>
+        <v>95.18000000000001</v>
       </c>
       <c r="R11" s="4" t="n">
-        <v>53.53</v>
+        <v>64.39</v>
       </c>
       <c r="S11" s="4" t="n">
-        <v>3.5281</v>
+        <v>7.5175</v>
       </c>
       <c r="T11" s="4" t="n">
-        <v>2.0492</v>
+        <v>7.5576</v>
       </c>
       <c r="U11" s="4" t="n">
-        <v>1.479</v>
+        <v>-0.0401</v>
       </c>
       <c r="V11" s="4" t="inlineStr"/>
       <c r="W11" s="4" t="n">
-        <v>16.42</v>
+        <v>44.9</v>
       </c>
       <c r="X11" s="4" t="n">
-        <v>11017851</v>
+        <v>1524085</v>
       </c>
       <c r="Y11" s="4" t="n">
-        <v>8664006</v>
+        <v>7397650</v>
       </c>
       <c r="Z11" s="4" t="n">
-        <v>1.27</v>
+        <v>0.21</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>153176</v>
+        <v>4722</v>
       </c>
       <c r="AB11" s="4" t="n">
-        <v>62.932762</v>
+        <v>24.445976</v>
       </c>
       <c r="AC11" s="4" t="n">
-        <v>31.458887</v>
+        <v>8.001505</v>
       </c>
       <c r="AD11" s="4" t="inlineStr"/>
       <c r="AE11" s="4" t="n">
-        <v>31.312</v>
+        <v>9.988</v>
       </c>
       <c r="AF11" s="4" t="n">
-        <v>40.3</v>
-      </c>
-      <c r="AG11" s="4" t="inlineStr"/>
+        <v>9.1</v>
+      </c>
+      <c r="AG11" s="4" t="n">
+        <v>18.5</v>
+      </c>
       <c r="AH11" s="4" t="n">
-        <v>5.8583817</v>
+        <v>3.1470847</v>
       </c>
       <c r="AI11" s="4" t="n">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="AJ11" s="4" t="inlineStr"/>
       <c r="AK11" s="4" t="inlineStr">
         <is>
-          <t>https://www.screener.in/company/BHEL/</t>
+          <t>https://www.screener.in/company/FILATEX/</t>
         </is>
       </c>
       <c r="AL11" s="4" t="inlineStr">
         <is>
-          <t>https://www.tradingview.com/chart/?symbol=NSE:BHEL</t>
+          <t>https://www.tradingview.com/chart/?symbol=NSE:FILATEX</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>BHEL</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Adani Ports and Special Economic Zone Limited</t>
+          <t>Bharat Heavy Electricals Limited</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -2040,17 +2042,17 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Marine Shipping</t>
+          <t>Specialty Industrial Machinery</t>
         </is>
       </c>
       <c r="E12" s="5" t="n">
-        <v>53.7</v>
+        <v>53.90000000000001</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>33</v>
+        <v>32.2</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>20.7</v>
+        <v>21.7</v>
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
@@ -2059,23 +2061,23 @@
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>✅ Supertrend Buy | 📈 EMA Bull Stack | 📊 High Volume | 🏆 Near 52W High | 📉 Tight Base</t>
+          <t>✅ Supertrend Buy | 📈 EMA Bull Stack | 🏆 Near 52W High | 📉 Tight Base</t>
         </is>
       </c>
       <c r="J12" s="2" t="n">
-        <v>1761</v>
+        <v>433.6</v>
       </c>
       <c r="K12" s="2" t="n">
-        <v>3.1</v>
+        <v>0.93</v>
       </c>
       <c r="L12" s="2" t="n">
-        <v>1757.28</v>
+        <v>427.96</v>
       </c>
       <c r="M12" s="2" t="n">
-        <v>1745.28</v>
+        <v>420.93</v>
       </c>
       <c r="N12" s="2" t="n">
-        <v>1651.87</v>
+        <v>363.41</v>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
@@ -2088,99 +2090,97 @@
         </is>
       </c>
       <c r="Q12" s="2" t="n">
-        <v>93.12</v>
+        <v>95.09999999999999</v>
       </c>
       <c r="R12" s="2" t="n">
-        <v>50.94</v>
+        <v>53.53</v>
       </c>
       <c r="S12" s="2" t="n">
-        <v>6.9333</v>
+        <v>3.5281</v>
       </c>
       <c r="T12" s="2" t="n">
-        <v>13.4209</v>
+        <v>2.0492</v>
       </c>
       <c r="U12" s="2" t="n">
-        <v>-6.4875</v>
+        <v>1.479</v>
       </c>
       <c r="V12" s="2" t="inlineStr"/>
       <c r="W12" s="2" t="n">
-        <v>17.79</v>
+        <v>16.42</v>
       </c>
       <c r="X12" s="2" t="n">
-        <v>9906351</v>
+        <v>11017851</v>
       </c>
       <c r="Y12" s="2" t="n">
-        <v>2433695</v>
+        <v>8664006</v>
       </c>
       <c r="Z12" s="2" t="n">
-        <v>4.07</v>
+        <v>1.27</v>
       </c>
       <c r="AA12" s="2" t="n">
-        <v>404114</v>
+        <v>154029</v>
       </c>
       <c r="AB12" s="2" t="n">
-        <v>29.93685</v>
+        <v>64.20174400000001</v>
       </c>
       <c r="AC12" s="2" t="n">
-        <v>22.425175</v>
+        <v>31.634096</v>
       </c>
       <c r="AD12" s="2" t="inlineStr"/>
       <c r="AE12" s="2" t="n">
-        <v>64.051</v>
+        <v>31.312</v>
       </c>
       <c r="AF12" s="2" t="n">
-        <v>18.6</v>
-      </c>
-      <c r="AG12" s="2" t="n">
-        <v>2.4</v>
-      </c>
+        <v>40.3</v>
+      </c>
+      <c r="AG12" s="2" t="inlineStr"/>
       <c r="AH12" s="2" t="n">
-        <v>4.211335</v>
+        <v>5.89101</v>
       </c>
       <c r="AI12" s="2" t="n">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="AJ12" s="2" t="inlineStr"/>
       <c r="AK12" s="2" t="inlineStr">
         <is>
-          <t>https://www.screener.in/company/ADANIPORTS/</t>
+          <t>https://www.screener.in/company/BHEL/</t>
         </is>
       </c>
       <c r="AL12" s="2" t="inlineStr">
         <is>
-          <t>https://www.tradingview.com/chart/?symbol=NSE:ADANIPORTS</t>
+          <t>https://www.tradingview.com/chart/?symbol=NSE:BHEL</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>GREENPLY</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Greenply Industries Limited</t>
+          <t>Adani Ports and Special Economic Zone Limited</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Basic Materials</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>Lumber &amp; Wood Production</t>
+          <t>Marine Shipping</t>
         </is>
       </c>
       <c r="E13" s="5" t="n">
-        <v>53.40000000000001</v>
+        <v>53.7</v>
       </c>
       <c r="F13" s="4" t="n">
-        <v>32.2</v>
+        <v>33</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>21.2</v>
+        <v>20.7</v>
       </c>
       <c r="H13" s="5" t="inlineStr">
         <is>
@@ -2189,23 +2189,23 @@
       </c>
       <c r="I13" s="4" t="inlineStr">
         <is>
-          <t>✅ Supertrend Buy | 📈 EMA Bull Stack | 🏆 Near 52W High | 📉 Tight Base</t>
+          <t>✅ Supertrend Buy | 📈 EMA Bull Stack | 📊 High Volume | 🏆 Near 52W High | 📉 Tight Base</t>
         </is>
       </c>
       <c r="J13" s="4" t="n">
-        <v>306.7</v>
+        <v>1761</v>
       </c>
       <c r="K13" s="4" t="n">
-        <v>0.33</v>
+        <v>3.1</v>
       </c>
       <c r="L13" s="4" t="n">
-        <v>298.66</v>
+        <v>1757.28</v>
       </c>
       <c r="M13" s="4" t="n">
-        <v>294.21</v>
+        <v>1745.28</v>
       </c>
       <c r="N13" s="4" t="n">
-        <v>279.76</v>
+        <v>1651.87</v>
       </c>
       <c r="O13" s="4" t="inlineStr">
         <is>
@@ -2218,67 +2218,67 @@
         </is>
       </c>
       <c r="Q13" s="4" t="n">
-        <v>91.88</v>
+        <v>93.12</v>
       </c>
       <c r="R13" s="4" t="n">
-        <v>57.05</v>
+        <v>50.94</v>
       </c>
       <c r="S13" s="4" t="n">
-        <v>4.4258</v>
+        <v>6.9333</v>
       </c>
       <c r="T13" s="4" t="n">
-        <v>2.5512</v>
+        <v>13.4209</v>
       </c>
       <c r="U13" s="4" t="n">
-        <v>1.8745</v>
+        <v>-6.4875</v>
       </c>
       <c r="V13" s="4" t="inlineStr"/>
       <c r="W13" s="4" t="n">
-        <v>16.09</v>
+        <v>17.79</v>
       </c>
       <c r="X13" s="4" t="n">
-        <v>126215</v>
+        <v>9906351</v>
       </c>
       <c r="Y13" s="4" t="n">
-        <v>239993</v>
+        <v>2433695</v>
       </c>
       <c r="Z13" s="4" t="n">
-        <v>0.53</v>
+        <v>4.07</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>3909</v>
+        <v>406188</v>
       </c>
       <c r="AB13" s="4" t="n">
-        <v>39.570164</v>
+        <v>29.9728</v>
       </c>
       <c r="AC13" s="4" t="n">
-        <v>18.670639</v>
+        <v>22.540241</v>
       </c>
       <c r="AD13" s="4" t="inlineStr"/>
       <c r="AE13" s="4" t="n">
-        <v>57.505</v>
+        <v>64.051</v>
       </c>
       <c r="AF13" s="4" t="n">
-        <v>20.7</v>
+        <v>18.6</v>
       </c>
       <c r="AG13" s="4" t="n">
-        <v>32</v>
+        <v>2.4</v>
       </c>
       <c r="AH13" s="4" t="n">
-        <v>4.3335595</v>
+        <v>4.232944</v>
       </c>
       <c r="AI13" s="4" t="n">
-        <v>16</v>
+        <v>43</v>
       </c>
       <c r="AJ13" s="4" t="inlineStr"/>
       <c r="AK13" s="4" t="inlineStr">
         <is>
-          <t>https://www.screener.in/company/GREENPLY/</t>
+          <t>https://www.screener.in/company/ADANIPORTS/</t>
         </is>
       </c>
       <c r="AL13" s="4" t="inlineStr">
         <is>
-          <t>https://www.tradingview.com/chart/?symbol=NSE:GREENPLY</t>
+          <t>https://www.tradingview.com/chart/?symbol=NSE:ADANIPORTS</t>
         </is>
       </c>
     </row>
@@ -2380,13 +2380,13 @@
         <v>0.37</v>
       </c>
       <c r="AA14" s="2" t="n">
-        <v>26852</v>
+        <v>27057</v>
       </c>
       <c r="AB14" s="2" t="n">
-        <v>72.56344</v>
+        <v>75.22110000000001</v>
       </c>
       <c r="AC14" s="2" t="n">
-        <v>34.60821</v>
+        <v>34.872494</v>
       </c>
       <c r="AD14" s="2" t="inlineStr"/>
       <c r="AE14" s="2" t="n">
@@ -2399,10 +2399,10 @@
         <v>40.6</v>
       </c>
       <c r="AH14" s="2" t="n">
-        <v>14.727769</v>
+        <v>14.840236</v>
       </c>
       <c r="AI14" s="2" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="AJ14" s="2" t="inlineStr"/>
       <c r="AK14" s="2" t="inlineStr">
@@ -2511,10 +2511,10 @@
       </c>
       <c r="AA15" s="4" t="inlineStr"/>
       <c r="AB15" s="4" t="n">
-        <v>70.80200000000001</v>
+        <v>70.57819000000001</v>
       </c>
       <c r="AC15" s="4" t="n">
-        <v>41.320282</v>
+        <v>40.320793</v>
       </c>
       <c r="AD15" s="4" t="inlineStr"/>
       <c r="AE15" s="4" t="n">
@@ -2527,7 +2527,7 @@
         <v>103.4</v>
       </c>
       <c r="AH15" s="4" t="n">
-        <v>20.50308</v>
+        <v>20.007137</v>
       </c>
       <c r="AI15" s="4" t="n">
         <v>24</v>
@@ -2547,12 +2547,12 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>FILATEX</t>
+          <t>NYKAA</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Filatex India Limited</t>
+          <t>FSN E-Commerce Ventures Limited</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -2562,17 +2562,17 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Textile Manufacturing</t>
+          <t>Internet Retail</t>
         </is>
       </c>
       <c r="E16" s="5" t="n">
-        <v>52.59999999999999</v>
+        <v>51.2</v>
       </c>
       <c r="F16" s="2" t="n">
-        <v>35.4</v>
+        <v>34.6</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>17.2</v>
+        <v>16.6</v>
       </c>
       <c r="H16" s="5" t="inlineStr">
         <is>
@@ -2581,23 +2581,23 @@
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>✅ Supertrend Buy | 📈 EMA Bull Stack | 🏆 Near 52W High</t>
+          <t>✅ Supertrend Buy | 📈 EMA Bull Stack | 🏆 At 52W High | 📉 Tight Base</t>
         </is>
       </c>
       <c r="J16" s="2" t="n">
-        <v>109.06</v>
+        <v>343</v>
       </c>
       <c r="K16" s="2" t="n">
-        <v>-0.62</v>
+        <v>3.22</v>
       </c>
       <c r="L16" s="2" t="n">
-        <v>101.73</v>
+        <v>334.34</v>
       </c>
       <c r="M16" s="2" t="n">
-        <v>89.47</v>
+        <v>329.95</v>
       </c>
       <c r="N16" s="2" t="n">
-        <v>66.42</v>
+        <v>295.89</v>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
@@ -2610,99 +2610,99 @@
         </is>
       </c>
       <c r="Q16" s="2" t="n">
-        <v>95.18000000000001</v>
+        <v>98.13</v>
       </c>
       <c r="R16" s="2" t="n">
-        <v>64.39</v>
+        <v>56.16</v>
       </c>
       <c r="S16" s="2" t="n">
-        <v>7.5175</v>
+        <v>1.0294</v>
       </c>
       <c r="T16" s="2" t="n">
-        <v>7.5576</v>
+        <v>0.1694</v>
       </c>
       <c r="U16" s="2" t="n">
-        <v>-0.0401</v>
+        <v>0.86</v>
       </c>
       <c r="V16" s="2" t="inlineStr"/>
       <c r="W16" s="2" t="n">
-        <v>44.9</v>
+        <v>18.04</v>
       </c>
       <c r="X16" s="2" t="n">
-        <v>1524085</v>
+        <v>5152542</v>
       </c>
       <c r="Y16" s="2" t="n">
-        <v>7397650</v>
+        <v>4886427</v>
       </c>
       <c r="Z16" s="2" t="n">
-        <v>0.21</v>
+        <v>1.05</v>
       </c>
       <c r="AA16" s="2" t="n">
-        <v>4786</v>
+        <v>96859</v>
       </c>
       <c r="AB16" s="2" t="n">
-        <v>25.065115</v>
+        <v>375.55557</v>
       </c>
       <c r="AC16" s="2" t="n">
-        <v>8.109857</v>
+        <v>115.97107</v>
       </c>
       <c r="AD16" s="2" t="inlineStr"/>
       <c r="AE16" s="2" t="n">
-        <v>9.988</v>
+        <v>82.82899999999999</v>
       </c>
       <c r="AF16" s="2" t="n">
-        <v>9.1</v>
+        <v>29.1</v>
       </c>
       <c r="AG16" s="2" t="n">
-        <v>18.5</v>
+        <v>250</v>
       </c>
       <c r="AH16" s="2" t="n">
-        <v>4.974844</v>
+        <v>67.30386</v>
       </c>
       <c r="AI16" s="2" t="n">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="AJ16" s="2" t="inlineStr"/>
       <c r="AK16" s="2" t="inlineStr">
         <is>
-          <t>https://www.screener.in/company/FILATEX/</t>
+          <t>https://www.screener.in/company/NYKAA/</t>
         </is>
       </c>
       <c r="AL16" s="2" t="inlineStr">
         <is>
-          <t>https://www.tradingview.com/chart/?symbol=NSE:FILATEX</t>
+          <t>https://www.tradingview.com/chart/?symbol=NSE:NYKAA</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>NYKAA</t>
+          <t>GREENPLY</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>FSN E-Commerce Ventures Limited</t>
+          <t>Greenply Industries Limited</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Consumer Cyclical</t>
+          <t>Basic Materials</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>Internet Retail</t>
+          <t>Lumber &amp; Wood Production</t>
         </is>
       </c>
       <c r="E17" s="5" t="n">
-        <v>51.2</v>
+        <v>50.90000000000001</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>34.6</v>
+        <v>32.2</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>16.6</v>
+        <v>18.7</v>
       </c>
       <c r="H17" s="5" t="inlineStr">
         <is>
@@ -2711,23 +2711,23 @@
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>✅ Supertrend Buy | 📈 EMA Bull Stack | 🏆 At 52W High | 📉 Tight Base</t>
+          <t>✅ Supertrend Buy | 📈 EMA Bull Stack | 🏆 Near 52W High | 📉 Tight Base</t>
         </is>
       </c>
       <c r="J17" s="4" t="n">
-        <v>343</v>
+        <v>306.7</v>
       </c>
       <c r="K17" s="4" t="n">
-        <v>3.22</v>
+        <v>0.33</v>
       </c>
       <c r="L17" s="4" t="n">
-        <v>334.34</v>
+        <v>298.66</v>
       </c>
       <c r="M17" s="4" t="n">
-        <v>329.95</v>
+        <v>294.21</v>
       </c>
       <c r="N17" s="4" t="n">
-        <v>295.89</v>
+        <v>279.76</v>
       </c>
       <c r="O17" s="4" t="inlineStr">
         <is>
@@ -2740,67 +2740,67 @@
         </is>
       </c>
       <c r="Q17" s="4" t="n">
-        <v>98.13</v>
+        <v>91.88</v>
       </c>
       <c r="R17" s="4" t="n">
-        <v>56.16</v>
+        <v>57.05</v>
       </c>
       <c r="S17" s="4" t="n">
-        <v>1.0294</v>
+        <v>4.4258</v>
       </c>
       <c r="T17" s="4" t="n">
-        <v>0.1694</v>
+        <v>2.5512</v>
       </c>
       <c r="U17" s="4" t="n">
-        <v>0.86</v>
+        <v>1.8745</v>
       </c>
       <c r="V17" s="4" t="inlineStr"/>
       <c r="W17" s="4" t="n">
-        <v>18.04</v>
+        <v>16.09</v>
       </c>
       <c r="X17" s="4" t="n">
-        <v>5152542</v>
+        <v>126215</v>
       </c>
       <c r="Y17" s="4" t="n">
-        <v>4886427</v>
+        <v>239993</v>
       </c>
       <c r="Z17" s="4" t="n">
-        <v>1.05</v>
+        <v>0.53</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>97433</v>
+        <v>3916</v>
       </c>
       <c r="AB17" s="4" t="n">
-        <v>382.0225</v>
+        <v>40.451614</v>
       </c>
       <c r="AC17" s="4" t="n">
-        <v>116.65729</v>
+        <v>18.700464</v>
       </c>
       <c r="AD17" s="4" t="inlineStr"/>
       <c r="AE17" s="4" t="n">
-        <v>82.82899999999999</v>
+        <v>57.505</v>
       </c>
       <c r="AF17" s="4" t="n">
-        <v>29.1</v>
+        <v>20.7</v>
       </c>
       <c r="AG17" s="4" t="n">
-        <v>250</v>
+        <v>32</v>
       </c>
       <c r="AH17" s="4" t="n">
-        <v>67.70211</v>
+        <v>4.340482</v>
       </c>
       <c r="AI17" s="4" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="AJ17" s="4" t="inlineStr"/>
       <c r="AK17" s="4" t="inlineStr">
         <is>
-          <t>https://www.screener.in/company/NYKAA/</t>
+          <t>https://www.screener.in/company/GREENPLY/</t>
         </is>
       </c>
       <c r="AL17" s="4" t="inlineStr">
         <is>
-          <t>https://www.tradingview.com/chart/?symbol=NSE:NYKAA</t>
+          <t>https://www.tradingview.com/chart/?symbol=NSE:GREENPLY</t>
         </is>
       </c>
     </row>
@@ -2902,13 +2902,13 @@
         <v>0.8</v>
       </c>
       <c r="AA18" s="2" t="n">
-        <v>81078</v>
+        <v>81399</v>
       </c>
       <c r="AB18" s="2" t="n">
-        <v>17.560192</v>
+        <v>17.535923</v>
       </c>
       <c r="AC18" s="2" t="n">
-        <v>11.653659</v>
+        <v>11.699819</v>
       </c>
       <c r="AD18" s="2" t="inlineStr"/>
       <c r="AE18" s="2" t="inlineStr"/>
@@ -2919,10 +2919,10 @@
         <v>32.7</v>
       </c>
       <c r="AH18" s="2" t="n">
-        <v>2.0203762</v>
+        <v>2.0283787</v>
       </c>
       <c r="AI18" s="2" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="AJ18" s="2" t="inlineStr"/>
       <c r="AK18" s="2" t="inlineStr">
@@ -3030,13 +3030,13 @@
         <v>0.87</v>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>390156</v>
+        <v>394951</v>
       </c>
       <c r="AB19" s="4" t="n">
-        <v>14.089733</v>
+        <v>14.19427</v>
       </c>
       <c r="AC19" s="4" t="n">
-        <v>10.380178</v>
+        <v>10.507756</v>
       </c>
       <c r="AD19" s="4" t="n">
         <v>13.35</v>
@@ -3049,7 +3049,7 @@
         <v>21.8</v>
       </c>
       <c r="AH19" s="4" t="n">
-        <v>1.746227</v>
+        <v>1.7676891</v>
       </c>
       <c r="AI19" s="4" t="n">
         <v>8</v>
@@ -3160,13 +3160,13 @@
         <v>0.42</v>
       </c>
       <c r="AA20" s="2" t="n">
-        <v>33463</v>
+        <v>32631</v>
       </c>
       <c r="AB20" s="2" t="n">
-        <v>90.33801</v>
+        <v>88.97058</v>
       </c>
       <c r="AC20" s="2" t="n">
-        <v>54.220943</v>
+        <v>52.8726</v>
       </c>
       <c r="AD20" s="2" t="inlineStr"/>
       <c r="AE20" s="2" t="n">
@@ -3179,7 +3179,7 @@
         <v>86</v>
       </c>
       <c r="AH20" s="2" t="n">
-        <v>11.610514</v>
+        <v>11.321789</v>
       </c>
       <c r="AI20" s="2" t="n">
         <v>9</v>
@@ -3294,13 +3294,13 @@
         <v>1.1</v>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>61032</v>
+        <v>60831</v>
       </c>
       <c r="AB21" s="4" t="n">
-        <v>86.71236</v>
+        <v>86.52563499999999</v>
       </c>
       <c r="AC21" s="4" t="n">
-        <v>56.69105</v>
+        <v>56.504364</v>
       </c>
       <c r="AD21" s="4" t="inlineStr"/>
       <c r="AE21" s="4" t="n">
@@ -3313,7 +3313,7 @@
         <v>76</v>
       </c>
       <c r="AH21" s="4" t="n">
-        <v>18.394304</v>
+        <v>18.33373</v>
       </c>
       <c r="AI21" s="4" t="n">
         <v>20</v>
@@ -3424,13 +3424,13 @@
         <v>0.24</v>
       </c>
       <c r="AA22" s="2" t="n">
-        <v>7706</v>
+        <v>7719</v>
       </c>
       <c r="AB22" s="2" t="n">
-        <v>164.0085</v>
+        <v>160.41495</v>
       </c>
       <c r="AC22" s="2" t="n">
-        <v>68.51479</v>
+        <v>68.62721999999999</v>
       </c>
       <c r="AD22" s="2" t="inlineStr"/>
       <c r="AE22" s="2" t="n">
@@ -3443,7 +3443,7 @@
         <v>-99.59999999999999</v>
       </c>
       <c r="AH22" s="2" t="n">
-        <v>2.7095776</v>
+        <v>2.7140238</v>
       </c>
       <c r="AI22" s="2" t="n">
         <v>0</v>
@@ -3554,13 +3554,13 @@
         <v>1.08</v>
       </c>
       <c r="AA23" s="4" t="n">
-        <v>64839</v>
+        <v>60236</v>
       </c>
       <c r="AB23" s="4" t="n">
-        <v>30.400293</v>
+        <v>27.997835</v>
       </c>
       <c r="AC23" s="4" t="n">
-        <v>21.386383</v>
+        <v>19.453848</v>
       </c>
       <c r="AD23" s="4" t="inlineStr"/>
       <c r="AE23" s="4" t="inlineStr"/>
@@ -3571,7 +3571,7 @@
         <v>-11.7</v>
       </c>
       <c r="AH23" s="4" t="n">
-        <v>1.541556</v>
+        <v>1.4321302</v>
       </c>
       <c r="AI23" s="4" t="n">
         <v>24</v>
@@ -3682,13 +3682,13 @@
         <v>0.5600000000000001</v>
       </c>
       <c r="AA24" s="2" t="n">
-        <v>135249</v>
+        <v>137085</v>
       </c>
       <c r="AB24" s="2" t="n">
-        <v>48.44632</v>
+        <v>49.747974</v>
       </c>
       <c r="AC24" s="2" t="n">
-        <v>37.490215</v>
+        <v>37.99906</v>
       </c>
       <c r="AD24" s="2" t="inlineStr"/>
       <c r="AE24" s="2" t="n">
@@ -3701,7 +3701,7 @@
         <v>62.1</v>
       </c>
       <c r="AH24" s="2" t="n">
-        <v>17.151037</v>
+        <v>17.383825</v>
       </c>
       <c r="AI24" s="2" t="n">
         <v>30</v>
@@ -3812,13 +3812,13 @@
         <v>10.52</v>
       </c>
       <c r="AA25" s="4" t="n">
-        <v>3775</v>
+        <v>3793</v>
       </c>
       <c r="AB25" s="4" t="n">
-        <v>30.320515</v>
+        <v>30.31538</v>
       </c>
       <c r="AC25" s="4" t="n">
-        <v>14.00329</v>
+        <v>14.070724</v>
       </c>
       <c r="AD25" s="4" t="inlineStr"/>
       <c r="AE25" s="4" t="n">
@@ -3829,7 +3829,7 @@
       </c>
       <c r="AG25" s="4" t="inlineStr"/>
       <c r="AH25" s="4" t="n">
-        <v>3.127962</v>
+        <v>3.1430252</v>
       </c>
       <c r="AI25" s="4" t="n">
         <v>0</v>
@@ -3940,13 +3940,13 @@
         <v>0.92</v>
       </c>
       <c r="AA26" s="2" t="n">
-        <v>90238</v>
+        <v>92677</v>
       </c>
       <c r="AB26" s="2" t="n">
-        <v>26.47788</v>
+        <v>26.805735</v>
       </c>
       <c r="AC26" s="2" t="n">
-        <v>22.84958</v>
+        <v>23.467138</v>
       </c>
       <c r="AD26" s="2" t="n">
         <v>49.9</v>
@@ -3961,10 +3961,10 @@
         <v>120.2</v>
       </c>
       <c r="AH26" s="2" t="n">
-        <v>13.021914</v>
+        <v>13.3738575</v>
       </c>
       <c r="AI26" s="2" t="n">
-        <v>381</v>
+        <v>386</v>
       </c>
       <c r="AJ26" s="2" t="n">
         <v>4.413</v>
@@ -4074,13 +4074,13 @@
         <v>1</v>
       </c>
       <c r="AA27" s="4" t="n">
-        <v>43575</v>
+        <v>43500</v>
       </c>
       <c r="AB27" s="4" t="n">
-        <v>10.352816</v>
+        <v>10.298296</v>
       </c>
       <c r="AC27" s="4" t="n">
-        <v>10.220337</v>
+        <v>10.202746</v>
       </c>
       <c r="AD27" s="4" t="inlineStr"/>
       <c r="AE27" s="4" t="n">
@@ -4093,10 +4093,10 @@
         <v>35.1</v>
       </c>
       <c r="AH27" s="4" t="n">
-        <v>1.9549916</v>
+        <v>1.9516267</v>
       </c>
       <c r="AI27" s="4" t="n">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="AJ27" s="4" t="inlineStr"/>
       <c r="AK27" s="4" t="inlineStr">
@@ -4204,13 +4204,13 @@
         <v>0.8</v>
       </c>
       <c r="AA28" s="2" t="n">
-        <v>111801</v>
+        <v>111272</v>
       </c>
       <c r="AB28" s="2" t="n">
-        <v>102.28374</v>
+        <v>103.435455</v>
       </c>
       <c r="AC28" s="2" t="n">
-        <v>70.10499</v>
+        <v>69.772964</v>
       </c>
       <c r="AD28" s="2" t="inlineStr"/>
       <c r="AE28" s="2" t="n">
@@ -4223,7 +4223,7 @@
         <v>125.2</v>
       </c>
       <c r="AH28" s="2" t="n">
-        <v>21.076647</v>
+        <v>20.976826</v>
       </c>
       <c r="AI28" s="2" t="n">
         <v>12</v>
@@ -4334,13 +4334,13 @@
         <v>0.13</v>
       </c>
       <c r="AA29" s="4" t="n">
-        <v>9110</v>
+        <v>9241</v>
       </c>
       <c r="AB29" s="4" t="n">
-        <v>287.6961</v>
+        <v>294.72772</v>
       </c>
       <c r="AC29" s="4" t="n">
-        <v>110.78414</v>
+        <v>112.379166</v>
       </c>
       <c r="AD29" s="4" t="inlineStr"/>
       <c r="AE29" s="4" t="n">
@@ -4353,7 +4353,7 @@
         <v>-50</v>
       </c>
       <c r="AH29" s="4" t="n">
-        <v>15.009847</v>
+        <v>15.225952</v>
       </c>
       <c r="AI29" s="4" t="n">
         <v>14</v>
@@ -4468,13 +4468,13 @@
         <v>1.06</v>
       </c>
       <c r="AA30" s="2" t="n">
-        <v>30059</v>
+        <v>30693</v>
       </c>
       <c r="AB30" s="2" t="n">
-        <v>19.692308</v>
+        <v>20.434647</v>
       </c>
       <c r="AC30" s="2" t="n">
-        <v>10.455507</v>
+        <v>10.676053</v>
       </c>
       <c r="AD30" s="2" t="inlineStr"/>
       <c r="AE30" s="2" t="n">
@@ -4487,10 +4487,10 @@
         <v>288.5</v>
       </c>
       <c r="AH30" s="2" t="n">
-        <v>1.8727359</v>
+        <v>1.912239</v>
       </c>
       <c r="AI30" s="2" t="n">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="AJ30" s="2" t="inlineStr"/>
       <c r="AK30" s="2" t="inlineStr">
@@ -4598,13 +4598,13 @@
         <v>0.84</v>
       </c>
       <c r="AA31" s="4" t="n">
-        <v>130787</v>
+        <v>131466</v>
       </c>
       <c r="AB31" s="4" t="n">
-        <v>6.3338265</v>
+        <v>6.303807</v>
       </c>
       <c r="AC31" s="4" t="n">
-        <v>6.284353</v>
+        <v>6.316998</v>
       </c>
       <c r="AD31" s="4" t="n">
         <v>15.8</v>
@@ -4617,10 +4617,10 @@
         <v>27.4</v>
       </c>
       <c r="AH31" s="4" t="n">
-        <v>0.9374077</v>
+        <v>0.9422772</v>
       </c>
       <c r="AI31" s="4" t="n">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="AJ31" s="4" t="inlineStr"/>
       <c r="AK31" s="4" t="inlineStr">
@@ -4728,13 +4728,13 @@
         <v>0.25</v>
       </c>
       <c r="AA32" s="2" t="n">
-        <v>9333</v>
+        <v>9390</v>
       </c>
       <c r="AB32" s="2" t="n">
-        <v>41.505917</v>
+        <v>42.156143</v>
       </c>
       <c r="AC32" s="2" t="n">
-        <v>39.55058</v>
+        <v>39.79552</v>
       </c>
       <c r="AD32" s="2" t="inlineStr"/>
       <c r="AE32" s="2" t="n">
@@ -4747,7 +4747,7 @@
         <v>91.40000000000001</v>
       </c>
       <c r="AH32" s="2" t="n">
-        <v>6.085773</v>
+        <v>6.123463</v>
       </c>
       <c r="AI32" s="2" t="n">
         <v>55</v>
@@ -4858,13 +4858,13 @@
         <v>0.88</v>
       </c>
       <c r="AA33" s="4" t="n">
-        <v>98211</v>
+        <v>96928</v>
       </c>
       <c r="AB33" s="4" t="n">
-        <v>26.670313</v>
+        <v>26.537493</v>
       </c>
       <c r="AC33" s="4" t="n">
-        <v>18.283337</v>
+        <v>18.030642</v>
       </c>
       <c r="AD33" s="4" t="inlineStr"/>
       <c r="AE33" s="4" t="n">
@@ -4877,7 +4877,7 @@
         <v>25.8</v>
       </c>
       <c r="AH33" s="4" t="n">
-        <v>2.616376</v>
+        <v>2.5821939</v>
       </c>
       <c r="AI33" s="4" t="n">
         <v>0</v>
@@ -4992,13 +4992,13 @@
         <v>0.9399999999999999</v>
       </c>
       <c r="AA34" s="2" t="n">
-        <v>6432</v>
+        <v>6639</v>
       </c>
       <c r="AB34" s="2" t="n">
-        <v>29.485027</v>
+        <v>29.566608</v>
       </c>
       <c r="AC34" s="2" t="n">
-        <v>21.69163</v>
+        <v>22.389868</v>
       </c>
       <c r="AD34" s="2" t="inlineStr"/>
       <c r="AE34" s="2" t="n">
@@ -5011,7 +5011,7 @@
         <v>95.7</v>
       </c>
       <c r="AH34" s="2" t="n">
-        <v>8.732044</v>
+        <v>9.013123</v>
       </c>
       <c r="AI34" s="2" t="n">
         <v>0</v>
@@ -5122,13 +5122,13 @@
         <v>0.68</v>
       </c>
       <c r="AA35" s="4" t="n">
-        <v>64432</v>
+        <v>63932</v>
       </c>
       <c r="AB35" s="4" t="n">
-        <v>35.8455</v>
+        <v>35.41191</v>
       </c>
       <c r="AC35" s="4" t="n">
-        <v>23.51473</v>
+        <v>23.354073</v>
       </c>
       <c r="AD35" s="4" t="inlineStr"/>
       <c r="AE35" s="4" t="n">
@@ -5141,7 +5141,7 @@
         <v>930.7</v>
       </c>
       <c r="AH35" s="4" t="n">
-        <v>6.1292706</v>
+        <v>6.0817504</v>
       </c>
       <c r="AI35" s="4" t="n">
         <v>11</v>
@@ -5252,13 +5252,13 @@
         <v>0.71</v>
       </c>
       <c r="AA36" s="2" t="n">
-        <v>167314</v>
+        <v>170522</v>
       </c>
       <c r="AB36" s="2" t="n">
-        <v>37.828915</v>
+        <v>39.603962</v>
       </c>
       <c r="AC36" s="2" t="n">
-        <v>22.603548</v>
+        <v>23.036928</v>
       </c>
       <c r="AD36" s="2" t="inlineStr"/>
       <c r="AE36" s="2" t="n">
@@ -5271,10 +5271,10 @@
         <v>104.2</v>
       </c>
       <c r="AH36" s="2" t="n">
-        <v>4.034488</v>
+        <v>4.111842</v>
       </c>
       <c r="AI36" s="2" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="AJ36" s="2" t="inlineStr"/>
       <c r="AK36" s="2" t="inlineStr">
@@ -5382,13 +5382,13 @@
         <v>1.19</v>
       </c>
       <c r="AA37" s="4" t="n">
-        <v>10211</v>
+        <v>10366</v>
       </c>
       <c r="AB37" s="4" t="n">
-        <v>42.10205</v>
+        <v>43.141026</v>
       </c>
       <c r="AC37" s="4" t="n">
-        <v>23.34085</v>
+        <v>23.683283</v>
       </c>
       <c r="AD37" s="4" t="inlineStr"/>
       <c r="AE37" s="4" t="n">
@@ -5401,7 +5401,7 @@
         <v>101.5</v>
       </c>
       <c r="AH37" s="4" t="n">
-        <v>5.0766277</v>
+        <v>5.151107</v>
       </c>
       <c r="AI37" s="4" t="n">
         <v>0</v>
@@ -5512,13 +5512,13 @@
         <v>0.28</v>
       </c>
       <c r="AA38" s="2" t="n">
-        <v>15905</v>
+        <v>15255</v>
       </c>
       <c r="AB38" s="2" t="n">
-        <v>119.31761</v>
+        <v>118.29875</v>
       </c>
       <c r="AC38" s="2" t="n">
-        <v>64.89892999999999</v>
+        <v>62.24621</v>
       </c>
       <c r="AD38" s="2" t="inlineStr"/>
       <c r="AE38" s="2" t="n">
@@ -5531,7 +5531,7 @@
         <v>145.3</v>
       </c>
       <c r="AH38" s="2" t="n">
-        <v>22.01159</v>
+        <v>21.111874</v>
       </c>
       <c r="AI38" s="2" t="n">
         <v>0</v>
@@ -5642,13 +5642,13 @@
         <v>0.77</v>
       </c>
       <c r="AA39" s="4" t="n">
-        <v>27644</v>
+        <v>28352</v>
       </c>
       <c r="AB39" s="4" t="n">
-        <v>27.352942</v>
+        <v>29.026217</v>
       </c>
       <c r="AC39" s="4" t="n">
-        <v>17.35745</v>
+        <v>17.802513</v>
       </c>
       <c r="AD39" s="4" t="inlineStr"/>
       <c r="AE39" s="4" t="n">
@@ -5661,10 +5661,10 @@
         <v>100</v>
       </c>
       <c r="AH39" s="4" t="n">
-        <v>4.5001116</v>
+        <v>4.615499</v>
       </c>
       <c r="AI39" s="4" t="n">
-        <v>173</v>
+        <v>167</v>
       </c>
       <c r="AJ39" s="4" t="inlineStr"/>
       <c r="AK39" s="4" t="inlineStr">
@@ -5772,13 +5772,13 @@
         <v>1.14</v>
       </c>
       <c r="AA40" s="2" t="n">
-        <v>16246</v>
+        <v>16467</v>
       </c>
       <c r="AB40" s="2" t="n">
-        <v>27.306454</v>
+        <v>27.682722</v>
       </c>
       <c r="AC40" s="2" t="n">
-        <v>26.922016</v>
+        <v>27.289165</v>
       </c>
       <c r="AD40" s="2" t="inlineStr"/>
       <c r="AE40" s="2" t="n">
@@ -5789,10 +5789,10 @@
       </c>
       <c r="AG40" s="2" t="inlineStr"/>
       <c r="AH40" s="2" t="n">
-        <v>5.5373235</v>
+        <v>5.6128387</v>
       </c>
       <c r="AI40" s="2" t="n">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="AJ40" s="2" t="inlineStr"/>
       <c r="AK40" s="2" t="inlineStr">
@@ -5900,13 +5900,13 @@
         <v>0.32</v>
       </c>
       <c r="AA41" s="4" t="n">
-        <v>24579</v>
+        <v>23799</v>
       </c>
       <c r="AB41" s="4" t="n">
-        <v>40.22352</v>
+        <v>40.392296</v>
       </c>
       <c r="AC41" s="4" t="n">
-        <v>28.084032</v>
+        <v>27.193275</v>
       </c>
       <c r="AD41" s="4" t="inlineStr"/>
       <c r="AE41" s="4" t="n">
@@ -5919,10 +5919,10 @@
         <v>13.5</v>
       </c>
       <c r="AH41" s="4" t="n">
-        <v>5.749352</v>
+        <v>5.566997</v>
       </c>
       <c r="AI41" s="4" t="n">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="AJ41" s="4" t="inlineStr"/>
       <c r="AK41" s="4" t="inlineStr">
@@ -6030,13 +6030,13 @@
         <v>0.73</v>
       </c>
       <c r="AA42" s="2" t="n">
-        <v>318337</v>
+        <v>325627</v>
       </c>
       <c r="AB42" s="2" t="n">
-        <v>34.15124</v>
+        <v>35.71481</v>
       </c>
       <c r="AC42" s="2" t="n">
-        <v>27.558949</v>
+        <v>28.190025</v>
       </c>
       <c r="AD42" s="2" t="inlineStr"/>
       <c r="AE42" s="2" t="n">
@@ -6049,10 +6049,10 @@
         <v>14.9</v>
       </c>
       <c r="AH42" s="2" t="n">
-        <v>7.7565355</v>
+        <v>7.934154</v>
       </c>
       <c r="AI42" s="2" t="n">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="AJ42" s="2" t="inlineStr"/>
       <c r="AK42" s="2" t="inlineStr">
@@ -6160,13 +6160,13 @@
         <v>0.4</v>
       </c>
       <c r="AA43" s="4" t="n">
-        <v>12002</v>
+        <v>12307</v>
       </c>
       <c r="AB43" s="4" t="n">
-        <v>31.105164</v>
+        <v>31.459627</v>
       </c>
       <c r="AC43" s="4" t="n">
-        <v>26.74337</v>
+        <v>27.42285</v>
       </c>
       <c r="AD43" s="4" t="inlineStr"/>
       <c r="AE43" s="4" t="n">
@@ -6179,10 +6179,10 @@
         <v>14.9</v>
       </c>
       <c r="AH43" s="4" t="n">
-        <v>6.1024427</v>
+        <v>6.2574897</v>
       </c>
       <c r="AI43" s="4" t="n">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="AJ43" s="4" t="inlineStr"/>
       <c r="AK43" s="4" t="inlineStr">
@@ -6290,13 +6290,13 @@
         <v>0.42</v>
       </c>
       <c r="AA44" s="2" t="n">
-        <v>160895</v>
+        <v>164559</v>
       </c>
       <c r="AB44" s="2" t="n">
-        <v>36.19154</v>
+        <v>37.098213</v>
       </c>
       <c r="AC44" s="2" t="n">
-        <v>25.574875</v>
+        <v>26.157194</v>
       </c>
       <c r="AD44" s="2" t="n">
         <v>10.1</v>
@@ -6311,7 +6311,7 @@
         <v>4.2</v>
       </c>
       <c r="AH44" s="2" t="n">
-        <v>3.5382237</v>
+        <v>3.6187863</v>
       </c>
       <c r="AI44" s="2" t="n">
         <v>123</v>
@@ -6425,7 +6425,7 @@
         <v>13342</v>
       </c>
       <c r="AB45" s="4" t="n">
-        <v>22.700161</v>
+        <v>22.626818</v>
       </c>
       <c r="AC45" s="4" t="n">
         <v>16.813925</v>
@@ -6546,13 +6546,13 @@
         <v>0.47</v>
       </c>
       <c r="AA46" s="2" t="n">
-        <v>21914</v>
+        <v>22218</v>
       </c>
       <c r="AB46" s="2" t="n">
-        <v>29.842123</v>
+        <v>29.813324</v>
       </c>
       <c r="AC46" s="2" t="n">
-        <v>20.50857</v>
+        <v>20.793217</v>
       </c>
       <c r="AD46" s="2" t="inlineStr"/>
       <c r="AE46" s="2" t="n">
@@ -6565,10 +6565,10 @@
         <v>53.4</v>
       </c>
       <c r="AH46" s="2" t="n">
-        <v>3.9148085</v>
+        <v>3.9691436</v>
       </c>
       <c r="AI46" s="2" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="AJ46" s="2" t="inlineStr"/>
       <c r="AK46" s="2" t="inlineStr">
@@ -6676,13 +6676,13 @@
         <v>1</v>
       </c>
       <c r="AA47" s="4" t="n">
-        <v>13410</v>
+        <v>13490</v>
       </c>
       <c r="AB47" s="4" t="n">
-        <v>32.37658</v>
+        <v>32.69377</v>
       </c>
       <c r="AC47" s="4" t="n">
-        <v>19.871529</v>
+        <v>19.990007</v>
       </c>
       <c r="AD47" s="4" t="inlineStr"/>
       <c r="AE47" s="4" t="n">
@@ -6695,7 +6695,7 @@
         <v>0.5</v>
       </c>
       <c r="AH47" s="4" t="n">
-        <v>3.315488</v>
+        <v>3.3352559</v>
       </c>
       <c r="AI47" s="4" t="n">
         <v>88</v>
@@ -6806,13 +6806,13 @@
         <v>0.31</v>
       </c>
       <c r="AA48" s="2" t="n">
-        <v>102926</v>
+        <v>104756</v>
       </c>
       <c r="AB48" s="2" t="n">
-        <v>47.213005</v>
+        <v>47.76715</v>
       </c>
       <c r="AC48" s="2" t="n">
-        <v>38.13897</v>
+        <v>38.790337</v>
       </c>
       <c r="AD48" s="2" t="inlineStr"/>
       <c r="AE48" s="2" t="n">
@@ -6825,10 +6825,10 @@
         <v>20.7</v>
       </c>
       <c r="AH48" s="2" t="n">
-        <v>7.759335</v>
+        <v>7.897291</v>
       </c>
       <c r="AI48" s="2" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AJ48" s="2" t="inlineStr"/>
       <c r="AK48" s="2" t="inlineStr">
@@ -6936,13 +6936,13 @@
         <v>2.62</v>
       </c>
       <c r="AA49" s="4" t="n">
-        <v>70632</v>
+        <v>71363</v>
       </c>
       <c r="AB49" s="4" t="n">
-        <v>16.537718</v>
+        <v>16.66056</v>
       </c>
       <c r="AC49" s="4" t="n">
-        <v>10.790993</v>
+        <v>10.902689</v>
       </c>
       <c r="AD49" s="4" t="inlineStr"/>
       <c r="AE49" s="4" t="n">
@@ -6955,7 +6955,7 @@
         <v>121.1</v>
       </c>
       <c r="AH49" s="4" t="n">
-        <v>1.1712248</v>
+        <v>1.1833481</v>
       </c>
       <c r="AI49" s="4" t="n">
         <v>137</v>
@@ -7062,13 +7062,13 @@
         <v>0.95</v>
       </c>
       <c r="AA50" s="2" t="n">
-        <v>29730</v>
+        <v>30048</v>
       </c>
       <c r="AB50" s="2" t="n">
-        <v>108.95425</v>
+        <v>116.65359</v>
       </c>
       <c r="AC50" s="2" t="n">
-        <v>59.36755</v>
+        <v>60.003845</v>
       </c>
       <c r="AD50" s="2" t="inlineStr"/>
       <c r="AE50" s="2" t="n">
@@ -7081,7 +7081,7 @@
         <v>178.4</v>
       </c>
       <c r="AH50" s="2" t="n">
-        <v>39.26726</v>
+        <v>39.68812</v>
       </c>
       <c r="AI50" s="2" t="n">
         <v>6</v>
@@ -7192,13 +7192,13 @@
         <v>0.9399999999999999</v>
       </c>
       <c r="AA51" s="4" t="n">
-        <v>178088</v>
+        <v>176601</v>
       </c>
       <c r="AB51" s="4" t="n">
-        <v>74.79233600000001</v>
+        <v>74.57276</v>
       </c>
       <c r="AC51" s="4" t="n">
-        <v>50.17372</v>
+        <v>49.76497</v>
       </c>
       <c r="AD51" s="4" t="inlineStr"/>
       <c r="AE51" s="4" t="n">
@@ -7211,10 +7211,10 @@
         <v>-8.199999999999999</v>
       </c>
       <c r="AH51" s="4" t="n">
-        <v>18.890305</v>
+        <v>18.73255</v>
       </c>
       <c r="AI51" s="4" t="n">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="AJ51" s="4" t="inlineStr"/>
       <c r="AK51" s="4" t="inlineStr">
@@ -7318,13 +7318,13 @@
         <v>1.25</v>
       </c>
       <c r="AA52" s="2" t="n">
-        <v>209850</v>
+        <v>211992</v>
       </c>
       <c r="AB52" s="2" t="n">
-        <v>122.030655</v>
+        <v>125.07288</v>
       </c>
       <c r="AC52" s="2" t="n">
-        <v>42.92119</v>
+        <v>43.141144</v>
       </c>
       <c r="AD52" s="2" t="inlineStr"/>
       <c r="AE52" s="2" t="n">
@@ -7337,7 +7337,7 @@
         <v>18.5</v>
       </c>
       <c r="AH52" s="2" t="n">
-        <v>10.878661</v>
+        <v>10.989668</v>
       </c>
       <c r="AI52" s="2" t="n">
         <v>0</v>
@@ -7448,13 +7448,13 @@
         <v>0.37</v>
       </c>
       <c r="AA53" s="4" t="n">
-        <v>68504</v>
+        <v>67978</v>
       </c>
       <c r="AB53" s="4" t="n">
-        <v>30.671816</v>
+        <v>30.436295</v>
       </c>
       <c r="AC53" s="4" t="n">
-        <v>11.604433</v>
+        <v>11.515325</v>
       </c>
       <c r="AD53" s="4" t="n">
         <v>5.26</v>
@@ -7467,7 +7467,7 @@
         <v>116.4</v>
       </c>
       <c r="AH53" s="4" t="n">
-        <v>1.4055699</v>
+        <v>1.3947768</v>
       </c>
       <c r="AI53" s="4" t="n">
         <v>31</v>
@@ -7578,13 +7578,13 @@
         <v>1.42</v>
       </c>
       <c r="AA54" s="2" t="n">
-        <v>130126</v>
+        <v>133260</v>
       </c>
       <c r="AB54" s="2" t="n">
-        <v>89.58078</v>
+        <v>93.24695</v>
       </c>
       <c r="AC54" s="2" t="n">
-        <v>54.488495</v>
+        <v>55.09112</v>
       </c>
       <c r="AD54" s="2" t="inlineStr"/>
       <c r="AE54" s="2" t="n">
@@ -7597,10 +7597,10 @@
         <v>406.1</v>
       </c>
       <c r="AH54" s="2" t="n">
-        <v>9.402065</v>
+        <v>9.628496999999999</v>
       </c>
       <c r="AI54" s="2" t="n">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="AJ54" s="2" t="inlineStr"/>
       <c r="AK54" s="2" t="inlineStr">
@@ -7708,13 +7708,13 @@
         <v>1.03</v>
       </c>
       <c r="AA55" s="4" t="n">
-        <v>130319</v>
+        <v>136742</v>
       </c>
       <c r="AB55" s="4" t="n">
-        <v>25.432226</v>
+        <v>25.928104</v>
       </c>
       <c r="AC55" s="4" t="n">
-        <v>16.756342</v>
+        <v>17.465141</v>
       </c>
       <c r="AD55" s="4" t="inlineStr"/>
       <c r="AE55" s="4" t="n">
@@ -7727,10 +7727,10 @@
         <v>28.3</v>
       </c>
       <c r="AH55" s="4" t="n">
-        <v>4.3988185</v>
+        <v>4.615619</v>
       </c>
       <c r="AI55" s="4" t="n">
-        <v>337</v>
+        <v>347</v>
       </c>
       <c r="AJ55" s="4" t="inlineStr"/>
       <c r="AK55" s="4" t="inlineStr">
@@ -8332,13 +8332,13 @@
         <v>1.44</v>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>441089</v>
+        <v>436712</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>21.735294</v>
+        <v>21.636272</v>
       </c>
       <c r="AC2" s="2" t="n">
-        <v>18.875738</v>
+        <v>18.688429</v>
       </c>
       <c r="AD2" s="2" t="inlineStr"/>
       <c r="AE2" s="2" t="inlineStr"/>
@@ -8349,7 +8349,7 @@
         <v>22.5</v>
       </c>
       <c r="AH2" s="2" t="n">
-        <v>2.433576</v>
+        <v>2.409427</v>
       </c>
       <c r="AI2" s="2" t="n">
         <v>15</v>
@@ -8460,13 +8460,13 @@
         <v>1.76</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>90785</v>
+        <v>93938</v>
       </c>
       <c r="AB3" s="4" t="n">
-        <v>47.376175</v>
+        <v>49.1666</v>
       </c>
       <c r="AC3" s="4" t="n">
-        <v>32.53733</v>
+        <v>33.667515</v>
       </c>
       <c r="AD3" s="4" t="n">
         <v>25.2</v>
@@ -8481,7 +8481,7 @@
         <v>12.1</v>
       </c>
       <c r="AH3" s="4" t="n">
-        <v>10.753688</v>
+        <v>11.127195</v>
       </c>
       <c r="AI3" s="4" t="n">
         <v>62</v>
@@ -8598,13 +8598,13 @@
         <v>0.9</v>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>133318</v>
+        <v>133950</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>6.0479665</v>
+        <v>6.0263705</v>
       </c>
       <c r="AC4" s="2" t="n">
-        <v>6.671329</v>
+        <v>6.7029605</v>
       </c>
       <c r="AD4" s="2" t="n">
         <v>14.97</v>
@@ -8617,10 +8617,10 @@
         <v>175</v>
       </c>
       <c r="AH4" s="2" t="n">
-        <v>0.85260266</v>
+        <v>0.85664517</v>
       </c>
       <c r="AI4" s="2" t="n">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="AJ4" s="2" t="inlineStr"/>
       <c r="AK4" s="2" t="inlineStr">
@@ -8728,13 +8728,13 @@
         <v>0.47</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>30446</v>
+        <v>30826</v>
       </c>
       <c r="AB5" s="4" t="n">
-        <v>9.688789</v>
+        <v>9.898142999999999</v>
       </c>
       <c r="AC5" s="4" t="n">
-        <v>3.3830576</v>
+        <v>3.4253166</v>
       </c>
       <c r="AD5" s="4" t="inlineStr"/>
       <c r="AE5" s="4" t="n">
@@ -8745,10 +8745,10 @@
       </c>
       <c r="AG5" s="4" t="inlineStr"/>
       <c r="AH5" s="4" t="n">
-        <v>2.136646</v>
+        <v>2.1633356</v>
       </c>
       <c r="AI5" s="4" t="n">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="AJ5" s="4" t="inlineStr"/>
       <c r="AK5" s="4" t="inlineStr">
@@ -9103,13 +9103,13 @@
         <v>1.44</v>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>441089</v>
+        <v>436712</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>21.735294</v>
+        <v>21.636272</v>
       </c>
       <c r="AC2" s="2" t="n">
-        <v>18.875738</v>
+        <v>18.688429</v>
       </c>
       <c r="AD2" s="2" t="inlineStr"/>
       <c r="AE2" s="2" t="inlineStr"/>
@@ -9120,7 +9120,7 @@
         <v>22.5</v>
       </c>
       <c r="AH2" s="2" t="n">
-        <v>2.433576</v>
+        <v>2.409427</v>
       </c>
       <c r="AI2" s="2" t="n">
         <v>15</v>
@@ -9231,13 +9231,13 @@
         <v>1.76</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>90785</v>
+        <v>93938</v>
       </c>
       <c r="AB3" s="4" t="n">
-        <v>47.376175</v>
+        <v>49.1666</v>
       </c>
       <c r="AC3" s="4" t="n">
-        <v>32.53733</v>
+        <v>33.667515</v>
       </c>
       <c r="AD3" s="4" t="n">
         <v>25.2</v>
@@ -9252,7 +9252,7 @@
         <v>12.1</v>
       </c>
       <c r="AH3" s="4" t="n">
-        <v>10.753688</v>
+        <v>11.127195</v>
       </c>
       <c r="AI3" s="4" t="n">
         <v>62</v>
@@ -9369,13 +9369,13 @@
         <v>0.9</v>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>133318</v>
+        <v>133950</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>6.0479665</v>
+        <v>6.0263705</v>
       </c>
       <c r="AC4" s="2" t="n">
-        <v>6.671329</v>
+        <v>6.7029605</v>
       </c>
       <c r="AD4" s="2" t="n">
         <v>14.97</v>
@@ -9388,10 +9388,10 @@
         <v>175</v>
       </c>
       <c r="AH4" s="2" t="n">
-        <v>0.85260266</v>
+        <v>0.85664517</v>
       </c>
       <c r="AI4" s="2" t="n">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="AJ4" s="2" t="inlineStr"/>
       <c r="AK4" s="2" t="inlineStr">
@@ -9499,13 +9499,13 @@
         <v>0.47</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>30446</v>
+        <v>30826</v>
       </c>
       <c r="AB5" s="4" t="n">
-        <v>9.688789</v>
+        <v>9.898142999999999</v>
       </c>
       <c r="AC5" s="4" t="n">
-        <v>3.3830576</v>
+        <v>3.4253166</v>
       </c>
       <c r="AD5" s="4" t="inlineStr"/>
       <c r="AE5" s="4" t="n">
@@ -9516,10 +9516,10 @@
       </c>
       <c r="AG5" s="4" t="inlineStr"/>
       <c r="AH5" s="4" t="n">
-        <v>2.136646</v>
+        <v>2.1633356</v>
       </c>
       <c r="AI5" s="4" t="n">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="AJ5" s="4" t="inlineStr"/>
       <c r="AK5" s="4" t="inlineStr">
@@ -9559,7 +9559,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Run Date: 12-Oct-2026 18:25 IST</t>
+          <t>Run Date: 13-Oct-2026 16:39 IST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>

</xml_diff>

<commit_message>
📈 Daily Screener Report — 21-Oct-2026 19:49 IST
</commit_message>
<xml_diff>
--- a/output/swing_screener_report.xlsx
+++ b/output/swing_screener_report.xlsx
@@ -517,7 +517,7 @@
     <col width="16" customWidth="1" min="25" max="25"/>
     <col width="14" customWidth="1" min="26" max="26"/>
     <col width="17" customWidth="1" min="27" max="27"/>
-    <col width="11" customWidth="1" min="28" max="28"/>
+    <col width="12" customWidth="1" min="28" max="28"/>
     <col width="13" customWidth="1" min="29" max="29"/>
     <col width="8" customWidth="1" min="30" max="30"/>
     <col width="13" customWidth="1" min="31" max="31"/>
@@ -816,13 +816,13 @@
         <v>3.72</v>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>137939</v>
+        <v>138932</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>6.2699513</v>
+        <v>6.315059</v>
       </c>
       <c r="AC2" s="2" t="n">
-        <v>6.559412</v>
+        <v>6.606602</v>
       </c>
       <c r="AD2" s="2" t="n">
         <v>16.29</v>
@@ -835,7 +835,7 @@
         <v>29.3</v>
       </c>
       <c r="AH2" s="2" t="n">
-        <v>0.96673405</v>
+        <v>0.973689</v>
       </c>
       <c r="AI2" s="2" t="n">
         <v>277</v>
@@ -946,13 +946,13 @@
         <v>3.54</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>86180</v>
+        <v>84981</v>
       </c>
       <c r="AB3" s="4" t="n">
-        <v>17.033691</v>
+        <v>16.796875</v>
       </c>
       <c r="AC3" s="4" t="n">
-        <v>14.115253</v>
+        <v>13.919011</v>
       </c>
       <c r="AD3" s="4" t="n">
         <v>13.27</v>
@@ -965,7 +965,7 @@
         <v>45.5</v>
       </c>
       <c r="AH3" s="4" t="n">
-        <v>2.0145292</v>
+        <v>1.9865216</v>
       </c>
       <c r="AI3" s="4" t="n">
         <v>34</v>
@@ -1076,13 +1076,13 @@
         <v>4.58</v>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>140099</v>
+        <v>140789</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>6.141058</v>
+        <v>6.1712847</v>
       </c>
       <c r="AC4" s="2" t="n">
-        <v>6.582365</v>
+        <v>6.6147637</v>
       </c>
       <c r="AD4" s="2" t="n">
         <v>15.06</v>
@@ -1095,7 +1095,7 @@
         <v>15</v>
       </c>
       <c r="AH4" s="2" t="n">
-        <v>0.8706459</v>
+        <v>0.8749312</v>
       </c>
       <c r="AI4" s="2" t="n">
         <v>246</v>
@@ -1206,13 +1206,13 @@
         <v>2</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>89263</v>
+        <v>91906</v>
       </c>
       <c r="AB5" s="4" t="n">
-        <v>49.772568</v>
+        <v>51.246502</v>
       </c>
       <c r="AC5" s="4" t="n">
-        <v>32.424732</v>
+        <v>33.47168</v>
       </c>
       <c r="AD5" s="4" t="n">
         <v>22.92</v>
@@ -1227,7 +1227,7 @@
         <v>-26.3</v>
       </c>
       <c r="AH5" s="4" t="n">
-        <v>10.38615</v>
+        <v>10.693719</v>
       </c>
       <c r="AI5" s="4" t="n">
         <v>63</v>
@@ -1340,13 +1340,13 @@
         <v>0.6</v>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>439995</v>
+        <v>435518</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>21.681372</v>
+        <v>21.460785</v>
       </c>
       <c r="AC6" s="2" t="n">
-        <v>18.82891</v>
+        <v>18.637344</v>
       </c>
       <c r="AD6" s="2" t="inlineStr"/>
       <c r="AE6" s="2" t="inlineStr"/>
@@ -1357,7 +1357,7 @@
         <v>22.5</v>
       </c>
       <c r="AH6" s="2" t="n">
-        <v>2.4275386</v>
+        <v>2.4028406</v>
       </c>
       <c r="AI6" s="2" t="n">
         <v>15</v>
@@ -1468,13 +1468,13 @@
         <v>2.27</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>991481</v>
+        <v>994353</v>
       </c>
       <c r="AB7" s="4" t="n">
-        <v>17.851603</v>
+        <v>17.903309</v>
       </c>
       <c r="AC7" s="4" t="n">
-        <v>14.7106085</v>
+        <v>14.753217</v>
       </c>
       <c r="AD7" s="4" t="n">
         <v>16.49</v>
@@ -1487,7 +1487,7 @@
         <v>22.1</v>
       </c>
       <c r="AH7" s="4" t="n">
-        <v>2.7235436</v>
+        <v>2.7314322</v>
       </c>
       <c r="AI7" s="4" t="n">
         <v>87</v>
@@ -1598,13 +1598,13 @@
         <v>2.03</v>
       </c>
       <c r="AA8" s="2" t="n">
-        <v>41135</v>
+        <v>40518</v>
       </c>
       <c r="AB8" s="2" t="n">
-        <v>46.91274</v>
+        <v>46.209423</v>
       </c>
       <c r="AC8" s="2" t="n">
-        <v>32.386745</v>
+        <v>31.901203</v>
       </c>
       <c r="AD8" s="2" t="n">
         <v>18.66</v>
@@ -1619,7 +1619,7 @@
         <v>402.1</v>
       </c>
       <c r="AH8" s="2" t="n">
-        <v>7.2864037</v>
+        <v>7.177166</v>
       </c>
       <c r="AI8" s="2" t="n">
         <v>7</v>
@@ -1732,13 +1732,13 @@
         <v>0.86</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>331646</v>
+        <v>324650</v>
       </c>
       <c r="AB9" s="4" t="n">
-        <v>35.57899</v>
+        <v>34.828526</v>
       </c>
       <c r="AC9" s="4" t="n">
-        <v>28.711098</v>
+        <v>28.105494</v>
       </c>
       <c r="AD9" s="4" t="inlineStr"/>
       <c r="AE9" s="4" t="n">
@@ -1751,7 +1751,7 @@
         <v>14.9</v>
       </c>
       <c r="AH9" s="4" t="n">
-        <v>8.080811499999999</v>
+        <v>7.9103627</v>
       </c>
       <c r="AI9" s="4" t="n">
         <v>91</v>
@@ -1862,13 +1862,13 @@
         <v>3.37</v>
       </c>
       <c r="AA10" s="2" t="n">
-        <v>28479</v>
+        <v>27181</v>
       </c>
       <c r="AB10" s="2" t="n">
-        <v>76.96013000000001</v>
+        <v>73.45417</v>
       </c>
       <c r="AC10" s="2" t="n">
-        <v>36.51351</v>
+        <v>34.850124</v>
       </c>
       <c r="AD10" s="2" t="inlineStr"/>
       <c r="AE10" s="2" t="n">
@@ -1881,7 +1881,7 @@
         <v>40.6</v>
       </c>
       <c r="AH10" s="2" t="n">
-        <v>15.620138</v>
+        <v>14.908556</v>
       </c>
       <c r="AI10" s="2" t="n">
         <v>34</v>
@@ -1939,19 +1939,19 @@
         </is>
       </c>
       <c r="J11" s="4" t="n">
-        <v>173.72</v>
+        <v>170.72</v>
       </c>
       <c r="K11" s="4" t="n">
         <v>0.58</v>
       </c>
       <c r="L11" s="4" t="n">
-        <v>173.39</v>
+        <v>170.4</v>
       </c>
       <c r="M11" s="4" t="n">
-        <v>171.36</v>
+        <v>168.4</v>
       </c>
       <c r="N11" s="4" t="n">
-        <v>164.38</v>
+        <v>161.55</v>
       </c>
       <c r="O11" s="4" t="inlineStr">
         <is>
@@ -1970,13 +1970,13 @@
         <v>50.84</v>
       </c>
       <c r="S11" s="4" t="n">
-        <v>1.4202</v>
+        <v>1.3957</v>
       </c>
       <c r="T11" s="4" t="n">
-        <v>1.1421</v>
+        <v>1.1223</v>
       </c>
       <c r="U11" s="4" t="n">
-        <v>0.2781</v>
+        <v>0.2733</v>
       </c>
       <c r="V11" s="4" t="inlineStr"/>
       <c r="W11" s="4" t="n">
@@ -1992,13 +1992,13 @@
         <v>0.68</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>30446</v>
+        <v>29360</v>
       </c>
       <c r="AB11" s="4" t="n">
-        <v>6.8963876</v>
+        <v>6.650258</v>
       </c>
       <c r="AC11" s="4" t="n">
-        <v>4.3053284</v>
+        <v>4.1516733</v>
       </c>
       <c r="AD11" s="4" t="inlineStr"/>
       <c r="AE11" s="4" t="n">
@@ -2009,7 +2009,7 @@
       </c>
       <c r="AG11" s="4" t="inlineStr"/>
       <c r="AH11" s="4" t="n">
-        <v>2.136646</v>
+        <v>2.06039</v>
       </c>
       <c r="AI11" s="4" t="n">
         <v>345</v>
@@ -2120,13 +2120,13 @@
         <v>0.85</v>
       </c>
       <c r="AA12" s="2" t="n">
-        <v>115415</v>
+        <v>115704</v>
       </c>
       <c r="AB12" s="2" t="n">
-        <v>8.731785</v>
+        <v>8.753695</v>
       </c>
       <c r="AC12" s="2" t="n">
-        <v>7.484807</v>
+        <v>7.5035877</v>
       </c>
       <c r="AD12" s="2" t="n">
         <v>16.14</v>
@@ -2139,7 +2139,7 @@
         <v>14</v>
       </c>
       <c r="AH12" s="2" t="n">
-        <v>1.3285382</v>
+        <v>1.3318717</v>
       </c>
       <c r="AI12" s="2" t="n">
         <v>213</v>
@@ -2251,10 +2251,10 @@
       </c>
       <c r="AA13" s="4" t="inlineStr"/>
       <c r="AB13" s="4" t="n">
-        <v>17.250105</v>
+        <v>17.727463</v>
       </c>
       <c r="AC13" s="4" t="n">
-        <v>15.272734</v>
+        <v>15.695374</v>
       </c>
       <c r="AD13" s="4" t="n">
         <v>45.57</v>
@@ -2269,7 +2269,7 @@
         <v>15</v>
       </c>
       <c r="AH13" s="4" t="n">
-        <v>7.4830317</v>
+        <v>7.690109</v>
       </c>
       <c r="AI13" s="4" t="n">
         <v>195</v>
@@ -2382,13 +2382,13 @@
         <v>1.26</v>
       </c>
       <c r="AA14" s="2" t="n">
-        <v>201746</v>
+        <v>196846</v>
       </c>
       <c r="AB14" s="2" t="n">
-        <v>34.97026</v>
+        <v>34.12087</v>
       </c>
       <c r="AC14" s="2" t="n">
-        <v>26.918304</v>
+        <v>26.264484</v>
       </c>
       <c r="AD14" s="2" t="inlineStr"/>
       <c r="AE14" s="2" t="n">
@@ -2401,7 +2401,7 @@
         <v>21.3</v>
       </c>
       <c r="AH14" s="2" t="n">
-        <v>8.031561999999999</v>
+        <v>7.8364835</v>
       </c>
       <c r="AI14" s="2" t="n">
         <v>112</v>
@@ -2512,13 +2512,13 @@
         <v>0.51</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>88966</v>
+        <v>89393</v>
       </c>
       <c r="AB15" s="4" t="n">
-        <v>26.104736</v>
+        <v>26.229969</v>
       </c>
       <c r="AC15" s="4" t="n">
-        <v>22.52757</v>
+        <v>22.635643</v>
       </c>
       <c r="AD15" s="4" t="n">
         <v>49.9</v>
@@ -2533,7 +2533,7 @@
         <v>120.2</v>
       </c>
       <c r="AH15" s="4" t="n">
-        <v>12.838401</v>
+        <v>12.899991</v>
       </c>
       <c r="AI15" s="4" t="n">
         <v>392</v>
@@ -2646,13 +2646,13 @@
         <v>0.64</v>
       </c>
       <c r="AA16" s="2" t="n">
-        <v>85285</v>
+        <v>86437</v>
       </c>
       <c r="AB16" s="2" t="n">
-        <v>39.422485</v>
+        <v>39.954945</v>
       </c>
       <c r="AC16" s="2" t="n">
-        <v>26.951775</v>
+        <v>27.3158</v>
       </c>
       <c r="AD16" s="2" t="inlineStr"/>
       <c r="AE16" s="2" t="n">
@@ -2665,7 +2665,7 @@
         <v>30.9</v>
       </c>
       <c r="AH16" s="2" t="n">
-        <v>6.779052</v>
+        <v>6.870613</v>
       </c>
       <c r="AI16" s="2" t="n">
         <v>83</v>
@@ -2780,13 +2780,13 @@
         <v>1.92</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>302999</v>
+        <v>298507</v>
       </c>
       <c r="AB17" s="4" t="n">
-        <v>12.247658</v>
+        <v>12.066108</v>
       </c>
       <c r="AC17" s="4" t="n">
-        <v>17.016588</v>
+        <v>16.764347</v>
       </c>
       <c r="AD17" s="4" t="inlineStr"/>
       <c r="AE17" s="4" t="n">
@@ -2799,7 +2799,7 @@
         <v>113</v>
       </c>
       <c r="AH17" s="4" t="n">
-        <v>3.0281963</v>
+        <v>2.9833088</v>
       </c>
       <c r="AI17" s="4" t="n">
         <v>57</v>
@@ -2910,13 +2910,13 @@
         <v>2.52</v>
       </c>
       <c r="AA18" s="2" t="n">
-        <v>147785</v>
+        <v>139001</v>
       </c>
       <c r="AB18" s="2" t="n">
-        <v>95.00068</v>
+        <v>89.35431</v>
       </c>
       <c r="AC18" s="2" t="n">
-        <v>66.50705000000001</v>
+        <v>62.5542</v>
       </c>
       <c r="AD18" s="2" t="n">
         <v>19.13</v>
@@ -2931,7 +2931,7 @@
         <v>3</v>
       </c>
       <c r="AH18" s="2" t="n">
-        <v>15.830176</v>
+        <v>14.889309</v>
       </c>
       <c r="AI18" s="2" t="n">
         <v>42</v>
@@ -3044,13 +3044,13 @@
         <v>0.95</v>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>4148</v>
+        <v>4046</v>
       </c>
       <c r="AB19" s="4" t="n">
-        <v>33.227352</v>
+        <v>32.41026</v>
       </c>
       <c r="AC19" s="4" t="n">
-        <v>22.799274</v>
+        <v>22.09054</v>
       </c>
       <c r="AD19" s="4" t="n">
         <v>16.49</v>
@@ -3065,7 +3065,7 @@
         <v>122.8</v>
       </c>
       <c r="AH19" s="4" t="n">
-        <v>5.1473665</v>
+        <v>5.0207877</v>
       </c>
       <c r="AI19" s="4" t="n">
         <v>77</v>
@@ -3178,13 +3178,13 @@
         <v>0.73</v>
       </c>
       <c r="AA20" s="2" t="n">
-        <v>166551</v>
+        <v>164361</v>
       </c>
       <c r="AB20" s="2" t="n">
-        <v>36.48861</v>
+        <v>36.008675</v>
       </c>
       <c r="AC20" s="2" t="n">
-        <v>26.693235</v>
+        <v>26.34214</v>
       </c>
       <c r="AD20" s="2" t="n">
         <v>10.31</v>
@@ -3199,7 +3199,7 @@
         <v>10.1</v>
       </c>
       <c r="AH20" s="2" t="n">
-        <v>3.658543</v>
+        <v>3.6104224</v>
       </c>
       <c r="AI20" s="2" t="n">
         <v>119</v>
@@ -3312,13 +3312,13 @@
         <v>1.12</v>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>157615</v>
+        <v>162540</v>
       </c>
       <c r="AB21" s="4" t="n">
-        <v>28.593699</v>
+        <v>29.4873</v>
       </c>
       <c r="AC21" s="4" t="n">
-        <v>19.936556</v>
+        <v>20.559607</v>
       </c>
       <c r="AD21" s="4" t="n">
         <v>19.19</v>
@@ -3333,7 +3333,7 @@
         <v>32.5</v>
       </c>
       <c r="AH21" s="4" t="n">
-        <v>5.312189</v>
+        <v>5.4782043</v>
       </c>
       <c r="AI21" s="4" t="n">
         <v>287</v>
@@ -3446,13 +3446,13 @@
         <v>0.29</v>
       </c>
       <c r="AA22" s="2" t="n">
-        <v>135485</v>
+        <v>131923</v>
       </c>
       <c r="AB22" s="2" t="n">
-        <v>48.530697</v>
+        <v>47.254875</v>
       </c>
       <c r="AC22" s="2" t="n">
-        <v>37.694603</v>
+        <v>36.70365</v>
       </c>
       <c r="AD22" s="2" t="inlineStr"/>
       <c r="AE22" s="2" t="n">
@@ -3465,7 +3465,7 @@
         <v>62.1</v>
       </c>
       <c r="AH22" s="2" t="n">
-        <v>17.180908</v>
+        <v>16.72924</v>
       </c>
       <c r="AI22" s="2" t="n">
         <v>30</v>
@@ -3576,13 +3576,13 @@
         <v>0.88</v>
       </c>
       <c r="AA23" s="4" t="n">
-        <v>241231</v>
+        <v>243966</v>
       </c>
       <c r="AB23" s="4" t="n">
-        <v>82.45168</v>
+        <v>83.38625999999999</v>
       </c>
       <c r="AC23" s="4" t="n">
-        <v>60.084335</v>
+        <v>60.76538</v>
       </c>
       <c r="AD23" s="4" t="inlineStr"/>
       <c r="AE23" s="4" t="n">
@@ -3595,7 +3595,7 @@
         <v>65.7</v>
       </c>
       <c r="AH23" s="4" t="n">
-        <v>14.39242</v>
+        <v>14.555556</v>
       </c>
       <c r="AI23" s="4" t="n">
         <v>33</v>
@@ -3706,13 +3706,13 @@
         <v>0.88</v>
       </c>
       <c r="AA24" s="2" t="n">
-        <v>373369</v>
+        <v>385355</v>
       </c>
       <c r="AB24" s="2" t="n">
-        <v>20.415743</v>
+        <v>21.071165</v>
       </c>
       <c r="AC24" s="2" t="n">
-        <v>17.226921</v>
+        <v>17.77997</v>
       </c>
       <c r="AD24" s="2" t="n">
         <v>24.65</v>
@@ -3727,7 +3727,7 @@
         <v>10.8</v>
       </c>
       <c r="AH24" s="2" t="n">
-        <v>4.951932</v>
+        <v>5.109936</v>
       </c>
       <c r="AI24" s="2" t="n">
         <v>348</v>
@@ -3840,13 +3840,13 @@
         <v>2.93</v>
       </c>
       <c r="AA25" s="4" t="n">
-        <v>12195</v>
+        <v>11850</v>
       </c>
       <c r="AB25" s="4" t="n">
-        <v>31.586494</v>
+        <v>30.6938</v>
       </c>
       <c r="AC25" s="4" t="n">
-        <v>20.238668</v>
+        <v>19.666685</v>
       </c>
       <c r="AD25" s="4" t="inlineStr"/>
       <c r="AE25" s="4" t="n">
@@ -3859,7 +3859,7 @@
         <v>19.8</v>
       </c>
       <c r="AH25" s="4" t="n">
-        <v>1.192247</v>
+        <v>1.1585519</v>
       </c>
       <c r="AI25" s="4" t="n">
         <v>0</v>
@@ -3970,13 +3970,13 @@
         <v>0.96</v>
       </c>
       <c r="AA26" s="2" t="n">
-        <v>7294</v>
+        <v>7423</v>
       </c>
       <c r="AB26" s="2" t="n">
-        <v>13.746888</v>
+        <v>13.989547</v>
       </c>
       <c r="AC26" s="2" t="n">
-        <v>11.994571</v>
+        <v>12.206297</v>
       </c>
       <c r="AD26" s="2" t="inlineStr"/>
       <c r="AE26" s="2" t="n">
@@ -3989,7 +3989,7 @@
         <v>22.2</v>
       </c>
       <c r="AH26" s="2" t="n">
-        <v>2.9441864</v>
+        <v>2.996157</v>
       </c>
       <c r="AI26" s="2" t="n">
         <v>217</v>
@@ -4100,13 +4100,13 @@
         <v>0.26</v>
       </c>
       <c r="AA27" s="4" t="n">
-        <v>7524</v>
+        <v>7247</v>
       </c>
       <c r="AB27" s="4" t="n">
-        <v>160.14165</v>
+        <v>154.23514</v>
       </c>
       <c r="AC27" s="4" t="n">
-        <v>66.89941</v>
+        <v>64.43195</v>
       </c>
       <c r="AD27" s="4" t="inlineStr"/>
       <c r="AE27" s="4" t="n">
@@ -4119,7 +4119,7 @@
         <v>-99.59999999999999</v>
       </c>
       <c r="AH27" s="4" t="n">
-        <v>2.6456933</v>
+        <v>2.5481122</v>
       </c>
       <c r="AI27" s="4" t="n">
         <v>0</v>
@@ -4230,13 +4230,13 @@
         <v>0.63</v>
       </c>
       <c r="AA28" s="2" t="n">
-        <v>44048</v>
+        <v>44250</v>
       </c>
       <c r="AB28" s="2" t="n">
-        <v>10.465075</v>
+        <v>10.513186</v>
       </c>
       <c r="AC28" s="2" t="n">
-        <v>10.33116</v>
+        <v>10.378655</v>
       </c>
       <c r="AD28" s="2" t="inlineStr"/>
       <c r="AE28" s="2" t="n">
@@ -4249,7 +4249,7 @@
         <v>35.1</v>
       </c>
       <c r="AH28" s="2" t="n">
-        <v>1.9761902</v>
+        <v>1.9852754</v>
       </c>
       <c r="AI28" s="2" t="n">
         <v>341</v>
@@ -4360,13 +4360,13 @@
         <v>0.28</v>
       </c>
       <c r="AA29" s="4" t="n">
-        <v>4580</v>
+        <v>4404</v>
       </c>
       <c r="AB29" s="4" t="n">
-        <v>23.983719</v>
+        <v>23.065115</v>
       </c>
       <c r="AC29" s="4" t="n">
-        <v>7.7599697</v>
+        <v>7.462754</v>
       </c>
       <c r="AD29" s="4" t="inlineStr"/>
       <c r="AE29" s="4" t="n">
@@ -4379,7 +4379,7 @@
         <v>18.5</v>
       </c>
       <c r="AH29" s="4" t="n">
-        <v>3.0520864</v>
+        <v>2.9351878</v>
       </c>
       <c r="AI29" s="4" t="n">
         <v>29</v>
@@ -4490,13 +4490,13 @@
         <v>0.91</v>
       </c>
       <c r="AA30" s="2" t="n">
-        <v>109942</v>
+        <v>108929</v>
       </c>
       <c r="AB30" s="2" t="n">
-        <v>50.43132</v>
+        <v>49.966824</v>
       </c>
       <c r="AC30" s="2" t="n">
-        <v>40.692547</v>
+        <v>40.317745</v>
       </c>
       <c r="AD30" s="2" t="inlineStr"/>
       <c r="AE30" s="2" t="n">
@@ -4509,7 +4509,7 @@
         <v>20.7</v>
       </c>
       <c r="AH30" s="2" t="n">
-        <v>8.288257</v>
+        <v>8.211918000000001</v>
       </c>
       <c r="AI30" s="2" t="n">
         <v>43</v>
@@ -4620,13 +4620,13 @@
         <v>0.99</v>
       </c>
       <c r="AA31" s="4" t="n">
-        <v>27703</v>
+        <v>26816</v>
       </c>
       <c r="AB31" s="4" t="n">
-        <v>24.506474</v>
+        <v>23.721685</v>
       </c>
       <c r="AC31" s="4" t="n">
-        <v>17.240358</v>
+        <v>16.688257</v>
       </c>
       <c r="AD31" s="4" t="n">
         <v>18.42</v>
@@ -4641,7 +4641,7 @@
         <v>57.2</v>
       </c>
       <c r="AH31" s="4" t="n">
-        <v>4.146475</v>
+        <v>4.013689</v>
       </c>
       <c r="AI31" s="4" t="n">
         <v>167</v>
@@ -4754,13 +4754,13 @@
         <v>0.77</v>
       </c>
       <c r="AA32" s="2" t="n">
-        <v>111791</v>
+        <v>108738</v>
       </c>
       <c r="AB32" s="2" t="n">
-        <v>102.27385</v>
+        <v>99.48097</v>
       </c>
       <c r="AC32" s="2" t="n">
-        <v>68.9789</v>
+        <v>67.09523</v>
       </c>
       <c r="AD32" s="2" t="inlineStr"/>
       <c r="AE32" s="2" t="n">
@@ -4773,7 +4773,7 @@
         <v>125.2</v>
       </c>
       <c r="AH32" s="2" t="n">
-        <v>21.074612</v>
+        <v>20.499107</v>
       </c>
       <c r="AI32" s="2" t="n">
         <v>12</v>
@@ -4884,13 +4884,13 @@
         <v>0.67</v>
       </c>
       <c r="AA33" s="4" t="n">
-        <v>166921</v>
+        <v>161919</v>
       </c>
       <c r="AB33" s="4" t="n">
-        <v>56.168728</v>
+        <v>54.4856</v>
       </c>
       <c r="AC33" s="4" t="n">
-        <v>37.94565</v>
+        <v>36.808582</v>
       </c>
       <c r="AD33" s="4" t="inlineStr"/>
       <c r="AE33" s="4" t="n">
@@ -4903,7 +4903,7 @@
         <v>124.1</v>
       </c>
       <c r="AH33" s="4" t="n">
-        <v>6.448245</v>
+        <v>6.2550197</v>
       </c>
       <c r="AI33" s="4" t="n">
         <v>0</v>
@@ -5014,13 +5014,13 @@
         <v>0.82</v>
       </c>
       <c r="AA34" s="2" t="n">
-        <v>96473</v>
+        <v>94481</v>
       </c>
       <c r="AB34" s="2" t="n">
-        <v>378.25842</v>
+        <v>370.44946</v>
       </c>
       <c r="AC34" s="2" t="n">
-        <v>116.61742</v>
+        <v>114.20991</v>
       </c>
       <c r="AD34" s="2" t="inlineStr"/>
       <c r="AE34" s="2" t="n">
@@ -5033,7 +5033,7 @@
         <v>250</v>
       </c>
       <c r="AH34" s="2" t="n">
-        <v>67.03505</v>
+        <v>65.65114</v>
       </c>
       <c r="AI34" s="2" t="n">
         <v>0</v>
@@ -5144,13 +5144,13 @@
         <v>1.3</v>
       </c>
       <c r="AA35" s="4" t="n">
-        <v>47718</v>
+        <v>49149</v>
       </c>
       <c r="AB35" s="4" t="n">
-        <v>25.010004</v>
+        <v>25.760303</v>
       </c>
       <c r="AC35" s="4" t="n">
-        <v>19.701529</v>
+        <v>20.292574</v>
       </c>
       <c r="AD35" s="4" t="n">
         <v>17.74</v>
@@ -5165,7 +5165,7 @@
         <v>10.7</v>
       </c>
       <c r="AH35" s="4" t="n">
-        <v>4.20835</v>
+        <v>4.334601</v>
       </c>
       <c r="AI35" s="4" t="n">
         <v>248</v>
@@ -5278,13 +5278,13 @@
         <v>0.73</v>
       </c>
       <c r="AA36" s="2" t="n">
-        <v>104674</v>
+        <v>103143</v>
       </c>
       <c r="AB36" s="2" t="n">
-        <v>19.277554</v>
+        <v>18.995577</v>
       </c>
       <c r="AC36" s="2" t="n">
-        <v>16.167715</v>
+        <v>15.931229</v>
       </c>
       <c r="AD36" s="2" t="inlineStr"/>
       <c r="AE36" s="2" t="n">
@@ -5297,7 +5297,7 @@
         <v>-17.2</v>
       </c>
       <c r="AH36" s="2" t="n">
-        <v>4.8422565</v>
+        <v>4.771428</v>
       </c>
       <c r="AI36" s="2" t="n">
         <v>354</v>
@@ -5408,13 +5408,13 @@
         <v>0.77</v>
       </c>
       <c r="AA37" s="4" t="n">
-        <v>3791</v>
+        <v>3636</v>
       </c>
       <c r="AB37" s="4" t="n">
-        <v>38.375473</v>
+        <v>36.801517</v>
       </c>
       <c r="AC37" s="4" t="n">
-        <v>18.10694</v>
+        <v>17.36429</v>
       </c>
       <c r="AD37" s="4" t="inlineStr"/>
       <c r="AE37" s="4" t="n">
@@ -5427,7 +5427,7 @@
         <v>32</v>
       </c>
       <c r="AH37" s="4" t="n">
-        <v>4.202722</v>
+        <v>4.030349</v>
       </c>
       <c r="AI37" s="4" t="n">
         <v>16</v>
@@ -5538,13 +5538,13 @@
         <v>0.51</v>
       </c>
       <c r="AA38" s="2" t="n">
-        <v>46746</v>
+        <v>46437</v>
       </c>
       <c r="AB38" s="2" t="n">
-        <v>37.357643</v>
+        <v>37.110798</v>
       </c>
       <c r="AC38" s="2" t="n">
-        <v>31.442703</v>
+        <v>31.234941</v>
       </c>
       <c r="AD38" s="2" t="inlineStr"/>
       <c r="AE38" s="2" t="n">
@@ -5557,7 +5557,7 @@
         <v>269</v>
       </c>
       <c r="AH38" s="2" t="n">
-        <v>7.720222</v>
+        <v>7.66921</v>
       </c>
       <c r="AI38" s="2" t="n">
         <v>101</v>
@@ -5668,13 +5668,13 @@
         <v>0.86</v>
       </c>
       <c r="AA39" s="4" t="n">
-        <v>406879</v>
+        <v>402916</v>
       </c>
       <c r="AB39" s="4" t="n">
-        <v>30.141663</v>
+        <v>29.848097</v>
       </c>
       <c r="AC39" s="4" t="n">
-        <v>22.578596</v>
+        <v>22.358692</v>
       </c>
       <c r="AD39" s="4" t="inlineStr"/>
       <c r="AE39" s="4" t="n">
@@ -5687,7 +5687,7 @@
         <v>2.4</v>
       </c>
       <c r="AH39" s="4" t="n">
-        <v>4.240147</v>
+        <v>4.19885</v>
       </c>
       <c r="AI39" s="4" t="n">
         <v>42</v>
@@ -5798,13 +5798,13 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="AA40" s="2" t="n">
-        <v>20459</v>
+        <v>19962</v>
       </c>
       <c r="AB40" s="2" t="n">
-        <v>74.937935</v>
+        <v>73.11723000000001</v>
       </c>
       <c r="AC40" s="2" t="n">
-        <v>23.443365</v>
+        <v>22.873785</v>
       </c>
       <c r="AD40" s="2" t="inlineStr"/>
       <c r="AE40" s="2" t="n">
@@ -5817,7 +5817,7 @@
         <v>83.7</v>
       </c>
       <c r="AH40" s="2" t="n">
-        <v>4.2388186</v>
+        <v>4.1358323</v>
       </c>
       <c r="AI40" s="2" t="n">
         <v>5</v>
@@ -5929,10 +5929,10 @@
       </c>
       <c r="AA41" s="4" t="inlineStr"/>
       <c r="AB41" s="4" t="n">
-        <v>66.510025</v>
+        <v>64.47369</v>
       </c>
       <c r="AC41" s="4" t="n">
-        <v>38.242786</v>
+        <v>37.071903</v>
       </c>
       <c r="AD41" s="4" t="inlineStr"/>
       <c r="AE41" s="4" t="n">
@@ -5945,7 +5945,7 @@
         <v>103.4</v>
       </c>
       <c r="AH41" s="4" t="n">
-        <v>19.260195</v>
+        <v>18.670506</v>
       </c>
       <c r="AI41" s="4" t="n">
         <v>25</v>
@@ -6184,13 +6184,13 @@
         <v>0.37</v>
       </c>
       <c r="AA43" s="4" t="n">
-        <v>58327</v>
+        <v>55696</v>
       </c>
       <c r="AB43" s="4" t="n">
-        <v>27.129963</v>
+        <v>25.906136</v>
       </c>
       <c r="AC43" s="4" t="n">
-        <v>18.581055</v>
+        <v>17.742867</v>
       </c>
       <c r="AD43" s="4" t="n">
         <v>4.04</v>
@@ -6203,7 +6203,7 @@
         <v>2.6</v>
       </c>
       <c r="AH43" s="4" t="n">
-        <v>1.3383126</v>
+        <v>1.2779416</v>
       </c>
       <c r="AI43" s="4" t="n">
         <v>27</v>
@@ -6314,13 +6314,13 @@
         <v>0.82</v>
       </c>
       <c r="AA44" s="2" t="n">
-        <v>168124</v>
+        <v>167188</v>
       </c>
       <c r="AB44" s="2" t="n">
-        <v>38.108433</v>
+        <v>37.896385</v>
       </c>
       <c r="AC44" s="2" t="n">
-        <v>22.717804</v>
+        <v>22.591396</v>
       </c>
       <c r="AD44" s="2" t="inlineStr"/>
       <c r="AE44" s="2" t="n">
@@ -6333,7 +6333,7 @@
         <v>104.2</v>
       </c>
       <c r="AH44" s="2" t="n">
-        <v>4.064299</v>
+        <v>4.041684</v>
       </c>
       <c r="AI44" s="2" t="n">
         <v>32</v>
@@ -6444,13 +6444,13 @@
         <v>0.45</v>
       </c>
       <c r="AA45" s="4" t="n">
-        <v>30016</v>
+        <v>28330</v>
       </c>
       <c r="AB45" s="4" t="n">
-        <v>19.664614</v>
+        <v>18.56</v>
       </c>
       <c r="AC45" s="4" t="n">
-        <v>10.440804</v>
+        <v>9.854316000000001</v>
       </c>
       <c r="AD45" s="4" t="inlineStr"/>
       <c r="AE45" s="4" t="n">
@@ -6463,7 +6463,7 @@
         <v>288.5</v>
       </c>
       <c r="AH45" s="4" t="n">
-        <v>1.8701023</v>
+        <v>1.7650536</v>
       </c>
       <c r="AI45" s="4" t="n">
         <v>125</v>
@@ -6483,32 +6483,32 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>RADICO</t>
+          <t>SYRMA</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Radico Khaitan Limited</t>
+          <t>Syrma SGS Technology Limited</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Consumer Defensive</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>Beverages - Wineries &amp; Distilleries</t>
+          <t>Electronic Components</t>
         </is>
       </c>
       <c r="E46" s="6" t="n">
-        <v>36.2</v>
+        <v>37</v>
       </c>
       <c r="F46" s="2" t="n">
-        <v>21.6</v>
+        <v>16.8</v>
       </c>
       <c r="G46" s="2" t="n">
-        <v>14.6</v>
+        <v>20.2</v>
       </c>
       <c r="H46" s="6" t="inlineStr">
         <is>
@@ -6517,23 +6517,23 @@
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t>📈 EMA Bull Stack | 🏆 Near 52W High | 📉 Tight Base</t>
+          <t>✅ Supertrend Buy | 📈 EMA Bull Stack</t>
         </is>
       </c>
       <c r="J46" s="2" t="n">
-        <v>4435.5</v>
+        <v>1547.6</v>
       </c>
       <c r="K46" s="2" t="n">
-        <v>-0.85</v>
+        <v>-3.55</v>
       </c>
       <c r="L46" s="2" t="n">
-        <v>4468.51</v>
+        <v>1663.53</v>
       </c>
       <c r="M46" s="2" t="n">
-        <v>4413.4</v>
+        <v>1588.39</v>
       </c>
       <c r="N46" s="2" t="n">
-        <v>3825.24</v>
+        <v>1256.88</v>
       </c>
       <c r="O46" s="2" t="inlineStr">
         <is>
@@ -6542,103 +6542,103 @@
       </c>
       <c r="P46" s="2" t="inlineStr">
         <is>
-          <t>Sell</t>
+          <t>Buy</t>
         </is>
       </c>
       <c r="Q46" s="2" t="n">
-        <v>93.44</v>
+        <v>84.91</v>
       </c>
       <c r="R46" s="2" t="n">
-        <v>48.2</v>
+        <v>39.99</v>
       </c>
       <c r="S46" s="2" t="n">
-        <v>5.5657</v>
+        <v>12.6515</v>
       </c>
       <c r="T46" s="2" t="n">
-        <v>3.0461</v>
+        <v>37.6504</v>
       </c>
       <c r="U46" s="2" t="n">
-        <v>2.5196</v>
+        <v>-24.9989</v>
       </c>
       <c r="V46" s="2" t="inlineStr"/>
       <c r="W46" s="2" t="n">
-        <v>17.22</v>
+        <v>21.73</v>
       </c>
       <c r="X46" s="2" t="n">
-        <v>143055</v>
+        <v>838862</v>
       </c>
       <c r="Y46" s="2" t="n">
-        <v>302844</v>
+        <v>1413652</v>
       </c>
       <c r="Z46" s="2" t="n">
-        <v>0.47</v>
+        <v>0.59</v>
       </c>
       <c r="AA46" s="2" t="n">
-        <v>59431</v>
+        <v>28376</v>
       </c>
       <c r="AB46" s="2" t="n">
-        <v>84.43747</v>
+        <v>76.60426</v>
       </c>
       <c r="AC46" s="2" t="n">
-        <v>54.395134</v>
+        <v>45.740376</v>
       </c>
       <c r="AD46" s="2" t="inlineStr"/>
       <c r="AE46" s="2" t="n">
-        <v>15.033</v>
+        <v>13.045</v>
       </c>
       <c r="AF46" s="2" t="n">
-        <v>11.8</v>
+        <v>68.3</v>
       </c>
       <c r="AG46" s="2" t="n">
-        <v>76</v>
+        <v>86</v>
       </c>
       <c r="AH46" s="2" t="n">
-        <v>17.911732</v>
+        <v>9.845411</v>
       </c>
       <c r="AI46" s="2" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="AJ46" s="2" t="inlineStr"/>
       <c r="AK46" s="2" t="inlineStr">
         <is>
-          <t>https://www.screener.in/company/RADICO/</t>
+          <t>https://www.screener.in/company/SYRMA/</t>
         </is>
       </c>
       <c r="AL46" s="2" t="inlineStr">
         <is>
-          <t>https://www.tradingview.com/chart/?symbol=NSE:RADICO</t>
+          <t>https://www.tradingview.com/chart/?symbol=NSE:SYRMA</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
         <is>
-          <t>BHEL</t>
+          <t>RADICO</t>
         </is>
       </c>
       <c r="B47" s="4" t="inlineStr">
         <is>
-          <t>Bharat Heavy Electricals Limited</t>
+          <t>Radico Khaitan Limited</t>
         </is>
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Consumer Defensive</t>
         </is>
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>Specialty Industrial Machinery</t>
+          <t>Beverages - Wineries &amp; Distilleries</t>
         </is>
       </c>
       <c r="E47" s="6" t="n">
-        <v>35.8</v>
+        <v>36.2</v>
       </c>
       <c r="F47" s="4" t="n">
-        <v>16.8</v>
+        <v>21.6</v>
       </c>
       <c r="G47" s="4" t="n">
-        <v>19</v>
+        <v>14.6</v>
       </c>
       <c r="H47" s="6" t="inlineStr">
         <is>
@@ -6647,23 +6647,23 @@
       </c>
       <c r="I47" s="4" t="inlineStr">
         <is>
-          <t>✅ Supertrend Buy | 📈 EMA Bull Stack | 🏆 Near 52W High | 📉 Tight Base</t>
+          <t>📈 EMA Bull Stack | 🏆 Near 52W High | 📉 Tight Base</t>
         </is>
       </c>
       <c r="J47" s="4" t="n">
-        <v>427.35</v>
+        <v>4435.5</v>
       </c>
       <c r="K47" s="4" t="n">
-        <v>-1.67</v>
+        <v>-0.85</v>
       </c>
       <c r="L47" s="4" t="n">
-        <v>433.11</v>
+        <v>4468.51</v>
       </c>
       <c r="M47" s="4" t="n">
-        <v>425</v>
+        <v>4413.4</v>
       </c>
       <c r="N47" s="4" t="n">
-        <v>367.65</v>
+        <v>3825.24</v>
       </c>
       <c r="O47" s="4" t="inlineStr">
         <is>
@@ -6672,107 +6672,103 @@
       </c>
       <c r="P47" s="4" t="inlineStr">
         <is>
-          <t>Buy</t>
+          <t>Sell</t>
         </is>
       </c>
       <c r="Q47" s="4" t="n">
-        <v>92.09999999999999</v>
+        <v>93.44</v>
       </c>
       <c r="R47" s="4" t="n">
-        <v>48.35</v>
+        <v>48.2</v>
       </c>
       <c r="S47" s="4" t="n">
-        <v>4.0663</v>
+        <v>5.5657</v>
       </c>
       <c r="T47" s="4" t="n">
-        <v>4.2666</v>
+        <v>3.0461</v>
       </c>
       <c r="U47" s="4" t="n">
-        <v>-0.2003</v>
+        <v>2.5196</v>
       </c>
       <c r="V47" s="4" t="inlineStr"/>
       <c r="W47" s="4" t="n">
-        <v>12.92</v>
+        <v>17.22</v>
       </c>
       <c r="X47" s="4" t="n">
-        <v>8639491</v>
+        <v>143055</v>
       </c>
       <c r="Y47" s="4" t="n">
-        <v>11912629</v>
+        <v>302844</v>
       </c>
       <c r="Z47" s="4" t="n">
-        <v>0.73</v>
+        <v>0.47</v>
       </c>
       <c r="AA47" s="4" t="n">
-        <v>148806</v>
+        <v>58367</v>
       </c>
       <c r="AB47" s="4" t="n">
-        <v>51.674725</v>
+        <v>82.92595</v>
       </c>
       <c r="AC47" s="4" t="n">
-        <v>26.482666</v>
-      </c>
-      <c r="AD47" s="4" t="n">
-        <v>11.25</v>
-      </c>
+        <v>53.421406</v>
+      </c>
+      <c r="AD47" s="4" t="inlineStr"/>
       <c r="AE47" s="4" t="n">
-        <v>22.496</v>
+        <v>15.033</v>
       </c>
       <c r="AF47" s="4" t="n">
-        <v>23.8</v>
+        <v>11.8</v>
       </c>
       <c r="AG47" s="4" t="n">
-        <v>118.5</v>
+        <v>76</v>
       </c>
       <c r="AH47" s="4" t="n">
-        <v>5.5567117</v>
+        <v>17.591093</v>
       </c>
       <c r="AI47" s="4" t="n">
-        <v>33</v>
-      </c>
-      <c r="AJ47" s="4" t="n">
-        <v>1.673</v>
-      </c>
+        <v>20</v>
+      </c>
+      <c r="AJ47" s="4" t="inlineStr"/>
       <c r="AK47" s="4" t="inlineStr">
         <is>
-          <t>https://www.screener.in/company/BHEL/</t>
+          <t>https://www.screener.in/company/RADICO/</t>
         </is>
       </c>
       <c r="AL47" s="4" t="inlineStr">
         <is>
-          <t>https://www.tradingview.com/chart/?symbol=NSE:BHEL</t>
+          <t>https://www.tradingview.com/chart/?symbol=NSE:RADICO</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>DRREDDY</t>
+          <t>BHEL</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Dr. Reddy's Laboratories Limited</t>
+          <t>Bharat Heavy Electricals Limited</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>Drug Manufacturers - Specialty &amp; Generic</t>
+          <t>Specialty Industrial Machinery</t>
         </is>
       </c>
       <c r="E48" s="6" t="n">
-        <v>35.5</v>
+        <v>35.8</v>
       </c>
       <c r="F48" s="2" t="n">
-        <v>26.2</v>
+        <v>16.8</v>
       </c>
       <c r="G48" s="2" t="n">
-        <v>9.300000000000001</v>
+        <v>19</v>
       </c>
       <c r="H48" s="6" t="inlineStr">
         <is>
@@ -6781,27 +6777,27 @@
       </c>
       <c r="I48" s="2" t="inlineStr">
         <is>
-          <t>✅ Supertrend Buy | 📉 Tight Base</t>
+          <t>✅ Supertrend Buy | 📈 EMA Bull Stack | 🏆 Near 52W High | 📉 Tight Base</t>
         </is>
       </c>
       <c r="J48" s="2" t="n">
-        <v>1242.5</v>
+        <v>427.35</v>
       </c>
       <c r="K48" s="2" t="n">
-        <v>0.77</v>
+        <v>-1.67</v>
       </c>
       <c r="L48" s="2" t="n">
-        <v>1211.75</v>
+        <v>433.11</v>
       </c>
       <c r="M48" s="2" t="n">
-        <v>1203.41</v>
+        <v>425</v>
       </c>
       <c r="N48" s="2" t="n">
-        <v>1230.5</v>
+        <v>367.65</v>
       </c>
       <c r="O48" s="2" t="inlineStr">
         <is>
-          <t>✗</t>
+          <t>✓</t>
         </is>
       </c>
       <c r="P48" s="2" t="inlineStr">
@@ -6810,103 +6806,103 @@
         </is>
       </c>
       <c r="Q48" s="2" t="n">
-        <v>88.37</v>
+        <v>92.09999999999999</v>
       </c>
       <c r="R48" s="2" t="n">
-        <v>59.94</v>
+        <v>48.35</v>
       </c>
       <c r="S48" s="2" t="n">
-        <v>12.2926</v>
+        <v>4.0663</v>
       </c>
       <c r="T48" s="2" t="n">
-        <v>10.1166</v>
+        <v>4.2666</v>
       </c>
       <c r="U48" s="2" t="n">
-        <v>2.1759</v>
+        <v>-0.2003</v>
       </c>
       <c r="V48" s="2" t="inlineStr"/>
       <c r="W48" s="2" t="n">
-        <v>22.2</v>
+        <v>12.92</v>
       </c>
       <c r="X48" s="2" t="n">
-        <v>1023837</v>
+        <v>8639491</v>
       </c>
       <c r="Y48" s="2" t="n">
-        <v>2191924</v>
+        <v>11912629</v>
       </c>
       <c r="Z48" s="2" t="n">
-        <v>0.47</v>
+        <v>0.73</v>
       </c>
       <c r="AA48" s="2" t="n">
-        <v>103499</v>
+        <v>142834</v>
       </c>
       <c r="AB48" s="2" t="n">
-        <v>31.265726</v>
+        <v>49.600967</v>
       </c>
       <c r="AC48" s="2" t="n">
-        <v>21.080463</v>
+        <v>25.41989</v>
       </c>
       <c r="AD48" s="2" t="n">
-        <v>8.84</v>
+        <v>11.25</v>
       </c>
       <c r="AE48" s="2" t="n">
-        <v>18.605</v>
+        <v>22.496</v>
       </c>
       <c r="AF48" s="2" t="n">
-        <v>-5.6</v>
+        <v>23.8</v>
       </c>
       <c r="AG48" s="2" t="n">
-        <v>-68.7</v>
+        <v>118.5</v>
       </c>
       <c r="AH48" s="2" t="n">
-        <v>2.6992912</v>
+        <v>5.333715</v>
       </c>
       <c r="AI48" s="2" t="n">
-        <v>64</v>
+        <v>33</v>
       </c>
       <c r="AJ48" s="2" t="n">
-        <v>1.902</v>
+        <v>1.673</v>
       </c>
       <c r="AK48" s="2" t="inlineStr">
         <is>
-          <t>https://www.screener.in/company/DRREDDY/</t>
+          <t>https://www.screener.in/company/BHEL/</t>
         </is>
       </c>
       <c r="AL48" s="2" t="inlineStr">
         <is>
-          <t>https://www.tradingview.com/chart/?symbol=NSE:DRREDDY</t>
+          <t>https://www.tradingview.com/chart/?symbol=NSE:BHEL</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
         <is>
-          <t>ADANIGREEN</t>
+          <t>DRREDDY</t>
         </is>
       </c>
       <c r="B49" s="4" t="inlineStr">
         <is>
-          <t>Adani Green Energy Limited</t>
+          <t>Dr. Reddy's Laboratories Limited</t>
         </is>
       </c>
       <c r="C49" s="4" t="inlineStr">
         <is>
-          <t>Utilities</t>
+          <t>Healthcare</t>
         </is>
       </c>
       <c r="D49" s="4" t="inlineStr">
         <is>
-          <t>Utilities - Renewable</t>
+          <t>Drug Manufacturers - Specialty &amp; Generic</t>
         </is>
       </c>
       <c r="E49" s="6" t="n">
-        <v>35.1</v>
+        <v>35.5</v>
       </c>
       <c r="F49" s="4" t="n">
-        <v>19</v>
+        <v>26.2</v>
       </c>
       <c r="G49" s="4" t="n">
-        <v>16.1</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="H49" s="6" t="inlineStr">
         <is>
@@ -6915,23 +6911,23 @@
       </c>
       <c r="I49" s="4" t="inlineStr">
         <is>
-          <t>📉 Tight Base</t>
+          <t>✅ Supertrend Buy | 📉 Tight Base</t>
         </is>
       </c>
       <c r="J49" s="4" t="n">
-        <v>1295.2</v>
+        <v>1242.5</v>
       </c>
       <c r="K49" s="4" t="n">
-        <v>-0.52</v>
+        <v>0.77</v>
       </c>
       <c r="L49" s="4" t="n">
-        <v>1291.44</v>
+        <v>1211.75</v>
       </c>
       <c r="M49" s="4" t="n">
-        <v>1310.61</v>
+        <v>1203.41</v>
       </c>
       <c r="N49" s="4" t="n">
-        <v>1246.25</v>
+        <v>1230.5</v>
       </c>
       <c r="O49" s="4" t="inlineStr">
         <is>
@@ -6940,103 +6936,107 @@
       </c>
       <c r="P49" s="4" t="inlineStr">
         <is>
-          <t>Sell</t>
+          <t>Buy</t>
         </is>
       </c>
       <c r="Q49" s="4" t="n">
-        <v>79.39</v>
+        <v>88.37</v>
       </c>
       <c r="R49" s="4" t="n">
-        <v>50.16</v>
+        <v>59.94</v>
       </c>
       <c r="S49" s="4" t="n">
-        <v>-1.5252</v>
+        <v>12.2926</v>
       </c>
       <c r="T49" s="4" t="n">
-        <v>-5.8828</v>
+        <v>10.1166</v>
       </c>
       <c r="U49" s="4" t="n">
-        <v>4.3576</v>
+        <v>2.1759</v>
       </c>
       <c r="V49" s="4" t="inlineStr"/>
       <c r="W49" s="4" t="n">
-        <v>11.13</v>
+        <v>22.2</v>
       </c>
       <c r="X49" s="4" t="n">
-        <v>965167</v>
+        <v>1023837</v>
       </c>
       <c r="Y49" s="4" t="n">
-        <v>2211497</v>
+        <v>2191924</v>
       </c>
       <c r="Z49" s="4" t="n">
-        <v>0.44</v>
+        <v>0.47</v>
       </c>
       <c r="AA49" s="4" t="n">
-        <v>213342</v>
+        <v>103665</v>
       </c>
       <c r="AB49" s="4" t="n">
-        <v>124.0613</v>
+        <v>31.316053</v>
       </c>
       <c r="AC49" s="4" t="n">
-        <v>44.04468</v>
-      </c>
-      <c r="AD49" s="4" t="inlineStr"/>
+        <v>21.114395</v>
+      </c>
+      <c r="AD49" s="4" t="n">
+        <v>8.84</v>
+      </c>
       <c r="AE49" s="4" t="n">
-        <v>346.548</v>
+        <v>18.605</v>
       </c>
       <c r="AF49" s="4" t="n">
-        <v>16.6</v>
+        <v>-5.6</v>
       </c>
       <c r="AG49" s="4" t="n">
-        <v>18.5</v>
+        <v>-68.7</v>
       </c>
       <c r="AH49" s="4" t="n">
-        <v>11.059687</v>
+        <v>2.7036362</v>
       </c>
       <c r="AI49" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ49" s="4" t="inlineStr"/>
+        <v>64</v>
+      </c>
+      <c r="AJ49" s="4" t="n">
+        <v>1.902</v>
+      </c>
       <c r="AK49" s="4" t="inlineStr">
         <is>
-          <t>https://www.screener.in/company/ADANIGREEN/</t>
+          <t>https://www.screener.in/company/DRREDDY/</t>
         </is>
       </c>
       <c r="AL49" s="4" t="inlineStr">
         <is>
-          <t>https://www.tradingview.com/chart/?symbol=NSE:ADANIGREEN</t>
+          <t>https://www.tradingview.com/chart/?symbol=NSE:DRREDDY</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>SYRMA</t>
+          <t>AUROPHARMA</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>Syrma SGS Technology Limited</t>
+          <t>Aurobindo Pharma Limited</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Healthcare</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>Electronic Components</t>
+          <t>Drug Manufacturers - Specialty &amp; Generic</t>
         </is>
       </c>
       <c r="E50" s="6" t="n">
-        <v>34.90000000000001</v>
+        <v>35.3</v>
       </c>
       <c r="F50" s="2" t="n">
-        <v>16.8</v>
+        <v>14.4</v>
       </c>
       <c r="G50" s="2" t="n">
-        <v>18.1</v>
+        <v>20.9</v>
       </c>
       <c r="H50" s="6" t="inlineStr">
         <is>
@@ -7045,23 +7045,23 @@
       </c>
       <c r="I50" s="2" t="inlineStr">
         <is>
-          <t>✅ Supertrend Buy | 📈 EMA Bull Stack</t>
+          <t>✅ Supertrend Buy | 📈 EMA Bull Stack | 🏆 Near 52W High | 📉 Tight Base</t>
         </is>
       </c>
       <c r="J50" s="2" t="n">
-        <v>1547.6</v>
+        <v>1621.4</v>
       </c>
       <c r="K50" s="2" t="n">
-        <v>-3.55</v>
+        <v>-2.73</v>
       </c>
       <c r="L50" s="2" t="n">
-        <v>1663.53</v>
+        <v>1674.46</v>
       </c>
       <c r="M50" s="2" t="n">
-        <v>1588.39</v>
+        <v>1653.98</v>
       </c>
       <c r="N50" s="2" t="n">
-        <v>1256.88</v>
+        <v>1476.7</v>
       </c>
       <c r="O50" s="2" t="inlineStr">
         <is>
@@ -7074,99 +7074,99 @@
         </is>
       </c>
       <c r="Q50" s="2" t="n">
-        <v>84.91</v>
+        <v>93.18000000000001</v>
       </c>
       <c r="R50" s="2" t="n">
-        <v>39.99</v>
+        <v>40.47</v>
       </c>
       <c r="S50" s="2" t="n">
-        <v>12.6515</v>
+        <v>-2.5029</v>
       </c>
       <c r="T50" s="2" t="n">
-        <v>37.6504</v>
+        <v>5.0185</v>
       </c>
       <c r="U50" s="2" t="n">
-        <v>-24.9989</v>
+        <v>-7.5214</v>
       </c>
       <c r="V50" s="2" t="inlineStr"/>
       <c r="W50" s="2" t="n">
-        <v>21.73</v>
+        <v>15.95</v>
       </c>
       <c r="X50" s="2" t="n">
-        <v>838862</v>
+        <v>736433</v>
       </c>
       <c r="Y50" s="2" t="n">
-        <v>1413652</v>
+        <v>854057</v>
       </c>
       <c r="Z50" s="2" t="n">
-        <v>0.59</v>
+        <v>0.86</v>
       </c>
       <c r="AA50" s="2" t="n">
-        <v>29811</v>
+        <v>90841</v>
       </c>
       <c r="AB50" s="2" t="n">
-        <v>80.47842</v>
+        <v>24.66875</v>
       </c>
       <c r="AC50" s="2" t="n">
-        <v>48.053635</v>
+        <v>16.898243</v>
       </c>
       <c r="AD50" s="2" t="inlineStr"/>
       <c r="AE50" s="2" t="n">
-        <v>13.045</v>
+        <v>21.31</v>
       </c>
       <c r="AF50" s="2" t="n">
-        <v>68.3</v>
+        <v>16.3</v>
       </c>
       <c r="AG50" s="2" t="n">
-        <v>86</v>
+        <v>25.8</v>
       </c>
       <c r="AH50" s="2" t="n">
-        <v>10.343329</v>
+        <v>2.4200213</v>
       </c>
       <c r="AI50" s="2" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="AJ50" s="2" t="inlineStr"/>
       <c r="AK50" s="2" t="inlineStr">
         <is>
-          <t>https://www.screener.in/company/SYRMA/</t>
+          <t>https://www.screener.in/company/AUROPHARMA/</t>
         </is>
       </c>
       <c r="AL50" s="2" t="inlineStr">
         <is>
-          <t>https://www.tradingview.com/chart/?symbol=NSE:SYRMA</t>
+          <t>https://www.tradingview.com/chart/?symbol=NSE:AUROPHARMA</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
         <is>
-          <t>AUROPHARMA</t>
+          <t>ADANIGREEN</t>
         </is>
       </c>
       <c r="B51" s="4" t="inlineStr">
         <is>
-          <t>Aurobindo Pharma Limited</t>
+          <t>Adani Green Energy Limited</t>
         </is>
       </c>
       <c r="C51" s="4" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Utilities</t>
         </is>
       </c>
       <c r="D51" s="4" t="inlineStr">
         <is>
-          <t>Drug Manufacturers - Specialty &amp; Generic</t>
+          <t>Utilities - Renewable</t>
         </is>
       </c>
       <c r="E51" s="6" t="n">
-        <v>33.6</v>
+        <v>35.1</v>
       </c>
       <c r="F51" s="4" t="n">
-        <v>14.4</v>
+        <v>19</v>
       </c>
       <c r="G51" s="4" t="n">
-        <v>19.2</v>
+        <v>16.1</v>
       </c>
       <c r="H51" s="6" t="inlineStr">
         <is>
@@ -7175,83 +7175,83 @@
       </c>
       <c r="I51" s="4" t="inlineStr">
         <is>
-          <t>✅ Supertrend Buy | 📈 EMA Bull Stack | 🏆 Near 52W High | 📉 Tight Base</t>
+          <t>📉 Tight Base</t>
         </is>
       </c>
       <c r="J51" s="4" t="n">
-        <v>1621.4</v>
+        <v>1295.2</v>
       </c>
       <c r="K51" s="4" t="n">
-        <v>-2.73</v>
+        <v>-0.52</v>
       </c>
       <c r="L51" s="4" t="n">
-        <v>1674.46</v>
+        <v>1291.44</v>
       </c>
       <c r="M51" s="4" t="n">
-        <v>1653.98</v>
+        <v>1310.61</v>
       </c>
       <c r="N51" s="4" t="n">
-        <v>1476.7</v>
+        <v>1246.25</v>
       </c>
       <c r="O51" s="4" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>✗</t>
         </is>
       </c>
       <c r="P51" s="4" t="inlineStr">
         <is>
-          <t>Buy</t>
+          <t>Sell</t>
         </is>
       </c>
       <c r="Q51" s="4" t="n">
-        <v>93.18000000000001</v>
+        <v>79.39</v>
       </c>
       <c r="R51" s="4" t="n">
-        <v>40.47</v>
+        <v>50.16</v>
       </c>
       <c r="S51" s="4" t="n">
-        <v>-2.5029</v>
+        <v>-1.5252</v>
       </c>
       <c r="T51" s="4" t="n">
-        <v>5.0185</v>
+        <v>-5.8828</v>
       </c>
       <c r="U51" s="4" t="n">
-        <v>-7.5214</v>
+        <v>4.3576</v>
       </c>
       <c r="V51" s="4" t="inlineStr"/>
       <c r="W51" s="4" t="n">
-        <v>15.95</v>
+        <v>11.13</v>
       </c>
       <c r="X51" s="4" t="n">
-        <v>736433</v>
+        <v>965167</v>
       </c>
       <c r="Y51" s="4" t="n">
-        <v>854057</v>
+        <v>2211497</v>
       </c>
       <c r="Z51" s="4" t="n">
-        <v>0.86</v>
+        <v>0.44</v>
       </c>
       <c r="AA51" s="4" t="n">
-        <v>93292</v>
+        <v>207297</v>
       </c>
       <c r="AB51" s="4" t="n">
-        <v>25.334375</v>
+        <v>120.54598</v>
       </c>
       <c r="AC51" s="4" t="n">
-        <v>17.354198</v>
+        <v>42.79666</v>
       </c>
       <c r="AD51" s="4" t="inlineStr"/>
       <c r="AE51" s="4" t="n">
-        <v>21.31</v>
+        <v>346.548</v>
       </c>
       <c r="AF51" s="4" t="n">
-        <v>16.3</v>
+        <v>16.6</v>
       </c>
       <c r="AG51" s="4" t="n">
-        <v>25.8</v>
+        <v>18.5</v>
       </c>
       <c r="AH51" s="4" t="n">
-        <v>2.4853194</v>
+        <v>10.746306</v>
       </c>
       <c r="AI51" s="4" t="n">
         <v>0</v>
@@ -7259,12 +7259,12 @@
       <c r="AJ51" s="4" t="inlineStr"/>
       <c r="AK51" s="4" t="inlineStr">
         <is>
-          <t>https://www.screener.in/company/AUROPHARMA/</t>
+          <t>https://www.screener.in/company/ADANIGREEN/</t>
         </is>
       </c>
       <c r="AL51" s="4" t="inlineStr">
         <is>
-          <t>https://www.tradingview.com/chart/?symbol=NSE:AUROPHARMA</t>
+          <t>https://www.tradingview.com/chart/?symbol=NSE:ADANIGREEN</t>
         </is>
       </c>
     </row>
@@ -7362,13 +7362,13 @@
         <v>0.78</v>
       </c>
       <c r="AA52" s="2" t="n">
-        <v>173398</v>
+        <v>173212</v>
       </c>
       <c r="AB52" s="2" t="n">
-        <v>72.82268500000001</v>
+        <v>72.74441</v>
       </c>
       <c r="AC52" s="2" t="n">
-        <v>48.862476</v>
+        <v>48.80995</v>
       </c>
       <c r="AD52" s="2" t="inlineStr"/>
       <c r="AE52" s="2" t="n">
@@ -7381,7 +7381,7 @@
         <v>-8.199999999999999</v>
       </c>
       <c r="AH52" s="2" t="n">
-        <v>18.392832</v>
+        <v>18.37306</v>
       </c>
       <c r="AI52" s="2" t="n">
         <v>83</v>
@@ -7492,13 +7492,13 @@
         <v>0.65</v>
       </c>
       <c r="AA53" s="4" t="n">
-        <v>27940</v>
+        <v>27311</v>
       </c>
       <c r="AB53" s="4" t="n">
-        <v>102.39433</v>
+        <v>100.089325</v>
       </c>
       <c r="AC53" s="4" t="n">
-        <v>55.79315</v>
+        <v>54.537186</v>
       </c>
       <c r="AD53" s="4" t="inlineStr"/>
       <c r="AE53" s="4" t="n">
@@ -7511,7 +7511,7 @@
         <v>178.4</v>
       </c>
       <c r="AH53" s="4" t="n">
-        <v>36.90306</v>
+        <v>36.07233</v>
       </c>
       <c r="AI53" s="4" t="n">
         <v>6</v>
@@ -7622,13 +7622,13 @@
         <v>0.68</v>
       </c>
       <c r="AA54" s="2" t="n">
-        <v>13514</v>
+        <v>13356</v>
       </c>
       <c r="AB54" s="2" t="n">
-        <v>101.37983</v>
+        <v>100.2007</v>
       </c>
       <c r="AC54" s="2" t="n">
-        <v>55.142258</v>
+        <v>54.50091</v>
       </c>
       <c r="AD54" s="2" t="inlineStr"/>
       <c r="AE54" s="2" t="n">
@@ -7641,7 +7641,7 @@
         <v>145.3</v>
       </c>
       <c r="AH54" s="2" t="n">
-        <v>18.702446</v>
+        <v>18.484922</v>
       </c>
       <c r="AI54" s="2" t="n">
         <v>0</v>
@@ -7752,13 +7752,13 @@
         <v>1.32</v>
       </c>
       <c r="AA55" s="4" t="n">
-        <v>9473</v>
+        <v>9238</v>
       </c>
       <c r="AB55" s="4" t="n">
-        <v>39.040527</v>
+        <v>38.07129</v>
       </c>
       <c r="AC55" s="4" t="n">
-        <v>21.64358</v>
+        <v>21.106247</v>
       </c>
       <c r="AD55" s="4" t="inlineStr"/>
       <c r="AE55" s="4" t="n">
@@ -7771,7 +7771,7 @@
         <v>101.5</v>
       </c>
       <c r="AH55" s="4" t="n">
-        <v>4.707472</v>
+        <v>4.5906024</v>
       </c>
       <c r="AI55" s="4" t="n">
         <v>0</v>
@@ -7882,13 +7882,13 @@
         <v>0.85</v>
       </c>
       <c r="AA56" s="2" t="n">
-        <v>67387</v>
+        <v>67043</v>
       </c>
       <c r="AB56" s="2" t="n">
-        <v>52.479107</v>
+        <v>52.211697</v>
       </c>
       <c r="AC56" s="2" t="n">
-        <v>37.989906</v>
+        <v>37.796326</v>
       </c>
       <c r="AD56" s="2" t="inlineStr"/>
       <c r="AE56" s="2" t="n">
@@ -7901,7 +7901,7 @@
         <v>23.3</v>
       </c>
       <c r="AH56" s="2" t="n">
-        <v>6.130677</v>
+        <v>6.099438</v>
       </c>
       <c r="AI56" s="2" t="n">
         <v>13</v>
@@ -8012,13 +8012,13 @@
         <v>0.57</v>
       </c>
       <c r="AA57" s="4" t="n">
-        <v>129022</v>
+        <v>121815</v>
       </c>
       <c r="AB57" s="4" t="n">
-        <v>88.820786</v>
+        <v>83.85879</v>
       </c>
       <c r="AC57" s="4" t="n">
-        <v>53.932774</v>
+        <v>50.919804</v>
       </c>
       <c r="AD57" s="4" t="inlineStr"/>
       <c r="AE57" s="4" t="n">
@@ -8031,7 +8031,7 @@
         <v>406.1</v>
       </c>
       <c r="AH57" s="4" t="n">
-        <v>9.3223</v>
+        <v>8.801507000000001</v>
       </c>
       <c r="AI57" s="4" t="n">
         <v>50</v>
@@ -8142,13 +8142,13 @@
         <v>1.28</v>
       </c>
       <c r="AA58" s="2" t="n">
-        <v>21987</v>
+        <v>22031</v>
       </c>
       <c r="AB58" s="2" t="n">
-        <v>29.942421</v>
+        <v>30.001858</v>
       </c>
       <c r="AC58" s="2" t="n">
-        <v>20.577497</v>
+        <v>20.618345</v>
       </c>
       <c r="AD58" s="2" t="inlineStr"/>
       <c r="AE58" s="2" t="n">
@@ -8161,7 +8161,7 @@
         <v>53.4</v>
       </c>
       <c r="AH58" s="2" t="n">
-        <v>3.9279659</v>
+        <v>3.935763</v>
       </c>
       <c r="AI58" s="2" t="n">
         <v>22</v>
@@ -8272,13 +8272,13 @@
         <v>1.02</v>
       </c>
       <c r="AA59" s="4" t="n">
-        <v>13346</v>
+        <v>12965</v>
       </c>
       <c r="AB59" s="4" t="n">
-        <v>32.22152</v>
+        <v>31.303797</v>
       </c>
       <c r="AC59" s="4" t="n">
-        <v>19.776358</v>
+        <v>19.213095</v>
       </c>
       <c r="AD59" s="4" t="inlineStr"/>
       <c r="AE59" s="4" t="n">
@@ -8291,7 +8291,7 @@
         <v>0.5</v>
       </c>
       <c r="AH59" s="4" t="n">
-        <v>3.2996092</v>
+        <v>3.205631</v>
       </c>
       <c r="AI59" s="4" t="n">
         <v>88</v>
@@ -8398,13 +8398,13 @@
         <v>0.44</v>
       </c>
       <c r="AA60" s="2" t="n">
-        <v>3505</v>
+        <v>3480</v>
       </c>
       <c r="AB60" s="2" t="n">
-        <v>89.80255</v>
+        <v>89.16561</v>
       </c>
       <c r="AC60" s="2" t="n">
-        <v>35.784264</v>
+        <v>35.530457</v>
       </c>
       <c r="AD60" s="2" t="inlineStr"/>
       <c r="AE60" s="2" t="n">
@@ -8415,7 +8415,7 @@
       </c>
       <c r="AG60" s="2" t="inlineStr"/>
       <c r="AH60" s="2" t="n">
-        <v>5.0926867</v>
+        <v>5.0565658</v>
       </c>
       <c r="AI60" s="2" t="n">
         <v>0</v>
@@ -8526,13 +8526,13 @@
         <v>0.26</v>
       </c>
       <c r="AA61" s="4" t="n">
-        <v>69793</v>
+        <v>70012</v>
       </c>
       <c r="AB61" s="4" t="n">
-        <v>16.341393</v>
+        <v>16.39265</v>
       </c>
       <c r="AC61" s="4" t="n">
-        <v>10.662889</v>
+        <v>10.696335</v>
       </c>
       <c r="AD61" s="4" t="inlineStr"/>
       <c r="AE61" s="4" t="n">
@@ -8545,7 +8545,7 @@
         <v>121.1</v>
       </c>
       <c r="AH61" s="4" t="n">
-        <v>1.1573207</v>
+        <v>1.1609509</v>
       </c>
       <c r="AI61" s="4" t="n">
         <v>139</v>
@@ -9150,13 +9150,13 @@
         <v>3.72</v>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>137939</v>
+        <v>138932</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>6.2699513</v>
+        <v>6.315059</v>
       </c>
       <c r="AC2" s="2" t="n">
-        <v>6.559412</v>
+        <v>6.606602</v>
       </c>
       <c r="AD2" s="2" t="n">
         <v>16.29</v>
@@ -9169,7 +9169,7 @@
         <v>29.3</v>
       </c>
       <c r="AH2" s="2" t="n">
-        <v>0.96673405</v>
+        <v>0.973689</v>
       </c>
       <c r="AI2" s="2" t="n">
         <v>277</v>
@@ -9280,13 +9280,13 @@
         <v>3.54</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>86180</v>
+        <v>84981</v>
       </c>
       <c r="AB3" s="4" t="n">
-        <v>17.033691</v>
+        <v>16.796875</v>
       </c>
       <c r="AC3" s="4" t="n">
-        <v>14.115253</v>
+        <v>13.919011</v>
       </c>
       <c r="AD3" s="4" t="n">
         <v>13.27</v>
@@ -9299,7 +9299,7 @@
         <v>45.5</v>
       </c>
       <c r="AH3" s="4" t="n">
-        <v>2.0145292</v>
+        <v>1.9865216</v>
       </c>
       <c r="AI3" s="4" t="n">
         <v>34</v>
@@ -9410,13 +9410,13 @@
         <v>4.58</v>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>140099</v>
+        <v>140789</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>6.141058</v>
+        <v>6.1712847</v>
       </c>
       <c r="AC4" s="2" t="n">
-        <v>6.582365</v>
+        <v>6.6147637</v>
       </c>
       <c r="AD4" s="2" t="n">
         <v>15.06</v>
@@ -9429,7 +9429,7 @@
         <v>15</v>
       </c>
       <c r="AH4" s="2" t="n">
-        <v>0.8706459</v>
+        <v>0.8749312</v>
       </c>
       <c r="AI4" s="2" t="n">
         <v>246</v>
@@ -9540,13 +9540,13 @@
         <v>2</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>89263</v>
+        <v>91906</v>
       </c>
       <c r="AB5" s="4" t="n">
-        <v>49.772568</v>
+        <v>51.246502</v>
       </c>
       <c r="AC5" s="4" t="n">
-        <v>32.424732</v>
+        <v>33.47168</v>
       </c>
       <c r="AD5" s="4" t="n">
         <v>22.92</v>
@@ -9561,7 +9561,7 @@
         <v>-26.3</v>
       </c>
       <c r="AH5" s="4" t="n">
-        <v>10.38615</v>
+        <v>10.693719</v>
       </c>
       <c r="AI5" s="4" t="n">
         <v>63</v>
@@ -9674,13 +9674,13 @@
         <v>0.6</v>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>439995</v>
+        <v>435518</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>21.681372</v>
+        <v>21.460785</v>
       </c>
       <c r="AC6" s="2" t="n">
-        <v>18.82891</v>
+        <v>18.637344</v>
       </c>
       <c r="AD6" s="2" t="inlineStr"/>
       <c r="AE6" s="2" t="inlineStr"/>
@@ -9691,7 +9691,7 @@
         <v>22.5</v>
       </c>
       <c r="AH6" s="2" t="n">
-        <v>2.4275386</v>
+        <v>2.4028406</v>
       </c>
       <c r="AI6" s="2" t="n">
         <v>15</v>
@@ -9802,13 +9802,13 @@
         <v>2.27</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>991481</v>
+        <v>994353</v>
       </c>
       <c r="AB7" s="4" t="n">
-        <v>17.851603</v>
+        <v>17.903309</v>
       </c>
       <c r="AC7" s="4" t="n">
-        <v>14.7106085</v>
+        <v>14.753217</v>
       </c>
       <c r="AD7" s="4" t="n">
         <v>16.49</v>
@@ -9821,7 +9821,7 @@
         <v>22.1</v>
       </c>
       <c r="AH7" s="4" t="n">
-        <v>2.7235436</v>
+        <v>2.7314322</v>
       </c>
       <c r="AI7" s="4" t="n">
         <v>87</v>
@@ -9932,13 +9932,13 @@
         <v>2.03</v>
       </c>
       <c r="AA8" s="2" t="n">
-        <v>41135</v>
+        <v>40518</v>
       </c>
       <c r="AB8" s="2" t="n">
-        <v>46.91274</v>
+        <v>46.209423</v>
       </c>
       <c r="AC8" s="2" t="n">
-        <v>32.386745</v>
+        <v>31.901203</v>
       </c>
       <c r="AD8" s="2" t="n">
         <v>18.66</v>
@@ -9953,7 +9953,7 @@
         <v>402.1</v>
       </c>
       <c r="AH8" s="2" t="n">
-        <v>7.2864037</v>
+        <v>7.177166</v>
       </c>
       <c r="AI8" s="2" t="n">
         <v>7</v>
@@ -10066,13 +10066,13 @@
         <v>0.86</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>331646</v>
+        <v>324650</v>
       </c>
       <c r="AB9" s="4" t="n">
-        <v>35.57899</v>
+        <v>34.828526</v>
       </c>
       <c r="AC9" s="4" t="n">
-        <v>28.711098</v>
+        <v>28.105494</v>
       </c>
       <c r="AD9" s="4" t="inlineStr"/>
       <c r="AE9" s="4" t="n">
@@ -10085,7 +10085,7 @@
         <v>14.9</v>
       </c>
       <c r="AH9" s="4" t="n">
-        <v>8.080811499999999</v>
+        <v>7.9103627</v>
       </c>
       <c r="AI9" s="4" t="n">
         <v>91</v>
@@ -10196,13 +10196,13 @@
         <v>3.37</v>
       </c>
       <c r="AA10" s="2" t="n">
-        <v>28479</v>
+        <v>27181</v>
       </c>
       <c r="AB10" s="2" t="n">
-        <v>76.96013000000001</v>
+        <v>73.45417</v>
       </c>
       <c r="AC10" s="2" t="n">
-        <v>36.51351</v>
+        <v>34.850124</v>
       </c>
       <c r="AD10" s="2" t="inlineStr"/>
       <c r="AE10" s="2" t="n">
@@ -10215,7 +10215,7 @@
         <v>40.6</v>
       </c>
       <c r="AH10" s="2" t="n">
-        <v>15.620138</v>
+        <v>14.908556</v>
       </c>
       <c r="AI10" s="2" t="n">
         <v>34</v>
@@ -10273,19 +10273,19 @@
         </is>
       </c>
       <c r="J11" s="4" t="n">
-        <v>173.72</v>
+        <v>170.72</v>
       </c>
       <c r="K11" s="4" t="n">
         <v>0.58</v>
       </c>
       <c r="L11" s="4" t="n">
-        <v>173.39</v>
+        <v>170.4</v>
       </c>
       <c r="M11" s="4" t="n">
-        <v>171.36</v>
+        <v>168.4</v>
       </c>
       <c r="N11" s="4" t="n">
-        <v>164.38</v>
+        <v>161.55</v>
       </c>
       <c r="O11" s="4" t="inlineStr">
         <is>
@@ -10304,13 +10304,13 @@
         <v>50.84</v>
       </c>
       <c r="S11" s="4" t="n">
-        <v>1.4202</v>
+        <v>1.3957</v>
       </c>
       <c r="T11" s="4" t="n">
-        <v>1.1421</v>
+        <v>1.1223</v>
       </c>
       <c r="U11" s="4" t="n">
-        <v>0.2781</v>
+        <v>0.2733</v>
       </c>
       <c r="V11" s="4" t="inlineStr"/>
       <c r="W11" s="4" t="n">
@@ -10326,13 +10326,13 @@
         <v>0.68</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>30446</v>
+        <v>29360</v>
       </c>
       <c r="AB11" s="4" t="n">
-        <v>6.8963876</v>
+        <v>6.650258</v>
       </c>
       <c r="AC11" s="4" t="n">
-        <v>4.3053284</v>
+        <v>4.1516733</v>
       </c>
       <c r="AD11" s="4" t="inlineStr"/>
       <c r="AE11" s="4" t="n">
@@ -10343,7 +10343,7 @@
       </c>
       <c r="AG11" s="4" t="inlineStr"/>
       <c r="AH11" s="4" t="n">
-        <v>2.136646</v>
+        <v>2.06039</v>
       </c>
       <c r="AI11" s="4" t="n">
         <v>345</v>
@@ -10701,13 +10701,13 @@
         <v>3.72</v>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>137939</v>
+        <v>138932</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>6.2699513</v>
+        <v>6.315059</v>
       </c>
       <c r="AC2" s="2" t="n">
-        <v>6.559412</v>
+        <v>6.606602</v>
       </c>
       <c r="AD2" s="2" t="n">
         <v>16.29</v>
@@ -10720,7 +10720,7 @@
         <v>29.3</v>
       </c>
       <c r="AH2" s="2" t="n">
-        <v>0.96673405</v>
+        <v>0.973689</v>
       </c>
       <c r="AI2" s="2" t="n">
         <v>277</v>
@@ -10831,13 +10831,13 @@
         <v>3.54</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>86180</v>
+        <v>84981</v>
       </c>
       <c r="AB3" s="4" t="n">
-        <v>17.033691</v>
+        <v>16.796875</v>
       </c>
       <c r="AC3" s="4" t="n">
-        <v>14.115253</v>
+        <v>13.919011</v>
       </c>
       <c r="AD3" s="4" t="n">
         <v>13.27</v>
@@ -10850,7 +10850,7 @@
         <v>45.5</v>
       </c>
       <c r="AH3" s="4" t="n">
-        <v>2.0145292</v>
+        <v>1.9865216</v>
       </c>
       <c r="AI3" s="4" t="n">
         <v>34</v>
@@ -10961,13 +10961,13 @@
         <v>4.58</v>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>140099</v>
+        <v>140789</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>6.141058</v>
+        <v>6.1712847</v>
       </c>
       <c r="AC4" s="2" t="n">
-        <v>6.582365</v>
+        <v>6.6147637</v>
       </c>
       <c r="AD4" s="2" t="n">
         <v>15.06</v>
@@ -10980,7 +10980,7 @@
         <v>15</v>
       </c>
       <c r="AH4" s="2" t="n">
-        <v>0.8706459</v>
+        <v>0.8749312</v>
       </c>
       <c r="AI4" s="2" t="n">
         <v>246</v>
@@ -11091,13 +11091,13 @@
         <v>2</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>89263</v>
+        <v>91906</v>
       </c>
       <c r="AB5" s="4" t="n">
-        <v>49.772568</v>
+        <v>51.246502</v>
       </c>
       <c r="AC5" s="4" t="n">
-        <v>32.424732</v>
+        <v>33.47168</v>
       </c>
       <c r="AD5" s="4" t="n">
         <v>22.92</v>
@@ -11112,7 +11112,7 @@
         <v>-26.3</v>
       </c>
       <c r="AH5" s="4" t="n">
-        <v>10.38615</v>
+        <v>10.693719</v>
       </c>
       <c r="AI5" s="4" t="n">
         <v>63</v>
@@ -11225,13 +11225,13 @@
         <v>0.6</v>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>439995</v>
+        <v>435518</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>21.681372</v>
+        <v>21.460785</v>
       </c>
       <c r="AC6" s="2" t="n">
-        <v>18.82891</v>
+        <v>18.637344</v>
       </c>
       <c r="AD6" s="2" t="inlineStr"/>
       <c r="AE6" s="2" t="inlineStr"/>
@@ -11242,7 +11242,7 @@
         <v>22.5</v>
       </c>
       <c r="AH6" s="2" t="n">
-        <v>2.4275386</v>
+        <v>2.4028406</v>
       </c>
       <c r="AI6" s="2" t="n">
         <v>15</v>
@@ -11353,13 +11353,13 @@
         <v>2.27</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>991481</v>
+        <v>994353</v>
       </c>
       <c r="AB7" s="4" t="n">
-        <v>17.851603</v>
+        <v>17.903309</v>
       </c>
       <c r="AC7" s="4" t="n">
-        <v>14.7106085</v>
+        <v>14.753217</v>
       </c>
       <c r="AD7" s="4" t="n">
         <v>16.49</v>
@@ -11372,7 +11372,7 @@
         <v>22.1</v>
       </c>
       <c r="AH7" s="4" t="n">
-        <v>2.7235436</v>
+        <v>2.7314322</v>
       </c>
       <c r="AI7" s="4" t="n">
         <v>87</v>
@@ -11483,13 +11483,13 @@
         <v>2.03</v>
       </c>
       <c r="AA8" s="2" t="n">
-        <v>41135</v>
+        <v>40518</v>
       </c>
       <c r="AB8" s="2" t="n">
-        <v>46.91274</v>
+        <v>46.209423</v>
       </c>
       <c r="AC8" s="2" t="n">
-        <v>32.386745</v>
+        <v>31.901203</v>
       </c>
       <c r="AD8" s="2" t="n">
         <v>18.66</v>
@@ -11504,7 +11504,7 @@
         <v>402.1</v>
       </c>
       <c r="AH8" s="2" t="n">
-        <v>7.2864037</v>
+        <v>7.177166</v>
       </c>
       <c r="AI8" s="2" t="n">
         <v>7</v>
@@ -11617,13 +11617,13 @@
         <v>0.86</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>331646</v>
+        <v>324650</v>
       </c>
       <c r="AB9" s="4" t="n">
-        <v>35.57899</v>
+        <v>34.828526</v>
       </c>
       <c r="AC9" s="4" t="n">
-        <v>28.711098</v>
+        <v>28.105494</v>
       </c>
       <c r="AD9" s="4" t="inlineStr"/>
       <c r="AE9" s="4" t="n">
@@ -11636,7 +11636,7 @@
         <v>14.9</v>
       </c>
       <c r="AH9" s="4" t="n">
-        <v>8.080811499999999</v>
+        <v>7.9103627</v>
       </c>
       <c r="AI9" s="4" t="n">
         <v>91</v>
@@ -11747,13 +11747,13 @@
         <v>3.37</v>
       </c>
       <c r="AA10" s="2" t="n">
-        <v>28479</v>
+        <v>27181</v>
       </c>
       <c r="AB10" s="2" t="n">
-        <v>76.96013000000001</v>
+        <v>73.45417</v>
       </c>
       <c r="AC10" s="2" t="n">
-        <v>36.51351</v>
+        <v>34.850124</v>
       </c>
       <c r="AD10" s="2" t="inlineStr"/>
       <c r="AE10" s="2" t="n">
@@ -11766,7 +11766,7 @@
         <v>40.6</v>
       </c>
       <c r="AH10" s="2" t="n">
-        <v>15.620138</v>
+        <v>14.908556</v>
       </c>
       <c r="AI10" s="2" t="n">
         <v>34</v>
@@ -11824,19 +11824,19 @@
         </is>
       </c>
       <c r="J11" s="4" t="n">
-        <v>173.72</v>
+        <v>170.72</v>
       </c>
       <c r="K11" s="4" t="n">
         <v>0.58</v>
       </c>
       <c r="L11" s="4" t="n">
-        <v>173.39</v>
+        <v>170.4</v>
       </c>
       <c r="M11" s="4" t="n">
-        <v>171.36</v>
+        <v>168.4</v>
       </c>
       <c r="N11" s="4" t="n">
-        <v>164.38</v>
+        <v>161.55</v>
       </c>
       <c r="O11" s="4" t="inlineStr">
         <is>
@@ -11855,13 +11855,13 @@
         <v>50.84</v>
       </c>
       <c r="S11" s="4" t="n">
-        <v>1.4202</v>
+        <v>1.3957</v>
       </c>
       <c r="T11" s="4" t="n">
-        <v>1.1421</v>
+        <v>1.1223</v>
       </c>
       <c r="U11" s="4" t="n">
-        <v>0.2781</v>
+        <v>0.2733</v>
       </c>
       <c r="V11" s="4" t="inlineStr"/>
       <c r="W11" s="4" t="n">
@@ -11877,13 +11877,13 @@
         <v>0.68</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>30446</v>
+        <v>29360</v>
       </c>
       <c r="AB11" s="4" t="n">
-        <v>6.8963876</v>
+        <v>6.650258</v>
       </c>
       <c r="AC11" s="4" t="n">
-        <v>4.3053284</v>
+        <v>4.1516733</v>
       </c>
       <c r="AD11" s="4" t="inlineStr"/>
       <c r="AE11" s="4" t="n">
@@ -11894,7 +11894,7 @@
       </c>
       <c r="AG11" s="4" t="inlineStr"/>
       <c r="AH11" s="4" t="n">
-        <v>2.136646</v>
+        <v>2.06039</v>
       </c>
       <c r="AI11" s="4" t="n">
         <v>345</v>
@@ -11937,7 +11937,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Run Date: 20-Oct-2026 14:03 IST</t>
+          <t>Run Date: 21-Oct-2026 14:19 IST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>

</xml_diff>